<commit_message>
Noviembre 2026: ajustar horarios a 42 h (tiempo completo) y 21 h (medio tiempo)
Parte de la versión editada por coordinación (Nicolás Mahecha, Diana Lasso,
cambios de sábados). Ajusta salidas L-V según haya o no sábado, corrige
semanas de la jefe Marly que no sumaban 42 h, quita el sáb 28 sobrante de
Nicolás Torres, iguala almuerzo de Herlinda y Nataly, y actualiza la tabla
de máximos y la leyenda.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QFEyfDRz3kAA5d3tShZ31H
</commit_message>
<xml_diff>
--- a/TURNOS_Noviembre_2026.xlsx
+++ b/TURNOS_Noviembre_2026.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="NOVIEMBRE" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,7 +11,7 @@
     <sheet name="Oferta OPS" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -65,12 +64,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -83,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -94,9 +108,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -109,17 +121,21 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -206,12 +222,17 @@
     </comment>
     <comment ref="C13" authorId="0" shapeId="0">
       <text>
-        <t>Nov-2026 (42 h/semana): semanas con sábado (14 y 28, igual que Nicolás) L-V 7:00-15:36 + sáb 8:00-12:00; semanas sin sábado L-V 7:00-16:24. Almuerzo 1 h.</t>
+        <t>Nov-2026 (42 h/semana): semanas con sábado (7 y 21, igual que Nicolás Torres) L-V 7:00-15:36 + sáb 8:00-12:00; semanas sin sábado L-V 7:00-16:24.</t>
       </text>
     </comment>
     <comment ref="A14" authorId="0" shapeId="0">
       <text>
         <t>Vacaciones 15 oct - 5 nov 2026. Regresa el viernes 6 de noviembre.</t>
+      </text>
+    </comment>
+    <comment ref="B33" authorId="0" shapeId="0">
+      <text>
+        <t>L-V en semanas con sábado. En semanas sin sábado L-V = 42 h (21 h medio tiempo).</t>
       </text>
     </comment>
     <comment ref="B44" authorId="0" shapeId="0">
@@ -513,49 +534,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AN53"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="38.4" customWidth="1" min="1" max="1"/>
-    <col width="18.1" customWidth="1" min="2" max="2"/>
-    <col width="13.4" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="11" customWidth="1" min="19" max="19"/>
-    <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="11" customWidth="1" min="21" max="21"/>
-    <col width="11" customWidth="1" min="22" max="22"/>
-    <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="11" customWidth="1" min="24" max="24"/>
-    <col width="11" customWidth="1" min="25" max="25"/>
-    <col width="11" customWidth="1" min="26" max="26"/>
-    <col width="11" customWidth="1" min="27" max="27"/>
-    <col width="11" customWidth="1" min="28" max="28"/>
-    <col width="11" customWidth="1" min="29" max="29"/>
-    <col width="11" customWidth="1" min="30" max="30"/>
-    <col width="11" customWidth="1" min="31" max="31"/>
-    <col width="11" customWidth="1" min="32" max="32"/>
-    <col width="11" customWidth="1" min="33" max="33"/>
-    <col width="12" customWidth="1" min="34" max="34"/>
-    <col width="12" customWidth="1" min="35" max="35"/>
-    <col width="12" customWidth="1" min="36" max="36"/>
-    <col width="12" customWidth="1" min="37" max="37"/>
-    <col width="12" customWidth="1" min="38" max="38"/>
-    <col width="12" customWidth="1" min="39" max="39"/>
-    <col width="12" customWidth="1" min="40" max="40"/>
-    <col width="12" customWidth="1" min="41" max="41"/>
+    <col width="38.42578125" customWidth="1" min="1" max="1"/>
+    <col width="18.140625" customWidth="1" min="2" max="2"/>
+    <col width="13.42578125" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="33"/>
+    <col width="12" customWidth="1" min="34" max="41"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -754,22 +739,22 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:06</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:06</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:06</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>8:00-17:00</t>
+          <t>8:00-16:36</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
@@ -884,7 +869,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Cristhian caicedo</t>
+          <t>Nicolas Mahecha</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -894,7 +879,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Medio tiempo</t>
         </is>
       </c>
       <c r="D3" s="6" t="n"/>
@@ -905,49 +890,53 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:30</t>
+          <t>7:30-10:54</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:30</t>
+          <t>7:30-10:54</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:30</t>
+          <t>7:30-10:54</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:30</t>
-        </is>
-      </c>
-      <c r="J3" s="6" t="n"/>
+          <t>7:30-10:54</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>8:00-12:00</t>
+        </is>
+      </c>
       <c r="K3" s="6" t="n"/>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:30</t>
+          <t>7:30-11:42</t>
         </is>
       </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:30</t>
+          <t>7:30-11:42</t>
         </is>
       </c>
       <c r="N3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:30</t>
+          <t>7:30-11:42</t>
         </is>
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:30</t>
+          <t>7:30-11:42</t>
         </is>
       </c>
       <c r="P3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:30</t>
+          <t>7:30-11:42</t>
         </is>
       </c>
       <c r="Q3" s="6" t="n"/>
@@ -959,56 +948,60 @@
       </c>
       <c r="T3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:30</t>
+          <t>7:30-10:54</t>
         </is>
       </c>
       <c r="U3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:30</t>
+          <t>7:30-10:54</t>
         </is>
       </c>
       <c r="V3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:30</t>
+          <t>7:30-10:54</t>
         </is>
       </c>
       <c r="W3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:30</t>
-        </is>
-      </c>
-      <c r="X3" s="6" t="n"/>
+          <t>7:30-10:54</t>
+        </is>
+      </c>
+      <c r="X3" s="6" t="inlineStr">
+        <is>
+          <t>8:00-12:00</t>
+        </is>
+      </c>
       <c r="Y3" s="6" t="n"/>
       <c r="Z3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:30</t>
+          <t>7:30-11:42</t>
         </is>
       </c>
       <c r="AA3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:30</t>
+          <t>7:30-11:42</t>
         </is>
       </c>
       <c r="AB3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:30</t>
+          <t>7:30-11:42</t>
         </is>
       </c>
       <c r="AC3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:30</t>
+          <t>7:30-11:42</t>
         </is>
       </c>
       <c r="AD3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:30</t>
+          <t>7:30-11:42</t>
         </is>
       </c>
       <c r="AE3" s="6" t="n"/>
       <c r="AF3" s="6" t="n"/>
       <c r="AG3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:30</t>
+          <t>7:30-10:54</t>
         </is>
       </c>
       <c r="AH3" s="5">
@@ -1040,49 +1033,49 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:18</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:18</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:18</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:30</t>
+          <t>7:00-16:48</t>
         </is>
       </c>
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="6" t="n"/>
       <c r="L4" s="5" t="inlineStr">
         <is>
+          <t>7:00-15:30</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>7:00-15:30</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>7:00-15:30</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>7:00-15:30</t>
+        </is>
+      </c>
+      <c r="P4" s="5" t="inlineStr">
+        <is>
           <t>7:00-16:00</t>
-        </is>
-      </c>
-      <c r="M4" s="5" t="inlineStr">
-        <is>
-          <t>7:00-16:00</t>
-        </is>
-      </c>
-      <c r="N4" s="5" t="inlineStr">
-        <is>
-          <t>7:00-16:00</t>
-        </is>
-      </c>
-      <c r="O4" s="5" t="inlineStr">
-        <is>
-          <t>7:00-16:00</t>
-        </is>
-      </c>
-      <c r="P4" s="5" t="inlineStr">
-        <is>
-          <t>7:00-16:30</t>
         </is>
       </c>
       <c r="Q4" s="5" t="inlineStr">
@@ -1098,49 +1091,49 @@
       </c>
       <c r="T4" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:18</t>
         </is>
       </c>
       <c r="U4" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:18</t>
         </is>
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:18</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:30</t>
+          <t>7:00-16:48</t>
         </is>
       </c>
       <c r="X4" s="6" t="n"/>
       <c r="Y4" s="6" t="n"/>
       <c r="Z4" s="5" t="inlineStr">
         <is>
+          <t>7:00-15:30</t>
+        </is>
+      </c>
+      <c r="AA4" s="5" t="inlineStr">
+        <is>
+          <t>7:00-15:30</t>
+        </is>
+      </c>
+      <c r="AB4" s="5" t="inlineStr">
+        <is>
+          <t>7:00-15:30</t>
+        </is>
+      </c>
+      <c r="AC4" s="5" t="inlineStr">
+        <is>
+          <t>7:00-15:30</t>
+        </is>
+      </c>
+      <c r="AD4" s="5" t="inlineStr">
+        <is>
           <t>7:00-16:00</t>
-        </is>
-      </c>
-      <c r="AA4" s="5" t="inlineStr">
-        <is>
-          <t>7:00-16:00</t>
-        </is>
-      </c>
-      <c r="AB4" s="5" t="inlineStr">
-        <is>
-          <t>7:00-16:00</t>
-        </is>
-      </c>
-      <c r="AC4" s="5" t="inlineStr">
-        <is>
-          <t>7:00-16:00</t>
-        </is>
-      </c>
-      <c r="AD4" s="5" t="inlineStr">
-        <is>
-          <t>7:00-16:30</t>
         </is>
       </c>
       <c r="AE4" s="5" t="inlineStr">
@@ -1151,7 +1144,7 @@
       <c r="AF4" s="6" t="n"/>
       <c r="AG4" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:18</t>
         </is>
       </c>
       <c r="AH4" s="5">
@@ -1183,56 +1176,56 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:36</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>9:00-18:00</t>
+          <t>8:24-18:00</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:36</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>9:00-18:00</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>7:00-13:00</t>
-        </is>
-      </c>
+          <t>8:24-18:00</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="n"/>
       <c r="K5" s="6" t="n"/>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>10:00-18:00</t>
+          <t>10:00-17:24</t>
         </is>
       </c>
       <c r="M5" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-15:24</t>
         </is>
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>9:00-18:00</t>
+          <t>9:00-17:24</t>
         </is>
       </c>
       <c r="O5" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-15:24</t>
         </is>
       </c>
       <c r="P5" s="5" t="inlineStr">
         <is>
-          <t>9:00-18:00</t>
-        </is>
-      </c>
-      <c r="Q5" s="6" t="n"/>
+          <t>9:00-17:24</t>
+        </is>
+      </c>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>7:00-13:00</t>
+        </is>
+      </c>
       <c r="R5" s="6" t="n"/>
       <c r="S5" s="7" t="inlineStr">
         <is>
@@ -1241,22 +1234,22 @@
       </c>
       <c r="T5" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-15:24</t>
         </is>
       </c>
       <c r="U5" s="5" t="inlineStr">
         <is>
-          <t>9:00-18:00</t>
+          <t>9:00-17:24</t>
         </is>
       </c>
       <c r="V5" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-15:24</t>
         </is>
       </c>
       <c r="W5" s="5" t="inlineStr">
         <is>
-          <t>9:00-18:00</t>
+          <t>9:00-17:24</t>
         </is>
       </c>
       <c r="X5" s="5" t="inlineStr">
@@ -1267,34 +1260,34 @@
       <c r="Y5" s="6" t="n"/>
       <c r="Z5" s="5" t="inlineStr">
         <is>
-          <t>10:00-18:00</t>
+          <t>9:24-18:00</t>
         </is>
       </c>
       <c r="AA5" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:36</t>
         </is>
       </c>
       <c r="AB5" s="5" t="inlineStr">
         <is>
-          <t>9:00-18:00</t>
+          <t>8:24-18:00</t>
         </is>
       </c>
       <c r="AC5" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:36</t>
         </is>
       </c>
       <c r="AD5" s="5" t="inlineStr">
         <is>
-          <t>9:00-18:00</t>
+          <t>8:24-18:00</t>
         </is>
       </c>
       <c r="AE5" s="6" t="n"/>
       <c r="AF5" s="6" t="n"/>
       <c r="AG5" s="5" t="inlineStr">
         <is>
-          <t>10:00-18:00</t>
+          <t>10:00-17:24</t>
         </is>
       </c>
       <c r="AH5" s="5">
@@ -1326,49 +1319,49 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>9:00-18:00</t>
+          <t>8:24-18:00</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:36</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>9:00-18:00</t>
+          <t>8:24-18:00</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:36</t>
         </is>
       </c>
       <c r="J6" s="6" t="n"/>
       <c r="K6" s="6" t="n"/>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:00</t>
+          <t>7:00-14:36</t>
         </is>
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>9:00-18:00</t>
+          <t>9:00-17:36</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-15:36</t>
         </is>
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>9:00-18:00</t>
+          <t>9:00-17:36</t>
         </is>
       </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-15:36</t>
         </is>
       </c>
       <c r="Q6" s="5" t="inlineStr">
@@ -1384,49 +1377,49 @@
       </c>
       <c r="T6" s="5" t="inlineStr">
         <is>
-          <t>9:00-18:00</t>
+          <t>8:24-18:00</t>
         </is>
       </c>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:36</t>
         </is>
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>9:00-18:00</t>
+          <t>8:24-18:00</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:36</t>
         </is>
       </c>
       <c r="X6" s="6" t="n"/>
       <c r="Y6" s="6" t="n"/>
       <c r="Z6" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:00</t>
+          <t>7:00-14:36</t>
         </is>
       </c>
       <c r="AA6" s="5" t="inlineStr">
         <is>
-          <t>9:00-18:00</t>
+          <t>9:00-17:36</t>
         </is>
       </c>
       <c r="AB6" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-15:36</t>
         </is>
       </c>
       <c r="AC6" s="5" t="inlineStr">
         <is>
-          <t>9:00-18:00</t>
+          <t>9:00-17:36</t>
         </is>
       </c>
       <c r="AD6" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-15:36</t>
         </is>
       </c>
       <c r="AE6" s="5" t="inlineStr">
@@ -1437,7 +1430,7 @@
       <c r="AF6" s="6" t="n"/>
       <c r="AG6" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:00</t>
+          <t>7:00-15:36</t>
         </is>
       </c>
       <c r="AH6" s="5">
@@ -1469,49 +1462,49 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:42</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:42</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:42</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:42</t>
         </is>
       </c>
       <c r="J7" s="6" t="n"/>
       <c r="K7" s="6" t="n"/>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>7:30-17:30</t>
+          <t>7:30-17:42</t>
         </is>
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:42</t>
         </is>
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:42</t>
         </is>
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:42</t>
         </is>
       </c>
       <c r="P7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:42</t>
         </is>
       </c>
       <c r="Q7" s="6" t="n"/>
@@ -1523,56 +1516,56 @@
       </c>
       <c r="T7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:42</t>
         </is>
       </c>
       <c r="U7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:42</t>
         </is>
       </c>
       <c r="V7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:42</t>
         </is>
       </c>
       <c r="W7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:42</t>
         </is>
       </c>
       <c r="X7" s="6" t="n"/>
       <c r="Y7" s="6" t="n"/>
       <c r="Z7" s="5" t="inlineStr">
         <is>
-          <t>7:30-17:30</t>
+          <t>7:30-17:42</t>
         </is>
       </c>
       <c r="AA7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:42</t>
         </is>
       </c>
       <c r="AB7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:42</t>
         </is>
       </c>
       <c r="AC7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:42</t>
         </is>
       </c>
       <c r="AD7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:42</t>
         </is>
       </c>
       <c r="AE7" s="6" t="n"/>
       <c r="AF7" s="6" t="n"/>
       <c r="AG7" s="5" t="inlineStr">
         <is>
-          <t>7:30-17:30</t>
+          <t>7:30-17:42</t>
         </is>
       </c>
       <c r="AH7" s="5">
@@ -1734,7 +1727,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Daniel Salas</t>
+          <t>Diana Lasso</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -1906,22 +1899,22 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:06</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:06</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:06</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:06</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
@@ -1932,27 +1925,27 @@
       <c r="K10" s="6" t="n"/>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:54</t>
         </is>
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:54</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:54</t>
         </is>
       </c>
       <c r="O10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:54</t>
         </is>
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:54</t>
         </is>
       </c>
       <c r="Q10" s="6" t="n"/>
@@ -1964,22 +1957,22 @@
       </c>
       <c r="T10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:06</t>
         </is>
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:06</t>
         </is>
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:06</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:06</t>
         </is>
       </c>
       <c r="X10" s="5" t="inlineStr">
@@ -1990,34 +1983,34 @@
       <c r="Y10" s="6" t="n"/>
       <c r="Z10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:54</t>
         </is>
       </c>
       <c r="AA10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:54</t>
         </is>
       </c>
       <c r="AB10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:54</t>
         </is>
       </c>
       <c r="AC10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:54</t>
         </is>
       </c>
       <c r="AD10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:54</t>
         </is>
       </c>
       <c r="AE10" s="6" t="n"/>
       <c r="AF10" s="6" t="n"/>
       <c r="AG10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:06</t>
         </is>
       </c>
       <c r="AH10" s="5">
@@ -2049,56 +2042,56 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:30</t>
+          <t>7:00-16:06</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:30</t>
+          <t>8:00-16:06</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:06</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:30</t>
-        </is>
-      </c>
-      <c r="J11" s="6" t="n"/>
+          <t>7:00-16:06</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>7:30-11:30</t>
+        </is>
+      </c>
       <c r="K11" s="6" t="n"/>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:30</t>
+          <t>8:00-16:54</t>
         </is>
       </c>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:30</t>
+          <t>7:00-16:54</t>
         </is>
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:30</t>
+          <t>8:00-16:54</t>
         </is>
       </c>
       <c r="O11" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:54</t>
         </is>
       </c>
       <c r="P11" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:30</t>
-        </is>
-      </c>
-      <c r="Q11" s="5" t="inlineStr">
-        <is>
-          <t>7:30-11:30</t>
-        </is>
-      </c>
+          <t>7:00-16:54</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="n"/>
       <c r="R11" s="6" t="n"/>
       <c r="S11" s="7" t="inlineStr">
         <is>
@@ -2107,60 +2100,60 @@
       </c>
       <c r="T11" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:30</t>
+          <t>7:00-16:06</t>
         </is>
       </c>
       <c r="U11" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:30</t>
+          <t>8:00-16:06</t>
         </is>
       </c>
       <c r="V11" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:06</t>
         </is>
       </c>
       <c r="W11" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:30</t>
-        </is>
-      </c>
-      <c r="X11" s="6" t="n"/>
+          <t>7:00-16:06</t>
+        </is>
+      </c>
+      <c r="X11" s="5" t="inlineStr">
+        <is>
+          <t>7:30-11:30</t>
+        </is>
+      </c>
       <c r="Y11" s="6" t="n"/>
       <c r="Z11" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:30</t>
+          <t>8:00-16:54</t>
         </is>
       </c>
       <c r="AA11" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:30</t>
+          <t>7:00-16:54</t>
         </is>
       </c>
       <c r="AB11" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:30</t>
+          <t>8:00-16:54</t>
         </is>
       </c>
       <c r="AC11" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:54</t>
         </is>
       </c>
       <c r="AD11" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:30</t>
-        </is>
-      </c>
-      <c r="AE11" s="5" t="inlineStr">
-        <is>
-          <t>7:30-11:30</t>
-        </is>
-      </c>
+          <t>7:00-16:54</t>
+        </is>
+      </c>
+      <c r="AE11" s="6" t="n"/>
       <c r="AF11" s="6" t="n"/>
       <c r="AG11" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:30</t>
+          <t>8:00-16:06</t>
         </is>
       </c>
       <c r="AH11" s="5">
@@ -2192,56 +2185,56 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
+          <t>7:00-15:36</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>7:00-15:36</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>7:00-15:36</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>7:00-15:36</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>8:00-12:00</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="n"/>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
           <t>7:00-16:24</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="M12" s="5" t="inlineStr">
         <is>
           <t>7:00-16:24</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="N12" s="5" t="inlineStr">
         <is>
           <t>7:00-16:24</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="O12" s="5" t="inlineStr">
         <is>
           <t>7:00-16:24</t>
         </is>
       </c>
-      <c r="J12" s="6" t="n"/>
-      <c r="K12" s="6" t="n"/>
-      <c r="L12" s="5" t="inlineStr">
-        <is>
-          <t>7:00-15:36</t>
-        </is>
-      </c>
-      <c r="M12" s="5" t="inlineStr">
-        <is>
-          <t>7:00-15:36</t>
-        </is>
-      </c>
-      <c r="N12" s="5" t="inlineStr">
-        <is>
-          <t>7:00-15:36</t>
-        </is>
-      </c>
-      <c r="O12" s="5" t="inlineStr">
-        <is>
-          <t>7:00-15:36</t>
-        </is>
-      </c>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
-        </is>
-      </c>
-      <c r="Q12" s="5" t="inlineStr">
-        <is>
-          <t>8:00-12:00</t>
-        </is>
-      </c>
+          <t>7:00-16:24</t>
+        </is>
+      </c>
+      <c r="Q12" s="5" t="n"/>
       <c r="R12" s="6" t="n"/>
       <c r="S12" s="7" t="inlineStr">
         <is>
@@ -2250,60 +2243,60 @@
       </c>
       <c r="T12" s="5" t="inlineStr">
         <is>
+          <t>7:00-15:36</t>
+        </is>
+      </c>
+      <c r="U12" s="5" t="inlineStr">
+        <is>
+          <t>7:00-15:36</t>
+        </is>
+      </c>
+      <c r="V12" s="5" t="inlineStr">
+        <is>
+          <t>7:00-15:36</t>
+        </is>
+      </c>
+      <c r="W12" s="5" t="inlineStr">
+        <is>
+          <t>7:00-15:36</t>
+        </is>
+      </c>
+      <c r="X12" s="5" t="inlineStr">
+        <is>
+          <t>8:00-12:00</t>
+        </is>
+      </c>
+      <c r="Y12" s="5" t="n"/>
+      <c r="Z12" s="5" t="inlineStr">
+        <is>
           <t>7:00-16:24</t>
         </is>
       </c>
-      <c r="U12" s="5" t="inlineStr">
+      <c r="AA12" s="5" t="inlineStr">
         <is>
           <t>7:00-16:24</t>
         </is>
       </c>
-      <c r="V12" s="5" t="inlineStr">
+      <c r="AB12" s="5" t="inlineStr">
         <is>
           <t>7:00-16:24</t>
         </is>
       </c>
-      <c r="W12" s="5" t="inlineStr">
+      <c r="AC12" s="5" t="inlineStr">
         <is>
           <t>7:00-16:24</t>
         </is>
       </c>
-      <c r="X12" s="6" t="n"/>
-      <c r="Y12" s="6" t="n"/>
-      <c r="Z12" s="5" t="inlineStr">
-        <is>
-          <t>7:00-15:36</t>
-        </is>
-      </c>
-      <c r="AA12" s="5" t="inlineStr">
-        <is>
-          <t>7:00-15:36</t>
-        </is>
-      </c>
-      <c r="AB12" s="5" t="inlineStr">
-        <is>
-          <t>7:00-15:36</t>
-        </is>
-      </c>
-      <c r="AC12" s="5" t="inlineStr">
-        <is>
-          <t>7:00-15:36</t>
-        </is>
-      </c>
       <c r="AD12" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
-        </is>
-      </c>
-      <c r="AE12" s="5" t="inlineStr">
-        <is>
-          <t>8:00-12:00</t>
-        </is>
-      </c>
+          <t>7:00-16:24</t>
+        </is>
+      </c>
+      <c r="AE12" s="5" t="n"/>
       <c r="AF12" s="6" t="n"/>
       <c r="AG12" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:24</t>
+          <t>7:00-15:36</t>
         </is>
       </c>
       <c r="AH12" s="5">
@@ -2335,22 +2328,22 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-15:36</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-15:36</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-15:36</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:06</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
@@ -2361,27 +2354,27 @@
       <c r="K13" s="6" t="n"/>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:54</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:24</t>
         </is>
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:24</t>
         </is>
       </c>
       <c r="O13" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:24</t>
         </is>
       </c>
       <c r="P13" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:54</t>
         </is>
       </c>
       <c r="Q13" s="6" t="n"/>
@@ -2393,22 +2386,22 @@
       </c>
       <c r="T13" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-15:36</t>
         </is>
       </c>
       <c r="U13" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-15:36</t>
         </is>
       </c>
       <c r="V13" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-15:36</t>
         </is>
       </c>
       <c r="W13" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:06</t>
         </is>
       </c>
       <c r="X13" s="5" t="inlineStr">
@@ -2419,34 +2412,34 @@
       <c r="Y13" s="6" t="n"/>
       <c r="Z13" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:54</t>
         </is>
       </c>
       <c r="AA13" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:24</t>
         </is>
       </c>
       <c r="AB13" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:24</t>
         </is>
       </c>
       <c r="AC13" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:24</t>
         </is>
       </c>
       <c r="AD13" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:54</t>
         </is>
       </c>
       <c r="AE13" s="6" t="n"/>
       <c r="AF13" s="6" t="n"/>
       <c r="AG13" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:30</t>
+          <t>7:30-16:06</t>
         </is>
       </c>
       <c r="AH13" s="5">
@@ -2493,41 +2486,41 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:30</t>
-        </is>
-      </c>
-      <c r="J14" s="6" t="n"/>
+          <t>8:00-16:06</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>7:30-11:30</t>
+        </is>
+      </c>
       <c r="K14" s="6" t="n"/>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:24</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:30</t>
+          <t>8:00-16:54</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:30</t>
+          <t>7:00-16:54</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:30</t>
+          <t>7:00-16:54</t>
         </is>
       </c>
       <c r="P14" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:30</t>
-        </is>
-      </c>
-      <c r="Q14" s="5" t="inlineStr">
-        <is>
-          <t>7:30-11:30</t>
-        </is>
-      </c>
+          <t>8:00-16:54</t>
+        </is>
+      </c>
+      <c r="Q14" s="5" t="n"/>
       <c r="R14" s="6" t="n"/>
       <c r="S14" s="7" t="inlineStr">
         <is>
@@ -2536,60 +2529,60 @@
       </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:30</t>
+          <t>8:00-16:06</t>
         </is>
       </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:30</t>
+          <t>7:00-16:06</t>
         </is>
       </c>
       <c r="V14" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:30</t>
+          <t>7:00-16:06</t>
         </is>
       </c>
       <c r="W14" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:30</t>
-        </is>
-      </c>
-      <c r="X14" s="6" t="n"/>
+          <t>8:00-16:06</t>
+        </is>
+      </c>
+      <c r="X14" s="5" t="inlineStr">
+        <is>
+          <t>7:30-11:30</t>
+        </is>
+      </c>
       <c r="Y14" s="6" t="n"/>
       <c r="Z14" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-16:24</t>
         </is>
       </c>
       <c r="AA14" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:30</t>
+          <t>8:00-16:54</t>
         </is>
       </c>
       <c r="AB14" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:30</t>
+          <t>7:00-16:54</t>
         </is>
       </c>
       <c r="AC14" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:30</t>
+          <t>7:00-16:54</t>
         </is>
       </c>
       <c r="AD14" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:30</t>
-        </is>
-      </c>
-      <c r="AE14" s="5" t="inlineStr">
-        <is>
-          <t>7:30-11:30</t>
-        </is>
-      </c>
+          <t>8:00-16:54</t>
+        </is>
+      </c>
+      <c r="AE14" s="5" t="n"/>
       <c r="AF14" s="6" t="n"/>
       <c r="AG14" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:00</t>
+          <t>7:00-15:36</t>
         </is>
       </c>
       <c r="AH14" s="5">
@@ -2610,7 +2603,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Medico Experto</t>
+          <t>Medio tiempo</t>
         </is>
       </c>
       <c r="D15" s="6" t="n"/>
@@ -2643,27 +2636,27 @@
       <c r="K15" s="6" t="n"/>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>14:00-18:00</t>
+          <t>14:00-16:48</t>
         </is>
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
-          <t>14:00-18:00</t>
+          <t>14:00-16:48</t>
         </is>
       </c>
       <c r="N15" s="5" t="inlineStr">
         <is>
-          <t>14:00-18:00</t>
+          <t>14:00-16:48</t>
         </is>
       </c>
       <c r="O15" s="5" t="inlineStr">
         <is>
-          <t>13:00-18:00</t>
+          <t>13:00-16:48</t>
         </is>
       </c>
       <c r="P15" s="5" t="inlineStr">
         <is>
-          <t>14:00-18:00</t>
+          <t>14:00-16:48</t>
         </is>
       </c>
       <c r="Q15" s="5" t="inlineStr">
@@ -2697,38 +2690,38 @@
           <t>14:00-18:00</t>
         </is>
       </c>
-      <c r="X15" s="5" t="inlineStr">
-        <is>
-          <t>7:00-13:00</t>
-        </is>
-      </c>
+      <c r="X15" s="5" t="n"/>
       <c r="Y15" s="6" t="n"/>
       <c r="Z15" s="5" t="inlineStr">
         <is>
-          <t>14:00-18:00</t>
+          <t>14:00-16:48</t>
         </is>
       </c>
       <c r="AA15" s="5" t="inlineStr">
         <is>
-          <t>14:00-18:00</t>
+          <t>14:00-16:48</t>
         </is>
       </c>
       <c r="AB15" s="5" t="inlineStr">
         <is>
-          <t>14:00-18:00</t>
+          <t>14:00-16:48</t>
         </is>
       </c>
       <c r="AC15" s="5" t="inlineStr">
         <is>
-          <t>13:00-18:00</t>
+          <t>13:00-16:48</t>
         </is>
       </c>
       <c r="AD15" s="5" t="inlineStr">
         <is>
-          <t>14:00-18:00</t>
-        </is>
-      </c>
-      <c r="AE15" s="6" t="n"/>
+          <t>14:00-16:48</t>
+        </is>
+      </c>
+      <c r="AE15" s="5" t="inlineStr">
+        <is>
+          <t>7:00-13:00</t>
+        </is>
+      </c>
       <c r="AF15" s="6" t="n"/>
       <c r="AG15" s="5" t="inlineStr">
         <is>
@@ -5230,6 +5223,11 @@
           <t>S</t>
         </is>
       </c>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>Total semana</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="9">
@@ -5237,10 +5235,14 @@
         <v/>
       </c>
       <c r="B34" s="5" t="n">
-        <v>39.5</v>
+        <v>38</v>
       </c>
       <c r="C34" s="5" t="n">
-        <v>2.5</v>
+        <v>4</v>
+      </c>
+      <c r="D34" s="14">
+        <f>B34+C34</f>
+        <v/>
       </c>
     </row>
     <row r="35">
@@ -5249,10 +5251,14 @@
         <v/>
       </c>
       <c r="B35" s="5" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C35" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="D35" s="14">
+        <f>B35+C35</f>
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -5261,10 +5267,14 @@
         <v/>
       </c>
       <c r="B36" s="5" t="n">
-        <v>39.5</v>
+        <v>38</v>
       </c>
       <c r="C36" s="5" t="n">
-        <v>2.5</v>
+        <v>4</v>
+      </c>
+      <c r="D36" s="14">
+        <f>B36+C36</f>
+        <v/>
       </c>
     </row>
     <row r="37">
@@ -5273,10 +5283,14 @@
         <v/>
       </c>
       <c r="B37" s="5" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C37" s="5" t="n">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="D37" s="14">
+        <f>B37+C37</f>
+        <v/>
       </c>
     </row>
     <row r="38">
@@ -5285,10 +5299,14 @@
         <v/>
       </c>
       <c r="B38" s="5" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C38" s="5" t="n">
-        <v>3</v>
+        <v>5</v>
+      </c>
+      <c r="D38" s="14">
+        <f>B38+C38</f>
+        <v/>
       </c>
     </row>
     <row r="39">
@@ -5297,10 +5315,14 @@
         <v/>
       </c>
       <c r="B39" s="5" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C39" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="D39" s="14">
+        <f>B39+C39</f>
+        <v/>
       </c>
     </row>
     <row r="40">
@@ -5314,6 +5336,10 @@
       <c r="C40" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="D40" s="14">
+        <f>B40+C40</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9">
@@ -5326,6 +5352,10 @@
       <c r="C41" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="D41" s="14">
+        <f>B41+C41</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="9">
@@ -5333,10 +5363,14 @@
         <v/>
       </c>
       <c r="B42" s="5" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C42" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="D42" s="14">
+        <f>B42+C42</f>
+        <v/>
       </c>
     </row>
     <row r="43">
@@ -5345,10 +5379,14 @@
         <v/>
       </c>
       <c r="B43" s="5" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C43" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="D43" s="14">
+        <f>B43+C43</f>
+        <v/>
       </c>
     </row>
     <row r="44">
@@ -5362,6 +5400,10 @@
       <c r="C44" s="5" t="n">
         <v>4</v>
       </c>
+      <c r="D44" s="14">
+        <f>B44+C44</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="9">
@@ -5369,10 +5411,14 @@
         <v/>
       </c>
       <c r="B45" s="5" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C45" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="D45" s="14">
+        <f>B45+C45</f>
+        <v/>
       </c>
     </row>
     <row r="46">
@@ -5381,10 +5427,14 @@
         <v/>
       </c>
       <c r="B46" s="5" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C46" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="D46" s="14">
+        <f>B46+C46</f>
+        <v/>
       </c>
     </row>
     <row r="47">
@@ -5393,10 +5443,14 @@
         <v/>
       </c>
       <c r="B47" s="5" t="n">
-        <v>21.5</v>
+        <v>15</v>
       </c>
       <c r="C47" s="5" t="n">
-        <v>1.5</v>
+        <v>6</v>
+      </c>
+      <c r="D47" s="14">
+        <f>B47+C47</f>
+        <v/>
       </c>
     </row>
     <row r="49">
@@ -5426,7 +5480,7 @@
       </c>
       <c r="B51" s="11" t="inlineStr">
         <is>
-          <t>Paula Bermúdez: hasta el 5 nov (regresa el 6) · Dr. Daniel Cortes: 9 al 30 nov.</t>
+          <t>Médicos: 7 Dr. Daniel y Dr. Nicolás Mahecha · 14 Dr. Fabio y Dra. Mafe · 21 Dr. Nicolás Mahecha · 28 Dr. Fabio y Dra. Mafe.</t>
         </is>
       </c>
     </row>
@@ -5438,15 +5492,19 @@
       </c>
       <c r="B52" s="11" t="inlineStr">
         <is>
-          <t>Médicos: 7 Dr. Daniel · 14 Dr. Fabio y Dra. Mafe · 21 Dr. Fabio · 28 Dra. Mafe.</t>
+          <t>Nicolás Torres, jefe Marly, Alejandra, Sandra y Paula: 7 y 21 · Damaris: 14 y 28 · Kiria: 14 y 21 · Mileidy y Diana Lasso: todos los sábados.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="10" t="inlineStr"/>
+      <c r="A53" s="10" t="inlineStr">
+        <is>
+          <t>Jornada</t>
+        </is>
+      </c>
       <c r="B53" s="11" t="inlineStr">
         <is>
-          <t>Nicolás, Damaris y jefe Marly: 14 y 28 · Kiria, Alejandra y Sandra: 7 y 21 · Paula: 14 y 28 · Mileidy y Daniel Salas: todos los sábados.</t>
+          <t>Tiempo completo 42 h/semana, medio tiempo 21 h/semana. En semanas con sábado se reduce la salida L-V; en semanas sin sábado se amplía. Semanas con festivo suman menos porque el festivo es día no laborado.</t>
         </is>
       </c>
     </row>
@@ -5463,41 +5521,12 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AM6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="11" customWidth="1" min="19" max="19"/>
-    <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="11" customWidth="1" min="21" max="21"/>
-    <col width="11" customWidth="1" min="22" max="22"/>
-    <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="11" customWidth="1" min="24" max="24"/>
-    <col width="11" customWidth="1" min="25" max="25"/>
-    <col width="11" customWidth="1" min="26" max="26"/>
-    <col width="11" customWidth="1" min="27" max="27"/>
-    <col width="11" customWidth="1" min="28" max="28"/>
-    <col width="11" customWidth="1" min="29" max="29"/>
-    <col width="11" customWidth="1" min="30" max="30"/>
-    <col width="11" customWidth="1" min="31" max="31"/>
-    <col width="11" customWidth="1" min="32" max="32"/>
-    <col width="11" customWidth="1" min="33" max="33"/>
+    <col width="11" customWidth="1" min="4" max="33"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5683,7 +5712,11 @@
           <t>Auxiliar Serv G</t>
         </is>
       </c>
-      <c r="C2" s="5" t="n"/>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 12 a 1pm</t>
+        </is>
+      </c>
       <c r="D2" s="6" t="n"/>
       <c r="E2" s="7" t="inlineStr">
         <is>
@@ -5692,22 +5725,22 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:00</t>
+          <t>6:00-14:36</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:00</t>
+          <t>6:00-14:36</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:00</t>
+          <t>6:00-14:36</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:00</t>
+          <t>6:00-14:36</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
@@ -5718,27 +5751,27 @@
       <c r="K2" s="6" t="n"/>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>11:00-19:00</t>
+          <t>9:36-19:00</t>
         </is>
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>11:00-19:00</t>
+          <t>9:36-19:00</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
-          <t>11:00-19:00</t>
+          <t>9:36-19:00</t>
         </is>
       </c>
       <c r="O2" s="5" t="inlineStr">
         <is>
-          <t>11:00-19:00</t>
+          <t>9:36-19:00</t>
         </is>
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>11:00-19:00</t>
+          <t>9:36-19:00</t>
         </is>
       </c>
       <c r="Q2" s="6" t="n"/>
@@ -5750,22 +5783,22 @@
       </c>
       <c r="T2" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:00</t>
+          <t>6:00-14:36</t>
         </is>
       </c>
       <c r="U2" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:00</t>
+          <t>6:00-14:36</t>
         </is>
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:00</t>
+          <t>6:00-14:36</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:00</t>
+          <t>6:00-14:36</t>
         </is>
       </c>
       <c r="X2" s="5" t="inlineStr">
@@ -5776,34 +5809,34 @@
       <c r="Y2" s="6" t="n"/>
       <c r="Z2" s="5" t="inlineStr">
         <is>
-          <t>11:00-19:00</t>
+          <t>9:36-19:00</t>
         </is>
       </c>
       <c r="AA2" s="5" t="inlineStr">
         <is>
-          <t>11:00-19:00</t>
+          <t>9:36-19:00</t>
         </is>
       </c>
       <c r="AB2" s="5" t="inlineStr">
         <is>
-          <t>11:00-19:00</t>
+          <t>9:36-19:00</t>
         </is>
       </c>
       <c r="AC2" s="5" t="inlineStr">
         <is>
-          <t>11:00-19:00</t>
+          <t>9:36-19:00</t>
         </is>
       </c>
       <c r="AD2" s="5" t="inlineStr">
         <is>
-          <t>11:00-19:00</t>
+          <t>9:36-19:00</t>
         </is>
       </c>
       <c r="AE2" s="6" t="n"/>
       <c r="AF2" s="6" t="n"/>
       <c r="AG2" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:00</t>
+          <t>6:00-14:36</t>
         </is>
       </c>
       <c r="AH2" s="5">
@@ -5835,49 +5868,49 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>11:00-19:00</t>
+          <t>9:36-19:00</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>11:00-19:00</t>
+          <t>9:36-19:00</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>11:00-19:00</t>
+          <t>9:36-19:00</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>11:00-19:00</t>
+          <t>9:36-19:00</t>
         </is>
       </c>
       <c r="J3" s="6" t="n"/>
       <c r="K3" s="6" t="n"/>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:00</t>
+          <t>6:00-14:36</t>
         </is>
       </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:00</t>
+          <t>6:00-14:36</t>
         </is>
       </c>
       <c r="N3" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:00</t>
+          <t>6:00-14:36</t>
         </is>
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:00</t>
+          <t>6:00-14:36</t>
         </is>
       </c>
       <c r="P3" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:00</t>
+          <t>6:00-14:36</t>
         </is>
       </c>
       <c r="Q3" s="5" t="inlineStr">
@@ -5893,49 +5926,49 @@
       </c>
       <c r="T3" s="5" t="inlineStr">
         <is>
-          <t>11:00-19:00</t>
+          <t>9:36-19:00</t>
         </is>
       </c>
       <c r="U3" s="5" t="inlineStr">
         <is>
-          <t>11:00-19:00</t>
+          <t>9:36-19:00</t>
         </is>
       </c>
       <c r="V3" s="5" t="inlineStr">
         <is>
-          <t>11:00-19:00</t>
+          <t>9:36-19:00</t>
         </is>
       </c>
       <c r="W3" s="5" t="inlineStr">
         <is>
-          <t>11:00-19:00</t>
+          <t>9:36-19:00</t>
         </is>
       </c>
       <c r="X3" s="6" t="n"/>
       <c r="Y3" s="6" t="n"/>
       <c r="Z3" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:00</t>
+          <t>6:00-14:36</t>
         </is>
       </c>
       <c r="AA3" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:00</t>
+          <t>6:00-14:36</t>
         </is>
       </c>
       <c r="AB3" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:00</t>
+          <t>6:00-14:36</t>
         </is>
       </c>
       <c r="AC3" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:00</t>
+          <t>6:00-14:36</t>
         </is>
       </c>
       <c r="AD3" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:00</t>
+          <t>6:00-14:36</t>
         </is>
       </c>
       <c r="AE3" s="5" t="inlineStr">
@@ -5946,7 +5979,7 @@
       <c r="AF3" s="6" t="n"/>
       <c r="AG3" s="5" t="inlineStr">
         <is>
-          <t>11:00-19:00</t>
+          <t>9:36-19:00</t>
         </is>
       </c>
       <c r="AH3" s="5">
@@ -6002,23 +6035,23 @@
         <v/>
       </c>
       <c r="E5">
-        <f>IF(E2="",0,IFERROR((TIMEVALUE(MID(E2,FIND("-",E2)+1,10))-TIMEVALUE(LEFT(E2,FIND("-",E2)-1)))*24,0))</f>
+        <f>IF(E2="",0,IFERROR((TIMEVALUE(MID(E2,FIND("-",E2)+1,10))-TIMEVALUE(LEFT(E2,FIND("-",E2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="F5">
-        <f>IF(F2="",0,IFERROR((TIMEVALUE(MID(F2,FIND("-",F2)+1,10))-TIMEVALUE(LEFT(F2,FIND("-",F2)-1)))*24,0))</f>
+        <f>IF(F2="",0,IFERROR((TIMEVALUE(MID(F2,FIND("-",F2)+1,10))-TIMEVALUE(LEFT(F2,FIND("-",F2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="G5">
-        <f>IF(G2="",0,IFERROR((TIMEVALUE(MID(G2,FIND("-",G2)+1,10))-TIMEVALUE(LEFT(G2,FIND("-",G2)-1)))*24,0))</f>
+        <f>IF(G2="",0,IFERROR((TIMEVALUE(MID(G2,FIND("-",G2)+1,10))-TIMEVALUE(LEFT(G2,FIND("-",G2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="H5">
-        <f>IF(H2="",0,IFERROR((TIMEVALUE(MID(H2,FIND("-",H2)+1,10))-TIMEVALUE(LEFT(H2,FIND("-",H2)-1)))*24,0))</f>
+        <f>IF(H2="",0,IFERROR((TIMEVALUE(MID(H2,FIND("-",H2)+1,10))-TIMEVALUE(LEFT(H2,FIND("-",H2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="I5">
-        <f>IF(I2="",0,IFERROR((TIMEVALUE(MID(I2,FIND("-",I2)+1,10))-TIMEVALUE(LEFT(I2,FIND("-",I2)-1)))*24,0))</f>
+        <f>IF(I2="",0,IFERROR((TIMEVALUE(MID(I2,FIND("-",I2)+1,10))-TIMEVALUE(LEFT(I2,FIND("-",I2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="J5">
@@ -6030,23 +6063,23 @@
         <v/>
       </c>
       <c r="L5">
-        <f>IF(L2="",0,IFERROR((TIMEVALUE(MID(L2,FIND("-",L2)+1,10))-TIMEVALUE(LEFT(L2,FIND("-",L2)-1)))*24,0))</f>
+        <f>IF(L2="",0,IFERROR((TIMEVALUE(MID(L2,FIND("-",L2)+1,10))-TIMEVALUE(LEFT(L2,FIND("-",L2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="M5">
-        <f>IF(M2="",0,IFERROR((TIMEVALUE(MID(M2,FIND("-",M2)+1,10))-TIMEVALUE(LEFT(M2,FIND("-",M2)-1)))*24,0))</f>
+        <f>IF(M2="",0,IFERROR((TIMEVALUE(MID(M2,FIND("-",M2)+1,10))-TIMEVALUE(LEFT(M2,FIND("-",M2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="N5">
-        <f>IF(N2="",0,IFERROR((TIMEVALUE(MID(N2,FIND("-",N2)+1,10))-TIMEVALUE(LEFT(N2,FIND("-",N2)-1)))*24,0))</f>
+        <f>IF(N2="",0,IFERROR((TIMEVALUE(MID(N2,FIND("-",N2)+1,10))-TIMEVALUE(LEFT(N2,FIND("-",N2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="O5">
-        <f>IF(O2="",0,IFERROR((TIMEVALUE(MID(O2,FIND("-",O2)+1,10))-TIMEVALUE(LEFT(O2,FIND("-",O2)-1)))*24,0))</f>
+        <f>IF(O2="",0,IFERROR((TIMEVALUE(MID(O2,FIND("-",O2)+1,10))-TIMEVALUE(LEFT(O2,FIND("-",O2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="P5">
-        <f>IF(P2="",0,IFERROR((TIMEVALUE(MID(P2,FIND("-",P2)+1,10))-TIMEVALUE(LEFT(P2,FIND("-",P2)-1)))*24,0))</f>
+        <f>IF(P2="",0,IFERROR((TIMEVALUE(MID(P2,FIND("-",P2)+1,10))-TIMEVALUE(LEFT(P2,FIND("-",P2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="Q5">
@@ -6058,23 +6091,23 @@
         <v/>
       </c>
       <c r="S5">
-        <f>IF(S2="",0,IFERROR((TIMEVALUE(MID(S2,FIND("-",S2)+1,10))-TIMEVALUE(LEFT(S2,FIND("-",S2)-1)))*24,0))</f>
+        <f>IF(S2="",0,IFERROR((TIMEVALUE(MID(S2,FIND("-",S2)+1,10))-TIMEVALUE(LEFT(S2,FIND("-",S2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="T5">
-        <f>IF(T2="",0,IFERROR((TIMEVALUE(MID(T2,FIND("-",T2)+1,10))-TIMEVALUE(LEFT(T2,FIND("-",T2)-1)))*24,0))</f>
+        <f>IF(T2="",0,IFERROR((TIMEVALUE(MID(T2,FIND("-",T2)+1,10))-TIMEVALUE(LEFT(T2,FIND("-",T2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="U5">
-        <f>IF(U2="",0,IFERROR((TIMEVALUE(MID(U2,FIND("-",U2)+1,10))-TIMEVALUE(LEFT(U2,FIND("-",U2)-1)))*24,0))</f>
+        <f>IF(U2="",0,IFERROR((TIMEVALUE(MID(U2,FIND("-",U2)+1,10))-TIMEVALUE(LEFT(U2,FIND("-",U2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="V5">
-        <f>IF(V2="",0,IFERROR((TIMEVALUE(MID(V2,FIND("-",V2)+1,10))-TIMEVALUE(LEFT(V2,FIND("-",V2)-1)))*24,0))</f>
+        <f>IF(V2="",0,IFERROR((TIMEVALUE(MID(V2,FIND("-",V2)+1,10))-TIMEVALUE(LEFT(V2,FIND("-",V2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="W5">
-        <f>IF(W2="",0,IFERROR((TIMEVALUE(MID(W2,FIND("-",W2)+1,10))-TIMEVALUE(LEFT(W2,FIND("-",W2)-1)))*24,0))</f>
+        <f>IF(W2="",0,IFERROR((TIMEVALUE(MID(W2,FIND("-",W2)+1,10))-TIMEVALUE(LEFT(W2,FIND("-",W2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="X5">
@@ -6086,23 +6119,23 @@
         <v/>
       </c>
       <c r="Z5">
-        <f>IF(Z2="",0,IFERROR((TIMEVALUE(MID(Z2,FIND("-",Z2)+1,10))-TIMEVALUE(LEFT(Z2,FIND("-",Z2)-1)))*24,0))</f>
+        <f>IF(Z2="",0,IFERROR((TIMEVALUE(MID(Z2,FIND("-",Z2)+1,10))-TIMEVALUE(LEFT(Z2,FIND("-",Z2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="AA5">
-        <f>IF(AA2="",0,IFERROR((TIMEVALUE(MID(AA2,FIND("-",AA2)+1,10))-TIMEVALUE(LEFT(AA2,FIND("-",AA2)-1)))*24,0))</f>
+        <f>IF(AA2="",0,IFERROR((TIMEVALUE(MID(AA2,FIND("-",AA2)+1,10))-TIMEVALUE(LEFT(AA2,FIND("-",AA2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="AB5">
-        <f>IF(AB2="",0,IFERROR((TIMEVALUE(MID(AB2,FIND("-",AB2)+1,10))-TIMEVALUE(LEFT(AB2,FIND("-",AB2)-1)))*24,0))</f>
+        <f>IF(AB2="",0,IFERROR((TIMEVALUE(MID(AB2,FIND("-",AB2)+1,10))-TIMEVALUE(LEFT(AB2,FIND("-",AB2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="AC5">
-        <f>IF(AC2="",0,IFERROR((TIMEVALUE(MID(AC2,FIND("-",AC2)+1,10))-TIMEVALUE(LEFT(AC2,FIND("-",AC2)-1)))*24,0))</f>
+        <f>IF(AC2="",0,IFERROR((TIMEVALUE(MID(AC2,FIND("-",AC2)+1,10))-TIMEVALUE(LEFT(AC2,FIND("-",AC2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="AD5">
-        <f>IF(AD2="",0,IFERROR((TIMEVALUE(MID(AD2,FIND("-",AD2)+1,10))-TIMEVALUE(LEFT(AD2,FIND("-",AD2)-1)))*24,0))</f>
+        <f>IF(AD2="",0,IFERROR((TIMEVALUE(MID(AD2,FIND("-",AD2)+1,10))-TIMEVALUE(LEFT(AD2,FIND("-",AD2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="AE5">
@@ -6114,7 +6147,7 @@
         <v/>
       </c>
       <c r="AG5">
-        <f>IF(AG2="",0,IFERROR((TIMEVALUE(MID(AG2,FIND("-",AG2)+1,10))-TIMEVALUE(LEFT(AG2,FIND("-",AG2)-1)))*24,0))</f>
+        <f>IF(AG2="",0,IFERROR((TIMEVALUE(MID(AG2,FIND("-",AG2)+1,10))-TIMEVALUE(LEFT(AG2,FIND("-",AG2)-1)))*24-1,0))</f>
         <v/>
       </c>
       <c r="AH5">
@@ -6305,41 +6338,12 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AG6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="11" customWidth="1" min="19" max="19"/>
-    <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="11" customWidth="1" min="21" max="21"/>
-    <col width="11" customWidth="1" min="22" max="22"/>
-    <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="11" customWidth="1" min="24" max="24"/>
-    <col width="11" customWidth="1" min="25" max="25"/>
-    <col width="11" customWidth="1" min="26" max="26"/>
-    <col width="11" customWidth="1" min="27" max="27"/>
-    <col width="11" customWidth="1" min="28" max="28"/>
-    <col width="11" customWidth="1" min="29" max="29"/>
-    <col width="11" customWidth="1" min="30" max="30"/>
-    <col width="11" customWidth="1" min="31" max="31"/>
-    <col width="11" customWidth="1" min="32" max="32"/>
-    <col width="11" customWidth="1" min="33" max="33"/>
+    <col width="11" customWidth="1" min="4" max="33"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Noviembre 2026: balancear horas por quincena en lugar de por semana
Quien trabaja sábado cada 15 días mantiene el mismo horario L-V todas las
semanas y la quincena suma 84 h (42 h medio tiempo); las horas de festivo
no se reponen. Se revierten los ajustes semanales anteriores y solo se
modifican los horarios que no cuadraban.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QFEyfDRz3kAA5d3tShZ31H
</commit_message>
<xml_diff>
--- a/TURNOS_Noviembre_2026.xlsx
+++ b/TURNOS_Noviembre_2026.xlsx
@@ -222,7 +222,7 @@
     </comment>
     <comment ref="C13" authorId="0" shapeId="0">
       <text>
-        <t>Nov-2026 (42 h/semana): semanas con sábado (7 y 21, igual que Nicolás Torres) L-V 7:00-15:36 + sáb 8:00-12:00; semanas sin sábado L-V 7:00-16:24.</t>
+        <t>Nov-2026: L-V 7:00-16:00 (8 h efectivas) + sábados 7 y 21 de 8:00-12:00 (igual que Nicolás Torres). 40 + 44 = 84 h por quincena.</t>
       </text>
     </comment>
     <comment ref="A14" authorId="0" shapeId="0">
@@ -232,7 +232,7 @@
     </comment>
     <comment ref="B33" authorId="0" shapeId="0">
       <text>
-        <t>L-V en semanas con sábado. En semanas sin sábado L-V = 42 h (21 h medio tiempo).</t>
+        <t>Horas L-V por semana (iguales todas las semanas). S = horas del sábado. Quien va sábado cada 15 días: L-V x2 + sábado = 84 h por quincena (42 h medio tiempo).</t>
       </text>
     </comment>
     <comment ref="B44" authorId="0" shapeId="0">
@@ -739,22 +739,22 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:06</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:06</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:06</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:36</t>
+          <t>8:00-17:00</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
@@ -890,22 +890,22 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>7:30-10:54</t>
+          <t>7:30-11:00</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>7:30-10:54</t>
+          <t>7:30-11:30</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>7:30-10:54</t>
+          <t>7:30-11:30</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>7:30-10:54</t>
+          <t>7:30-11:30</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr">
@@ -916,27 +916,27 @@
       <c r="K3" s="6" t="n"/>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:42</t>
+          <t>7:30-11:00</t>
         </is>
       </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:42</t>
+          <t>7:30-11:00</t>
         </is>
       </c>
       <c r="N3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:42</t>
+          <t>7:30-11:30</t>
         </is>
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:42</t>
+          <t>7:30-11:30</t>
         </is>
       </c>
       <c r="P3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:42</t>
+          <t>7:30-11:30</t>
         </is>
       </c>
       <c r="Q3" s="6" t="n"/>
@@ -948,22 +948,22 @@
       </c>
       <c r="T3" s="5" t="inlineStr">
         <is>
-          <t>7:30-10:54</t>
+          <t>7:30-11:00</t>
         </is>
       </c>
       <c r="U3" s="5" t="inlineStr">
         <is>
-          <t>7:30-10:54</t>
+          <t>7:30-11:30</t>
         </is>
       </c>
       <c r="V3" s="5" t="inlineStr">
         <is>
-          <t>7:30-10:54</t>
+          <t>7:30-11:30</t>
         </is>
       </c>
       <c r="W3" s="5" t="inlineStr">
         <is>
-          <t>7:30-10:54</t>
+          <t>7:30-11:30</t>
         </is>
       </c>
       <c r="X3" s="6" t="inlineStr">
@@ -974,34 +974,34 @@
       <c r="Y3" s="6" t="n"/>
       <c r="Z3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:42</t>
+          <t>7:30-11:00</t>
         </is>
       </c>
       <c r="AA3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:42</t>
+          <t>7:30-11:00</t>
         </is>
       </c>
       <c r="AB3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:42</t>
+          <t>7:30-11:30</t>
         </is>
       </c>
       <c r="AC3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:42</t>
+          <t>7:30-11:30</t>
         </is>
       </c>
       <c r="AD3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:42</t>
+          <t>7:30-11:30</t>
         </is>
       </c>
       <c r="AE3" s="6" t="n"/>
       <c r="AF3" s="6" t="n"/>
       <c r="AG3" s="5" t="inlineStr">
         <is>
-          <t>7:30-10:54</t>
+          <t>7:30-11:00</t>
         </is>
       </c>
       <c r="AH3" s="5">
@@ -1033,44 +1033,44 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:18</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:18</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:18</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:48</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="6" t="n"/>
       <c r="L4" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:30</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:30</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:30</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:30</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="P4" s="5" t="inlineStr">
@@ -1091,44 +1091,44 @@
       </c>
       <c r="T4" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:18</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="U4" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:18</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:18</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:48</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="X4" s="6" t="n"/>
       <c r="Y4" s="6" t="n"/>
       <c r="Z4" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:30</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="AA4" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:30</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="AB4" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:30</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="AC4" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:30</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="AD4" s="5" t="inlineStr">
@@ -1144,7 +1144,7 @@
       <c r="AF4" s="6" t="n"/>
       <c r="AG4" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:18</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="AH4" s="5">
@@ -1176,49 +1176,49 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>8:24-18:00</t>
+          <t>9:00-18:00</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>8:24-18:00</t>
+          <t>9:00-18:00</t>
         </is>
       </c>
       <c r="J5" s="5" t="n"/>
       <c r="K5" s="6" t="n"/>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>10:00-17:24</t>
+          <t>10:00-18:00</t>
         </is>
       </c>
       <c r="M5" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>9:00-17:24</t>
+          <t>9:00-18:00</t>
         </is>
       </c>
       <c r="O5" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="P5" s="5" t="inlineStr">
         <is>
-          <t>9:00-17:24</t>
+          <t>9:00-18:00</t>
         </is>
       </c>
       <c r="Q5" s="5" t="inlineStr">
@@ -1234,22 +1234,22 @@
       </c>
       <c r="T5" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="U5" s="5" t="inlineStr">
         <is>
-          <t>9:00-17:24</t>
+          <t>9:00-18:00</t>
         </is>
       </c>
       <c r="V5" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="W5" s="5" t="inlineStr">
         <is>
-          <t>9:00-17:24</t>
+          <t>9:00-18:00</t>
         </is>
       </c>
       <c r="X5" s="5" t="inlineStr">
@@ -1260,34 +1260,34 @@
       <c r="Y5" s="6" t="n"/>
       <c r="Z5" s="5" t="inlineStr">
         <is>
-          <t>9:24-18:00</t>
+          <t>10:00-18:00</t>
         </is>
       </c>
       <c r="AA5" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="AB5" s="5" t="inlineStr">
         <is>
-          <t>8:24-18:00</t>
+          <t>9:00-18:00</t>
         </is>
       </c>
       <c r="AC5" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="AD5" s="5" t="inlineStr">
         <is>
-          <t>8:24-18:00</t>
+          <t>9:00-18:00</t>
         </is>
       </c>
       <c r="AE5" s="6" t="n"/>
       <c r="AF5" s="6" t="n"/>
       <c r="AG5" s="5" t="inlineStr">
         <is>
-          <t>10:00-17:24</t>
+          <t>10:00-18:00</t>
         </is>
       </c>
       <c r="AH5" s="5">
@@ -1319,49 +1319,49 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>8:24-18:00</t>
+          <t>9:00-18:00</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>8:24-18:00</t>
+          <t>9:00-18:00</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="J6" s="6" t="n"/>
       <c r="K6" s="6" t="n"/>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>7:00-14:36</t>
+          <t>7:00-15:30</t>
         </is>
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>9:00-17:36</t>
+          <t>9:00-18:00</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>9:00-17:36</t>
+          <t>9:00-18:00</t>
         </is>
       </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="Q6" s="5" t="inlineStr">
@@ -1377,49 +1377,49 @@
       </c>
       <c r="T6" s="5" t="inlineStr">
         <is>
-          <t>8:24-18:00</t>
+          <t>9:00-18:00</t>
         </is>
       </c>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>8:24-18:00</t>
+          <t>9:00-18:00</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="X6" s="6" t="n"/>
       <c r="Y6" s="6" t="n"/>
       <c r="Z6" s="5" t="inlineStr">
         <is>
-          <t>7:00-14:36</t>
+          <t>7:00-15:30</t>
         </is>
       </c>
       <c r="AA6" s="5" t="inlineStr">
         <is>
-          <t>9:00-17:36</t>
+          <t>9:00-18:00</t>
         </is>
       </c>
       <c r="AB6" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="AC6" s="5" t="inlineStr">
         <is>
-          <t>9:00-17:36</t>
+          <t>9:00-18:00</t>
         </is>
       </c>
       <c r="AD6" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="AE6" s="5" t="inlineStr">
@@ -1430,7 +1430,7 @@
       <c r="AF6" s="6" t="n"/>
       <c r="AG6" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-15:30</t>
         </is>
       </c>
       <c r="AH6" s="5">
@@ -1462,49 +1462,49 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:42</t>
+          <t>7:30-17:00</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:42</t>
+          <t>7:30-17:00</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:42</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:42</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="J7" s="6" t="n"/>
       <c r="K7" s="6" t="n"/>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>7:30-17:42</t>
+          <t>7:30-17:30</t>
         </is>
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:42</t>
+          <t>7:30-17:00</t>
         </is>
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:42</t>
+          <t>7:30-17:00</t>
         </is>
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:42</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="P7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:42</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="Q7" s="6" t="n"/>
@@ -1516,56 +1516,56 @@
       </c>
       <c r="T7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:42</t>
+          <t>7:30-17:00</t>
         </is>
       </c>
       <c r="U7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:42</t>
+          <t>7:30-17:00</t>
         </is>
       </c>
       <c r="V7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:42</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="W7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:42</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="X7" s="6" t="n"/>
       <c r="Y7" s="6" t="n"/>
       <c r="Z7" s="5" t="inlineStr">
         <is>
-          <t>7:30-17:42</t>
+          <t>7:30-17:30</t>
         </is>
       </c>
       <c r="AA7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:42</t>
+          <t>7:30-17:00</t>
         </is>
       </c>
       <c r="AB7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:42</t>
+          <t>7:30-17:00</t>
         </is>
       </c>
       <c r="AC7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:42</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="AD7" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:42</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="AE7" s="6" t="n"/>
       <c r="AF7" s="6" t="n"/>
       <c r="AG7" s="5" t="inlineStr">
         <is>
-          <t>7:30-17:42</t>
+          <t>7:30-17:30</t>
         </is>
       </c>
       <c r="AH7" s="5">
@@ -1899,22 +1899,22 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:06</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:06</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:06</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:06</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
@@ -1925,27 +1925,27 @@
       <c r="K10" s="6" t="n"/>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:54</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:54</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:54</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="O10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:54</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:54</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="Q10" s="6" t="n"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="T10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:06</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:06</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:06</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:06</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="X10" s="5" t="inlineStr">
@@ -1983,34 +1983,34 @@
       <c r="Y10" s="6" t="n"/>
       <c r="Z10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:54</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="AA10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:54</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="AB10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:54</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="AC10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:54</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="AD10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:54</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="AE10" s="6" t="n"/>
       <c r="AF10" s="6" t="n"/>
       <c r="AG10" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:06</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="AH10" s="5">
@@ -2042,22 +2042,22 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:06</t>
+          <t>7:00-16:30</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:06</t>
+          <t>8:00-16:30</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:06</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:06</t>
+          <t>7:00-16:30</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
@@ -2068,27 +2068,27 @@
       <c r="K11" s="6" t="n"/>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:54</t>
+          <t>8:00-16:30</t>
         </is>
       </c>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:54</t>
+          <t>7:00-16:30</t>
         </is>
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:54</t>
+          <t>8:00-16:30</t>
         </is>
       </c>
       <c r="O11" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:54</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="P11" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:54</t>
+          <t>7:00-16:30</t>
         </is>
       </c>
       <c r="Q11" s="5" t="n"/>
@@ -2100,22 +2100,22 @@
       </c>
       <c r="T11" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:06</t>
+          <t>7:00-16:30</t>
         </is>
       </c>
       <c r="U11" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:06</t>
+          <t>8:00-16:30</t>
         </is>
       </c>
       <c r="V11" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:06</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="W11" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:06</t>
+          <t>7:00-16:30</t>
         </is>
       </c>
       <c r="X11" s="5" t="inlineStr">
@@ -2126,34 +2126,34 @@
       <c r="Y11" s="6" t="n"/>
       <c r="Z11" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:54</t>
+          <t>8:00-16:30</t>
         </is>
       </c>
       <c r="AA11" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:54</t>
+          <t>7:00-16:30</t>
         </is>
       </c>
       <c r="AB11" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:54</t>
+          <t>8:00-16:30</t>
         </is>
       </c>
       <c r="AC11" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:54</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="AD11" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:54</t>
+          <t>7:00-16:30</t>
         </is>
       </c>
       <c r="AE11" s="6" t="n"/>
       <c r="AF11" s="6" t="n"/>
       <c r="AG11" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:06</t>
+          <t>8:00-16:30</t>
         </is>
       </c>
       <c r="AH11" s="5">
@@ -2185,22 +2185,22 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
@@ -2211,27 +2211,27 @@
       <c r="K12" s="5" t="n"/>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="O12" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="Q12" s="5" t="n"/>
@@ -2243,22 +2243,22 @@
       </c>
       <c r="T12" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="X12" s="5" t="inlineStr">
@@ -2269,34 +2269,34 @@
       <c r="Y12" s="5" t="n"/>
       <c r="Z12" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="AA12" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="AB12" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="AC12" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="AD12" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="AE12" s="5" t="n"/>
       <c r="AF12" s="6" t="n"/>
       <c r="AG12" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="AH12" s="5">
@@ -2328,22 +2328,22 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:06</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
@@ -2354,27 +2354,27 @@
       <c r="K13" s="6" t="n"/>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:54</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="O13" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="P13" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:54</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="Q13" s="6" t="n"/>
@@ -2386,22 +2386,22 @@
       </c>
       <c r="T13" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="U13" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="V13" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="W13" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:06</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="X13" s="5" t="inlineStr">
@@ -2412,34 +2412,34 @@
       <c r="Y13" s="6" t="n"/>
       <c r="Z13" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:54</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="AA13" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="AB13" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="AC13" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="AD13" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:54</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="AE13" s="6" t="n"/>
       <c r="AF13" s="6" t="n"/>
       <c r="AG13" s="5" t="inlineStr">
         <is>
-          <t>7:30-16:06</t>
+          <t>7:30-16:30</t>
         </is>
       </c>
       <c r="AH13" s="5">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:06</t>
+          <t>8:00-16:30</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
@@ -2497,27 +2497,27 @@
       <c r="K14" s="6" t="n"/>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:54</t>
+          <t>8:00-16:30</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:54</t>
+          <t>7:00-16:30</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:54</t>
+          <t>7:00-16:30</t>
         </is>
       </c>
       <c r="P14" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:54</t>
+          <t>8:00-16:30</t>
         </is>
       </c>
       <c r="Q14" s="5" t="n"/>
@@ -2529,22 +2529,22 @@
       </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:06</t>
+          <t>8:00-16:30</t>
         </is>
       </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:06</t>
+          <t>7:00-16:30</t>
         </is>
       </c>
       <c r="V14" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:06</t>
+          <t>7:00-16:30</t>
         </is>
       </c>
       <c r="W14" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:06</t>
+          <t>8:00-16:30</t>
         </is>
       </c>
       <c r="X14" s="5" t="inlineStr">
@@ -2555,34 +2555,34 @@
       <c r="Y14" s="6" t="n"/>
       <c r="Z14" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:24</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="AA14" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:54</t>
+          <t>8:00-16:30</t>
         </is>
       </c>
       <c r="AB14" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:54</t>
+          <t>7:00-16:30</t>
         </is>
       </c>
       <c r="AC14" s="5" t="inlineStr">
         <is>
-          <t>7:00-16:54</t>
+          <t>7:00-16:30</t>
         </is>
       </c>
       <c r="AD14" s="5" t="inlineStr">
         <is>
-          <t>8:00-16:54</t>
+          <t>8:00-16:30</t>
         </is>
       </c>
       <c r="AE14" s="5" t="n"/>
       <c r="AF14" s="6" t="n"/>
       <c r="AG14" s="5" t="inlineStr">
         <is>
-          <t>7:00-15:36</t>
+          <t>7:00-16:00</t>
         </is>
       </c>
       <c r="AH14" s="5">
@@ -2614,17 +2614,17 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>14:00-18:00</t>
+          <t>14:30-18:00</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>14:00-18:00</t>
+          <t>14:30-18:00</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>13:00-18:00</t>
+          <t>14:30-18:00</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
@@ -2636,27 +2636,27 @@
       <c r="K15" s="6" t="n"/>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>14:00-16:48</t>
+          <t>14:30-18:00</t>
         </is>
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
-          <t>14:00-16:48</t>
+          <t>14:30-18:00</t>
         </is>
       </c>
       <c r="N15" s="5" t="inlineStr">
         <is>
-          <t>14:00-16:48</t>
+          <t>14:30-18:00</t>
         </is>
       </c>
       <c r="O15" s="5" t="inlineStr">
         <is>
-          <t>13:00-16:48</t>
+          <t>14:30-18:00</t>
         </is>
       </c>
       <c r="P15" s="5" t="inlineStr">
         <is>
-          <t>14:00-16:48</t>
+          <t>14:00-18:00</t>
         </is>
       </c>
       <c r="Q15" s="5" t="inlineStr">
@@ -2672,17 +2672,17 @@
       </c>
       <c r="T15" s="5" t="inlineStr">
         <is>
-          <t>14:00-18:00</t>
+          <t>14:30-18:00</t>
         </is>
       </c>
       <c r="U15" s="5" t="inlineStr">
         <is>
-          <t>14:00-18:00</t>
+          <t>14:30-18:00</t>
         </is>
       </c>
       <c r="V15" s="5" t="inlineStr">
         <is>
-          <t>13:00-18:00</t>
+          <t>14:30-18:00</t>
         </is>
       </c>
       <c r="W15" s="5" t="inlineStr">
@@ -2694,27 +2694,27 @@
       <c r="Y15" s="6" t="n"/>
       <c r="Z15" s="5" t="inlineStr">
         <is>
-          <t>14:00-16:48</t>
+          <t>14:30-18:00</t>
         </is>
       </c>
       <c r="AA15" s="5" t="inlineStr">
         <is>
-          <t>14:00-16:48</t>
+          <t>14:30-18:00</t>
         </is>
       </c>
       <c r="AB15" s="5" t="inlineStr">
         <is>
-          <t>14:00-16:48</t>
+          <t>14:30-18:00</t>
         </is>
       </c>
       <c r="AC15" s="5" t="inlineStr">
         <is>
-          <t>13:00-16:48</t>
+          <t>14:30-18:00</t>
         </is>
       </c>
       <c r="AD15" s="5" t="inlineStr">
         <is>
-          <t>14:00-16:48</t>
+          <t>14:00-18:00</t>
         </is>
       </c>
       <c r="AE15" s="5" t="inlineStr">
@@ -2725,7 +2725,7 @@
       <c r="AF15" s="6" t="n"/>
       <c r="AG15" s="5" t="inlineStr">
         <is>
-          <t>14:00-18:00</t>
+          <t>14:30-18:00</t>
         </is>
       </c>
       <c r="AH15" s="5">
@@ -5225,7 +5225,7 @@
       </c>
       <c r="D33" s="13" t="inlineStr">
         <is>
-          <t>Total semana</t>
+          <t>Prom. semanal</t>
         </is>
       </c>
     </row>
@@ -5235,13 +5235,13 @@
         <v/>
       </c>
       <c r="B34" s="5" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C34" s="5" t="n">
         <v>4</v>
       </c>
       <c r="D34" s="14">
-        <f>B34+C34</f>
+        <f>B34+C34*0.5</f>
         <v/>
       </c>
     </row>
@@ -5251,13 +5251,13 @@
         <v/>
       </c>
       <c r="B35" s="5" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C35" s="5" t="n">
         <v>4</v>
       </c>
       <c r="D35" s="14">
-        <f>B35+C35</f>
+        <f>B35+C35*0.5</f>
         <v/>
       </c>
     </row>
@@ -5267,13 +5267,13 @@
         <v/>
       </c>
       <c r="B36" s="5" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C36" s="5" t="n">
         <v>4</v>
       </c>
       <c r="D36" s="14">
-        <f>B36+C36</f>
+        <f>B36+C36*0.5</f>
         <v/>
       </c>
     </row>
@@ -5283,13 +5283,13 @@
         <v/>
       </c>
       <c r="B37" s="5" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C37" s="5" t="n">
         <v>6</v>
       </c>
       <c r="D37" s="14">
-        <f>B37+C37</f>
+        <f>B37+C37*0.5</f>
         <v/>
       </c>
     </row>
@@ -5299,13 +5299,13 @@
         <v/>
       </c>
       <c r="B38" s="5" t="n">
-        <v>37</v>
+        <v>39.5</v>
       </c>
       <c r="C38" s="5" t="n">
         <v>5</v>
       </c>
       <c r="D38" s="14">
-        <f>B38+C38</f>
+        <f>B38+C38*0.5</f>
         <v/>
       </c>
     </row>
@@ -5321,7 +5321,7 @@
         <v>0</v>
       </c>
       <c r="D39" s="14">
-        <f>B39+C39</f>
+        <f>B39</f>
         <v/>
       </c>
     </row>
@@ -5363,13 +5363,13 @@
         <v/>
       </c>
       <c r="B42" s="5" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C42" s="5" t="n">
         <v>4</v>
       </c>
       <c r="D42" s="14">
-        <f>B42+C42</f>
+        <f>B42+C42*0.5</f>
         <v/>
       </c>
     </row>
@@ -5379,13 +5379,13 @@
         <v/>
       </c>
       <c r="B43" s="5" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C43" s="5" t="n">
         <v>4</v>
       </c>
       <c r="D43" s="14">
-        <f>B43+C43</f>
+        <f>B43+C43*0.5</f>
         <v/>
       </c>
     </row>
@@ -5395,13 +5395,13 @@
         <v/>
       </c>
       <c r="B44" s="5" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C44" s="5" t="n">
         <v>4</v>
       </c>
       <c r="D44" s="14">
-        <f>B44+C44</f>
+        <f>B44+C44*0.5</f>
         <v/>
       </c>
     </row>
@@ -5411,13 +5411,13 @@
         <v/>
       </c>
       <c r="B45" s="5" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C45" s="5" t="n">
         <v>4</v>
       </c>
       <c r="D45" s="14">
-        <f>B45+C45</f>
+        <f>B45+C45*0.5</f>
         <v/>
       </c>
     </row>
@@ -5427,13 +5427,13 @@
         <v/>
       </c>
       <c r="B46" s="5" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C46" s="5" t="n">
         <v>4</v>
       </c>
       <c r="D46" s="14">
-        <f>B46+C46</f>
+        <f>B46+C46*0.5</f>
         <v/>
       </c>
     </row>
@@ -5443,13 +5443,13 @@
         <v/>
       </c>
       <c r="B47" s="5" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C47" s="5" t="n">
         <v>6</v>
       </c>
       <c r="D47" s="14">
-        <f>B47+C47</f>
+        <f>B47+C47*0.5</f>
         <v/>
       </c>
     </row>
@@ -5504,7 +5504,7 @@
       </c>
       <c r="B53" s="11" t="inlineStr">
         <is>
-          <t>Tiempo completo 42 h/semana, medio tiempo 21 h/semana. En semanas con sábado se reduce la salida L-V; en semanas sin sábado se amplía. Semanas con festivo suman menos porque el festivo es día no laborado.</t>
+          <t>Tiempo completo 42 h/semana y medio tiempo 21 h/semana, balanceado por quincena: la semana con sábado suma más y la siguiente menos (ej. 44 + 40 = 84 h). Las horas de los festivos no se reponen.</t>
         </is>
       </c>
     </row>
@@ -5725,22 +5725,22 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:36</t>
+          <t>6:00-15:00</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:36</t>
+          <t>6:00-15:00</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:36</t>
+          <t>6:00-15:00</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:36</t>
+          <t>6:00-15:00</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
@@ -5751,27 +5751,27 @@
       <c r="K2" s="6" t="n"/>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>9:36-19:00</t>
+          <t>10:00-19:00</t>
         </is>
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>9:36-19:00</t>
+          <t>10:00-19:00</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
-          <t>9:36-19:00</t>
+          <t>10:00-19:00</t>
         </is>
       </c>
       <c r="O2" s="5" t="inlineStr">
         <is>
-          <t>9:36-19:00</t>
+          <t>10:00-19:00</t>
         </is>
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>9:36-19:00</t>
+          <t>10:00-19:00</t>
         </is>
       </c>
       <c r="Q2" s="6" t="n"/>
@@ -5783,22 +5783,22 @@
       </c>
       <c r="T2" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:36</t>
+          <t>6:00-15:00</t>
         </is>
       </c>
       <c r="U2" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:36</t>
+          <t>6:00-15:00</t>
         </is>
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:36</t>
+          <t>6:00-15:00</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:36</t>
+          <t>6:00-15:00</t>
         </is>
       </c>
       <c r="X2" s="5" t="inlineStr">
@@ -5809,34 +5809,34 @@
       <c r="Y2" s="6" t="n"/>
       <c r="Z2" s="5" t="inlineStr">
         <is>
-          <t>9:36-19:00</t>
+          <t>10:00-19:00</t>
         </is>
       </c>
       <c r="AA2" s="5" t="inlineStr">
         <is>
-          <t>9:36-19:00</t>
+          <t>10:00-19:00</t>
         </is>
       </c>
       <c r="AB2" s="5" t="inlineStr">
         <is>
-          <t>9:36-19:00</t>
+          <t>10:00-19:00</t>
         </is>
       </c>
       <c r="AC2" s="5" t="inlineStr">
         <is>
-          <t>9:36-19:00</t>
+          <t>10:00-19:00</t>
         </is>
       </c>
       <c r="AD2" s="5" t="inlineStr">
         <is>
-          <t>9:36-19:00</t>
+          <t>10:00-19:00</t>
         </is>
       </c>
       <c r="AE2" s="6" t="n"/>
       <c r="AF2" s="6" t="n"/>
       <c r="AG2" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:36</t>
+          <t>6:00-15:00</t>
         </is>
       </c>
       <c r="AH2" s="5">
@@ -5868,49 +5868,49 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>9:36-19:00</t>
+          <t>10:00-19:00</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>9:36-19:00</t>
+          <t>10:00-19:00</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>9:36-19:00</t>
+          <t>10:00-19:00</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>9:36-19:00</t>
+          <t>10:00-19:00</t>
         </is>
       </c>
       <c r="J3" s="6" t="n"/>
       <c r="K3" s="6" t="n"/>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:36</t>
+          <t>6:00-15:00</t>
         </is>
       </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:36</t>
+          <t>6:00-15:00</t>
         </is>
       </c>
       <c r="N3" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:36</t>
+          <t>6:00-15:00</t>
         </is>
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:36</t>
+          <t>6:00-15:00</t>
         </is>
       </c>
       <c r="P3" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:36</t>
+          <t>6:00-15:00</t>
         </is>
       </c>
       <c r="Q3" s="5" t="inlineStr">
@@ -5926,49 +5926,49 @@
       </c>
       <c r="T3" s="5" t="inlineStr">
         <is>
-          <t>9:36-19:00</t>
+          <t>10:00-19:00</t>
         </is>
       </c>
       <c r="U3" s="5" t="inlineStr">
         <is>
-          <t>9:36-19:00</t>
+          <t>10:00-19:00</t>
         </is>
       </c>
       <c r="V3" s="5" t="inlineStr">
         <is>
-          <t>9:36-19:00</t>
+          <t>10:00-19:00</t>
         </is>
       </c>
       <c r="W3" s="5" t="inlineStr">
         <is>
-          <t>9:36-19:00</t>
+          <t>10:00-19:00</t>
         </is>
       </c>
       <c r="X3" s="6" t="n"/>
       <c r="Y3" s="6" t="n"/>
       <c r="Z3" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:36</t>
+          <t>6:00-15:00</t>
         </is>
       </c>
       <c r="AA3" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:36</t>
+          <t>6:00-15:00</t>
         </is>
       </c>
       <c r="AB3" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:36</t>
+          <t>6:00-15:00</t>
         </is>
       </c>
       <c r="AC3" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:36</t>
+          <t>6:00-15:00</t>
         </is>
       </c>
       <c r="AD3" s="5" t="inlineStr">
         <is>
-          <t>6:00-14:36</t>
+          <t>6:00-15:00</t>
         </is>
       </c>
       <c r="AE3" s="5" t="inlineStr">
@@ -5979,7 +5979,7 @@
       <c r="AF3" s="6" t="n"/>
       <c r="AG3" s="5" t="inlineStr">
         <is>
-          <t>9:36-19:00</t>
+          <t>10:00-19:00</t>
         </is>
       </c>
       <c r="AH3" s="5">

</xml_diff>

<commit_message>
Noviembre 2026: Nicolás Mahecha L-V 7:30-11:30 y sábados 8:00-10:00
Se recorta el sábado en lugar de los días de semana: 20 + 20 + 2 = 42 h
por quincena (medio tiempo).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QFEyfDRz3kAA5d3tShZ31H
</commit_message>
<xml_diff>
--- a/TURNOS_Noviembre_2026.xlsx
+++ b/TURNOS_Noviembre_2026.xlsx
@@ -890,7 +890,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:00</t>
+          <t>7:30-11:30</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
@@ -910,18 +910,18 @@
       </c>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>8:00-12:00</t>
+          <t>8:00-10:00</t>
         </is>
       </c>
       <c r="K3" s="6" t="n"/>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:00</t>
+          <t>7:30-11:30</t>
         </is>
       </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:00</t>
+          <t>7:30-11:30</t>
         </is>
       </c>
       <c r="N3" s="5" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="T3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:00</t>
+          <t>7:30-11:30</t>
         </is>
       </c>
       <c r="U3" s="5" t="inlineStr">
@@ -968,18 +968,18 @@
       </c>
       <c r="X3" s="6" t="inlineStr">
         <is>
-          <t>8:00-12:00</t>
+          <t>8:00-10:00</t>
         </is>
       </c>
       <c r="Y3" s="6" t="n"/>
       <c r="Z3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:00</t>
+          <t>7:30-11:30</t>
         </is>
       </c>
       <c r="AA3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:00</t>
+          <t>7:30-11:30</t>
         </is>
       </c>
       <c r="AB3" s="5" t="inlineStr">
@@ -1001,7 +1001,7 @@
       <c r="AF3" s="6" t="n"/>
       <c r="AG3" s="5" t="inlineStr">
         <is>
-          <t>7:30-11:00</t>
+          <t>7:30-11:30</t>
         </is>
       </c>
       <c r="AH3" s="5">
@@ -5251,10 +5251,10 @@
         <v/>
       </c>
       <c r="B35" s="5" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C35" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D35" s="14">
         <f>B35+C35*0.5</f>

</xml_diff>

<commit_message>
Noviembre 2026: restaurar turnos de Herlinda y Nataly (6-14 / 11-19) sin descuento de almuerzo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QFEyfDRz3kAA5d3tShZ31H
</commit_message>
<xml_diff>
--- a/TURNOS_Noviembre_2026.xlsx
+++ b/TURNOS_Noviembre_2026.xlsx
@@ -5712,11 +5712,7 @@
           <t>Auxiliar Serv G</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 12 a 1pm</t>
-        </is>
-      </c>
+      <c r="C2" s="5" t="n"/>
       <c r="D2" s="6" t="n"/>
       <c r="E2" s="7" t="inlineStr">
         <is>
@@ -5725,22 +5721,22 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>6:00-15:00</t>
+          <t>6:00-14:00</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>6:00-15:00</t>
+          <t>6:00-14:00</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>6:00-15:00</t>
+          <t>6:00-14:00</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>6:00-15:00</t>
+          <t>6:00-14:00</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
@@ -5751,27 +5747,27 @@
       <c r="K2" s="6" t="n"/>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>10:00-19:00</t>
+          <t>11:00-19:00</t>
         </is>
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>10:00-19:00</t>
+          <t>11:00-19:00</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
-          <t>10:00-19:00</t>
+          <t>11:00-19:00</t>
         </is>
       </c>
       <c r="O2" s="5" t="inlineStr">
         <is>
-          <t>10:00-19:00</t>
+          <t>11:00-19:00</t>
         </is>
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>10:00-19:00</t>
+          <t>11:00-19:00</t>
         </is>
       </c>
       <c r="Q2" s="6" t="n"/>
@@ -5783,22 +5779,22 @@
       </c>
       <c r="T2" s="5" t="inlineStr">
         <is>
-          <t>6:00-15:00</t>
+          <t>6:00-14:00</t>
         </is>
       </c>
       <c r="U2" s="5" t="inlineStr">
         <is>
-          <t>6:00-15:00</t>
+          <t>6:00-14:00</t>
         </is>
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>6:00-15:00</t>
+          <t>6:00-14:00</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
         <is>
-          <t>6:00-15:00</t>
+          <t>6:00-14:00</t>
         </is>
       </c>
       <c r="X2" s="5" t="inlineStr">
@@ -5809,34 +5805,34 @@
       <c r="Y2" s="6" t="n"/>
       <c r="Z2" s="5" t="inlineStr">
         <is>
-          <t>10:00-19:00</t>
+          <t>11:00-19:00</t>
         </is>
       </c>
       <c r="AA2" s="5" t="inlineStr">
         <is>
-          <t>10:00-19:00</t>
+          <t>11:00-19:00</t>
         </is>
       </c>
       <c r="AB2" s="5" t="inlineStr">
         <is>
-          <t>10:00-19:00</t>
+          <t>11:00-19:00</t>
         </is>
       </c>
       <c r="AC2" s="5" t="inlineStr">
         <is>
-          <t>10:00-19:00</t>
+          <t>11:00-19:00</t>
         </is>
       </c>
       <c r="AD2" s="5" t="inlineStr">
         <is>
-          <t>10:00-19:00</t>
+          <t>11:00-19:00</t>
         </is>
       </c>
       <c r="AE2" s="6" t="n"/>
       <c r="AF2" s="6" t="n"/>
       <c r="AG2" s="5" t="inlineStr">
         <is>
-          <t>6:00-15:00</t>
+          <t>6:00-14:00</t>
         </is>
       </c>
       <c r="AH2" s="5">
@@ -5868,49 +5864,49 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>10:00-19:00</t>
+          <t>11:00-19:00</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>10:00-19:00</t>
+          <t>11:00-19:00</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>10:00-19:00</t>
+          <t>11:00-19:00</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>10:00-19:00</t>
+          <t>11:00-19:00</t>
         </is>
       </c>
       <c r="J3" s="6" t="n"/>
       <c r="K3" s="6" t="n"/>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>6:00-15:00</t>
+          <t>6:00-14:00</t>
         </is>
       </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>6:00-15:00</t>
+          <t>6:00-14:00</t>
         </is>
       </c>
       <c r="N3" s="5" t="inlineStr">
         <is>
-          <t>6:00-15:00</t>
+          <t>6:00-14:00</t>
         </is>
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
-          <t>6:00-15:00</t>
+          <t>6:00-14:00</t>
         </is>
       </c>
       <c r="P3" s="5" t="inlineStr">
         <is>
-          <t>6:00-15:00</t>
+          <t>6:00-14:00</t>
         </is>
       </c>
       <c r="Q3" s="5" t="inlineStr">
@@ -5926,49 +5922,49 @@
       </c>
       <c r="T3" s="5" t="inlineStr">
         <is>
-          <t>10:00-19:00</t>
+          <t>11:00-19:00</t>
         </is>
       </c>
       <c r="U3" s="5" t="inlineStr">
         <is>
-          <t>10:00-19:00</t>
+          <t>11:00-19:00</t>
         </is>
       </c>
       <c r="V3" s="5" t="inlineStr">
         <is>
-          <t>10:00-19:00</t>
+          <t>11:00-19:00</t>
         </is>
       </c>
       <c r="W3" s="5" t="inlineStr">
         <is>
-          <t>10:00-19:00</t>
+          <t>11:00-19:00</t>
         </is>
       </c>
       <c r="X3" s="6" t="n"/>
       <c r="Y3" s="6" t="n"/>
       <c r="Z3" s="5" t="inlineStr">
         <is>
-          <t>6:00-15:00</t>
+          <t>6:00-14:00</t>
         </is>
       </c>
       <c r="AA3" s="5" t="inlineStr">
         <is>
-          <t>6:00-15:00</t>
+          <t>6:00-14:00</t>
         </is>
       </c>
       <c r="AB3" s="5" t="inlineStr">
         <is>
-          <t>6:00-15:00</t>
+          <t>6:00-14:00</t>
         </is>
       </c>
       <c r="AC3" s="5" t="inlineStr">
         <is>
-          <t>6:00-15:00</t>
+          <t>6:00-14:00</t>
         </is>
       </c>
       <c r="AD3" s="5" t="inlineStr">
         <is>
-          <t>6:00-15:00</t>
+          <t>6:00-14:00</t>
         </is>
       </c>
       <c r="AE3" s="5" t="inlineStr">
@@ -5979,7 +5975,7 @@
       <c r="AF3" s="6" t="n"/>
       <c r="AG3" s="5" t="inlineStr">
         <is>
-          <t>10:00-19:00</t>
+          <t>11:00-19:00</t>
         </is>
       </c>
       <c r="AH3" s="5">
@@ -6035,23 +6031,23 @@
         <v/>
       </c>
       <c r="E5">
-        <f>IF(E2="",0,IFERROR((TIMEVALUE(MID(E2,FIND("-",E2)+1,10))-TIMEVALUE(LEFT(E2,FIND("-",E2)-1)))*24-1,0))</f>
+        <f>IF(E2="",0,IFERROR((TIMEVALUE(MID(E2,FIND("-",E2)+1,10))-TIMEVALUE(LEFT(E2,FIND("-",E2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="F5">
-        <f>IF(F2="",0,IFERROR((TIMEVALUE(MID(F2,FIND("-",F2)+1,10))-TIMEVALUE(LEFT(F2,FIND("-",F2)-1)))*24-1,0))</f>
+        <f>IF(F2="",0,IFERROR((TIMEVALUE(MID(F2,FIND("-",F2)+1,10))-TIMEVALUE(LEFT(F2,FIND("-",F2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="G5">
-        <f>IF(G2="",0,IFERROR((TIMEVALUE(MID(G2,FIND("-",G2)+1,10))-TIMEVALUE(LEFT(G2,FIND("-",G2)-1)))*24-1,0))</f>
+        <f>IF(G2="",0,IFERROR((TIMEVALUE(MID(G2,FIND("-",G2)+1,10))-TIMEVALUE(LEFT(G2,FIND("-",G2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="H5">
-        <f>IF(H2="",0,IFERROR((TIMEVALUE(MID(H2,FIND("-",H2)+1,10))-TIMEVALUE(LEFT(H2,FIND("-",H2)-1)))*24-1,0))</f>
+        <f>IF(H2="",0,IFERROR((TIMEVALUE(MID(H2,FIND("-",H2)+1,10))-TIMEVALUE(LEFT(H2,FIND("-",H2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="I5">
-        <f>IF(I2="",0,IFERROR((TIMEVALUE(MID(I2,FIND("-",I2)+1,10))-TIMEVALUE(LEFT(I2,FIND("-",I2)-1)))*24-1,0))</f>
+        <f>IF(I2="",0,IFERROR((TIMEVALUE(MID(I2,FIND("-",I2)+1,10))-TIMEVALUE(LEFT(I2,FIND("-",I2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="J5">
@@ -6063,23 +6059,23 @@
         <v/>
       </c>
       <c r="L5">
-        <f>IF(L2="",0,IFERROR((TIMEVALUE(MID(L2,FIND("-",L2)+1,10))-TIMEVALUE(LEFT(L2,FIND("-",L2)-1)))*24-1,0))</f>
+        <f>IF(L2="",0,IFERROR((TIMEVALUE(MID(L2,FIND("-",L2)+1,10))-TIMEVALUE(LEFT(L2,FIND("-",L2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="M5">
-        <f>IF(M2="",0,IFERROR((TIMEVALUE(MID(M2,FIND("-",M2)+1,10))-TIMEVALUE(LEFT(M2,FIND("-",M2)-1)))*24-1,0))</f>
+        <f>IF(M2="",0,IFERROR((TIMEVALUE(MID(M2,FIND("-",M2)+1,10))-TIMEVALUE(LEFT(M2,FIND("-",M2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="N5">
-        <f>IF(N2="",0,IFERROR((TIMEVALUE(MID(N2,FIND("-",N2)+1,10))-TIMEVALUE(LEFT(N2,FIND("-",N2)-1)))*24-1,0))</f>
+        <f>IF(N2="",0,IFERROR((TIMEVALUE(MID(N2,FIND("-",N2)+1,10))-TIMEVALUE(LEFT(N2,FIND("-",N2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="O5">
-        <f>IF(O2="",0,IFERROR((TIMEVALUE(MID(O2,FIND("-",O2)+1,10))-TIMEVALUE(LEFT(O2,FIND("-",O2)-1)))*24-1,0))</f>
+        <f>IF(O2="",0,IFERROR((TIMEVALUE(MID(O2,FIND("-",O2)+1,10))-TIMEVALUE(LEFT(O2,FIND("-",O2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="P5">
-        <f>IF(P2="",0,IFERROR((TIMEVALUE(MID(P2,FIND("-",P2)+1,10))-TIMEVALUE(LEFT(P2,FIND("-",P2)-1)))*24-1,0))</f>
+        <f>IF(P2="",0,IFERROR((TIMEVALUE(MID(P2,FIND("-",P2)+1,10))-TIMEVALUE(LEFT(P2,FIND("-",P2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="Q5">
@@ -6091,23 +6087,23 @@
         <v/>
       </c>
       <c r="S5">
-        <f>IF(S2="",0,IFERROR((TIMEVALUE(MID(S2,FIND("-",S2)+1,10))-TIMEVALUE(LEFT(S2,FIND("-",S2)-1)))*24-1,0))</f>
+        <f>IF(S2="",0,IFERROR((TIMEVALUE(MID(S2,FIND("-",S2)+1,10))-TIMEVALUE(LEFT(S2,FIND("-",S2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="T5">
-        <f>IF(T2="",0,IFERROR((TIMEVALUE(MID(T2,FIND("-",T2)+1,10))-TIMEVALUE(LEFT(T2,FIND("-",T2)-1)))*24-1,0))</f>
+        <f>IF(T2="",0,IFERROR((TIMEVALUE(MID(T2,FIND("-",T2)+1,10))-TIMEVALUE(LEFT(T2,FIND("-",T2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="U5">
-        <f>IF(U2="",0,IFERROR((TIMEVALUE(MID(U2,FIND("-",U2)+1,10))-TIMEVALUE(LEFT(U2,FIND("-",U2)-1)))*24-1,0))</f>
+        <f>IF(U2="",0,IFERROR((TIMEVALUE(MID(U2,FIND("-",U2)+1,10))-TIMEVALUE(LEFT(U2,FIND("-",U2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="V5">
-        <f>IF(V2="",0,IFERROR((TIMEVALUE(MID(V2,FIND("-",V2)+1,10))-TIMEVALUE(LEFT(V2,FIND("-",V2)-1)))*24-1,0))</f>
+        <f>IF(V2="",0,IFERROR((TIMEVALUE(MID(V2,FIND("-",V2)+1,10))-TIMEVALUE(LEFT(V2,FIND("-",V2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="W5">
-        <f>IF(W2="",0,IFERROR((TIMEVALUE(MID(W2,FIND("-",W2)+1,10))-TIMEVALUE(LEFT(W2,FIND("-",W2)-1)))*24-1,0))</f>
+        <f>IF(W2="",0,IFERROR((TIMEVALUE(MID(W2,FIND("-",W2)+1,10))-TIMEVALUE(LEFT(W2,FIND("-",W2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="X5">
@@ -6119,23 +6115,23 @@
         <v/>
       </c>
       <c r="Z5">
-        <f>IF(Z2="",0,IFERROR((TIMEVALUE(MID(Z2,FIND("-",Z2)+1,10))-TIMEVALUE(LEFT(Z2,FIND("-",Z2)-1)))*24-1,0))</f>
+        <f>IF(Z2="",0,IFERROR((TIMEVALUE(MID(Z2,FIND("-",Z2)+1,10))-TIMEVALUE(LEFT(Z2,FIND("-",Z2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="AA5">
-        <f>IF(AA2="",0,IFERROR((TIMEVALUE(MID(AA2,FIND("-",AA2)+1,10))-TIMEVALUE(LEFT(AA2,FIND("-",AA2)-1)))*24-1,0))</f>
+        <f>IF(AA2="",0,IFERROR((TIMEVALUE(MID(AA2,FIND("-",AA2)+1,10))-TIMEVALUE(LEFT(AA2,FIND("-",AA2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="AB5">
-        <f>IF(AB2="",0,IFERROR((TIMEVALUE(MID(AB2,FIND("-",AB2)+1,10))-TIMEVALUE(LEFT(AB2,FIND("-",AB2)-1)))*24-1,0))</f>
+        <f>IF(AB2="",0,IFERROR((TIMEVALUE(MID(AB2,FIND("-",AB2)+1,10))-TIMEVALUE(LEFT(AB2,FIND("-",AB2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="AC5">
-        <f>IF(AC2="",0,IFERROR((TIMEVALUE(MID(AC2,FIND("-",AC2)+1,10))-TIMEVALUE(LEFT(AC2,FIND("-",AC2)-1)))*24-1,0))</f>
+        <f>IF(AC2="",0,IFERROR((TIMEVALUE(MID(AC2,FIND("-",AC2)+1,10))-TIMEVALUE(LEFT(AC2,FIND("-",AC2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="AD5">
-        <f>IF(AD2="",0,IFERROR((TIMEVALUE(MID(AD2,FIND("-",AD2)+1,10))-TIMEVALUE(LEFT(AD2,FIND("-",AD2)-1)))*24-1,0))</f>
+        <f>IF(AD2="",0,IFERROR((TIMEVALUE(MID(AD2,FIND("-",AD2)+1,10))-TIMEVALUE(LEFT(AD2,FIND("-",AD2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="AE5">
@@ -6147,7 +6143,7 @@
         <v/>
       </c>
       <c r="AG5">
-        <f>IF(AG2="",0,IFERROR((TIMEVALUE(MID(AG2,FIND("-",AG2)+1,10))-TIMEVALUE(LEFT(AG2,FIND("-",AG2)-1)))*24-1,0))</f>
+        <f>IF(AG2="",0,IFERROR((TIMEVALUE(MID(AG2,FIND("-",AG2)+1,10))-TIMEVALUE(LEFT(AG2,FIND("-",AG2)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="AH5">
@@ -6182,27 +6178,27 @@
         </is>
       </c>
       <c r="D6">
-        <f>IF(D3="",0,IFERROR((TIMEVALUE(MID(D3,FIND("-",D3)+1,10))-TIMEVALUE(LEFT(D3,FIND("-",D3)-1)))*24-1,0))</f>
+        <f>IF(D3="",0,IFERROR((TIMEVALUE(MID(D3,FIND("-",D3)+1,10))-TIMEVALUE(LEFT(D3,FIND("-",D3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="E6">
-        <f>IF(E3="",0,IFERROR((TIMEVALUE(MID(E3,FIND("-",E3)+1,10))-TIMEVALUE(LEFT(E3,FIND("-",E3)-1)))*24-1,0))</f>
+        <f>IF(E3="",0,IFERROR((TIMEVALUE(MID(E3,FIND("-",E3)+1,10))-TIMEVALUE(LEFT(E3,FIND("-",E3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="F6">
-        <f>IF(F3="",0,IFERROR((TIMEVALUE(MID(F3,FIND("-",F3)+1,10))-TIMEVALUE(LEFT(F3,FIND("-",F3)-1)))*24-1,0))</f>
+        <f>IF(F3="",0,IFERROR((TIMEVALUE(MID(F3,FIND("-",F3)+1,10))-TIMEVALUE(LEFT(F3,FIND("-",F3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="G6">
-        <f>IF(G3="",0,IFERROR((TIMEVALUE(MID(G3,FIND("-",G3)+1,10))-TIMEVALUE(LEFT(G3,FIND("-",G3)-1)))*24-1,0))</f>
+        <f>IF(G3="",0,IFERROR((TIMEVALUE(MID(G3,FIND("-",G3)+1,10))-TIMEVALUE(LEFT(G3,FIND("-",G3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="H6">
-        <f>IF(H3="",0,IFERROR((TIMEVALUE(MID(H3,FIND("-",H3)+1,10))-TIMEVALUE(LEFT(H3,FIND("-",H3)-1)))*24-1,0))</f>
+        <f>IF(H3="",0,IFERROR((TIMEVALUE(MID(H3,FIND("-",H3)+1,10))-TIMEVALUE(LEFT(H3,FIND("-",H3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="I6">
-        <f>IF(I3="",0,IFERROR((TIMEVALUE(MID(I3,FIND("-",I3)+1,10))-TIMEVALUE(LEFT(I3,FIND("-",I3)-1)))*24-1,0))</f>
+        <f>IF(I3="",0,IFERROR((TIMEVALUE(MID(I3,FIND("-",I3)+1,10))-TIMEVALUE(LEFT(I3,FIND("-",I3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="J6">
@@ -6210,27 +6206,27 @@
         <v/>
       </c>
       <c r="K6">
-        <f>IF(K3="",0,IFERROR((TIMEVALUE(MID(K3,FIND("-",K3)+1,10))-TIMEVALUE(LEFT(K3,FIND("-",K3)-1)))*24-1,0))</f>
+        <f>IF(K3="",0,IFERROR((TIMEVALUE(MID(K3,FIND("-",K3)+1,10))-TIMEVALUE(LEFT(K3,FIND("-",K3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="L6">
-        <f>IF(L3="",0,IFERROR((TIMEVALUE(MID(L3,FIND("-",L3)+1,10))-TIMEVALUE(LEFT(L3,FIND("-",L3)-1)))*24-1,0))</f>
+        <f>IF(L3="",0,IFERROR((TIMEVALUE(MID(L3,FIND("-",L3)+1,10))-TIMEVALUE(LEFT(L3,FIND("-",L3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="M6">
-        <f>IF(M3="",0,IFERROR((TIMEVALUE(MID(M3,FIND("-",M3)+1,10))-TIMEVALUE(LEFT(M3,FIND("-",M3)-1)))*24-1,0))</f>
+        <f>IF(M3="",0,IFERROR((TIMEVALUE(MID(M3,FIND("-",M3)+1,10))-TIMEVALUE(LEFT(M3,FIND("-",M3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="N6">
-        <f>IF(N3="",0,IFERROR((TIMEVALUE(MID(N3,FIND("-",N3)+1,10))-TIMEVALUE(LEFT(N3,FIND("-",N3)-1)))*24-1,0))</f>
+        <f>IF(N3="",0,IFERROR((TIMEVALUE(MID(N3,FIND("-",N3)+1,10))-TIMEVALUE(LEFT(N3,FIND("-",N3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="O6">
-        <f>IF(O3="",0,IFERROR((TIMEVALUE(MID(O3,FIND("-",O3)+1,10))-TIMEVALUE(LEFT(O3,FIND("-",O3)-1)))*24-1,0))</f>
+        <f>IF(O3="",0,IFERROR((TIMEVALUE(MID(O3,FIND("-",O3)+1,10))-TIMEVALUE(LEFT(O3,FIND("-",O3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="P6">
-        <f>IF(P3="",0,IFERROR((TIMEVALUE(MID(P3,FIND("-",P3)+1,10))-TIMEVALUE(LEFT(P3,FIND("-",P3)-1)))*24-1,0))</f>
+        <f>IF(P3="",0,IFERROR((TIMEVALUE(MID(P3,FIND("-",P3)+1,10))-TIMEVALUE(LEFT(P3,FIND("-",P3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="Q6">
@@ -6238,27 +6234,27 @@
         <v/>
       </c>
       <c r="R6">
-        <f>IF(R3="",0,IFERROR((TIMEVALUE(MID(R3,FIND("-",R3)+1,10))-TIMEVALUE(LEFT(R3,FIND("-",R3)-1)))*24-1,0))</f>
+        <f>IF(R3="",0,IFERROR((TIMEVALUE(MID(R3,FIND("-",R3)+1,10))-TIMEVALUE(LEFT(R3,FIND("-",R3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="S6">
-        <f>IF(S3="",0,IFERROR((TIMEVALUE(MID(S3,FIND("-",S3)+1,10))-TIMEVALUE(LEFT(S3,FIND("-",S3)-1)))*24-1,0))</f>
+        <f>IF(S3="",0,IFERROR((TIMEVALUE(MID(S3,FIND("-",S3)+1,10))-TIMEVALUE(LEFT(S3,FIND("-",S3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="T6">
-        <f>IF(T3="",0,IFERROR((TIMEVALUE(MID(T3,FIND("-",T3)+1,10))-TIMEVALUE(LEFT(T3,FIND("-",T3)-1)))*24-1,0))</f>
+        <f>IF(T3="",0,IFERROR((TIMEVALUE(MID(T3,FIND("-",T3)+1,10))-TIMEVALUE(LEFT(T3,FIND("-",T3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="U6">
-        <f>IF(U3="",0,IFERROR((TIMEVALUE(MID(U3,FIND("-",U3)+1,10))-TIMEVALUE(LEFT(U3,FIND("-",U3)-1)))*24-1,0))</f>
+        <f>IF(U3="",0,IFERROR((TIMEVALUE(MID(U3,FIND("-",U3)+1,10))-TIMEVALUE(LEFT(U3,FIND("-",U3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="V6">
-        <f>IF(V3="",0,IFERROR((TIMEVALUE(MID(V3,FIND("-",V3)+1,10))-TIMEVALUE(LEFT(V3,FIND("-",V3)-1)))*24-1,0))</f>
+        <f>IF(V3="",0,IFERROR((TIMEVALUE(MID(V3,FIND("-",V3)+1,10))-TIMEVALUE(LEFT(V3,FIND("-",V3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="W6">
-        <f>IF(W3="",0,IFERROR((TIMEVALUE(MID(W3,FIND("-",W3)+1,10))-TIMEVALUE(LEFT(W3,FIND("-",W3)-1)))*24-1,0))</f>
+        <f>IF(W3="",0,IFERROR((TIMEVALUE(MID(W3,FIND("-",W3)+1,10))-TIMEVALUE(LEFT(W3,FIND("-",W3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="X6">
@@ -6266,27 +6262,27 @@
         <v/>
       </c>
       <c r="Y6">
-        <f>IF(Y3="",0,IFERROR((TIMEVALUE(MID(Y3,FIND("-",Y3)+1,10))-TIMEVALUE(LEFT(Y3,FIND("-",Y3)-1)))*24-1,0))</f>
+        <f>IF(Y3="",0,IFERROR((TIMEVALUE(MID(Y3,FIND("-",Y3)+1,10))-TIMEVALUE(LEFT(Y3,FIND("-",Y3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="Z6">
-        <f>IF(Z3="",0,IFERROR((TIMEVALUE(MID(Z3,FIND("-",Z3)+1,10))-TIMEVALUE(LEFT(Z3,FIND("-",Z3)-1)))*24-1,0))</f>
+        <f>IF(Z3="",0,IFERROR((TIMEVALUE(MID(Z3,FIND("-",Z3)+1,10))-TIMEVALUE(LEFT(Z3,FIND("-",Z3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="AA6">
-        <f>IF(AA3="",0,IFERROR((TIMEVALUE(MID(AA3,FIND("-",AA3)+1,10))-TIMEVALUE(LEFT(AA3,FIND("-",AA3)-1)))*24-1,0))</f>
+        <f>IF(AA3="",0,IFERROR((TIMEVALUE(MID(AA3,FIND("-",AA3)+1,10))-TIMEVALUE(LEFT(AA3,FIND("-",AA3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="AB6">
-        <f>IF(AB3="",0,IFERROR((TIMEVALUE(MID(AB3,FIND("-",AB3)+1,10))-TIMEVALUE(LEFT(AB3,FIND("-",AB3)-1)))*24-1,0))</f>
+        <f>IF(AB3="",0,IFERROR((TIMEVALUE(MID(AB3,FIND("-",AB3)+1,10))-TIMEVALUE(LEFT(AB3,FIND("-",AB3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="AC6">
-        <f>IF(AC3="",0,IFERROR((TIMEVALUE(MID(AC3,FIND("-",AC3)+1,10))-TIMEVALUE(LEFT(AC3,FIND("-",AC3)-1)))*24-1,0))</f>
+        <f>IF(AC3="",0,IFERROR((TIMEVALUE(MID(AC3,FIND("-",AC3)+1,10))-TIMEVALUE(LEFT(AC3,FIND("-",AC3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="AD6">
-        <f>IF(AD3="",0,IFERROR((TIMEVALUE(MID(AD3,FIND("-",AD3)+1,10))-TIMEVALUE(LEFT(AD3,FIND("-",AD3)-1)))*24-1,0))</f>
+        <f>IF(AD3="",0,IFERROR((TIMEVALUE(MID(AD3,FIND("-",AD3)+1,10))-TIMEVALUE(LEFT(AD3,FIND("-",AD3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="AE6">
@@ -6294,11 +6290,11 @@
         <v/>
       </c>
       <c r="AF6">
-        <f>IF(AF3="",0,IFERROR((TIMEVALUE(MID(AF3,FIND("-",AF3)+1,10))-TIMEVALUE(LEFT(AF3,FIND("-",AF3)-1)))*24-1,0))</f>
+        <f>IF(AF3="",0,IFERROR((TIMEVALUE(MID(AF3,FIND("-",AF3)+1,10))-TIMEVALUE(LEFT(AF3,FIND("-",AF3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="AG6">
-        <f>IF(AG3="",0,IFERROR((TIMEVALUE(MID(AG3,FIND("-",AG3)+1,10))-TIMEVALUE(LEFT(AG3,FIND("-",AG3)-1)))*24-1,0))</f>
+        <f>IF(AG3="",0,IFERROR((TIMEVALUE(MID(AG3,FIND("-",AG3)+1,10))-TIMEVALUE(LEFT(AG3,FIND("-",AG3)-1)))*24,0))</f>
         <v/>
       </c>
       <c r="AH6">

</xml_diff>

<commit_message>
Noviembre 2026: fórmula de horas descuenta el almuerzo según la columna C
Horas = salida - entrada - duración del almuerzo indicado en 'Hora Almuerzo'
(solo L-V y solo si hay un horario). Medio tiempo y servicios generales sin
descuento.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QFEyfDRz3kAA5d3tShZ31H
</commit_message>
<xml_diff>
--- a/TURNOS_Noviembre_2026.xlsx
+++ b/TURNOS_Noviembre_2026.xlsx
@@ -228,6 +228,11 @@
     <comment ref="A14" authorId="0" shapeId="0">
       <text>
         <t>Vacaciones 15 oct - 5 nov 2026. Regresa el viernes 6 de noviembre.</t>
+      </text>
+    </comment>
+    <comment ref="C17" authorId="0" shapeId="0">
+      <text>
+        <t>Horas trabajadas = salida - entrada - almuerzo. El almuerzo se descuenta de lunes a viernes solo si la columna C tiene un horario (ej. 13:00-14:00). Sábados sin almuerzo.</t>
       </text>
     </comment>
     <comment ref="B33" authorId="0" shapeId="0">
@@ -2949,27 +2954,27 @@
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>IF(D2="",0,IFERROR((TIMEVALUE(MID(D2,FIND("-",D2)+1,10))-TIMEVALUE(LEFT(D2,FIND("-",D2)-1)))*24-1,0))</f>
+        <f>IF(D2="",0,IFERROR((TIMEVALUE(MID(D2,FIND("-",D2)+1,10))-TIMEVALUE(LEFT(D2,FIND("-",D2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>IF(E2="",0,IFERROR((TIMEVALUE(MID(E2,FIND("-",E2)+1,10))-TIMEVALUE(LEFT(E2,FIND("-",E2)-1)))*24-1,0))</f>
+        <f>IF(E2="",0,IFERROR((TIMEVALUE(MID(E2,FIND("-",E2)+1,10))-TIMEVALUE(LEFT(E2,FIND("-",E2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="F18" s="5">
-        <f>IF(F2="",0,IFERROR((TIMEVALUE(MID(F2,FIND("-",F2)+1,10))-TIMEVALUE(LEFT(F2,FIND("-",F2)-1)))*24-1,0))</f>
+        <f>IF(F2="",0,IFERROR((TIMEVALUE(MID(F2,FIND("-",F2)+1,10))-TIMEVALUE(LEFT(F2,FIND("-",F2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="G18" s="5">
-        <f>IF(G2="",0,IFERROR((TIMEVALUE(MID(G2,FIND("-",G2)+1,10))-TIMEVALUE(LEFT(G2,FIND("-",G2)-1)))*24-1,0))</f>
+        <f>IF(G2="",0,IFERROR((TIMEVALUE(MID(G2,FIND("-",G2)+1,10))-TIMEVALUE(LEFT(G2,FIND("-",G2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="H18" s="5">
-        <f>IF(H2="",0,IFERROR((TIMEVALUE(MID(H2,FIND("-",H2)+1,10))-TIMEVALUE(LEFT(H2,FIND("-",H2)-1)))*24-1,0))</f>
+        <f>IF(H2="",0,IFERROR((TIMEVALUE(MID(H2,FIND("-",H2)+1,10))-TIMEVALUE(LEFT(H2,FIND("-",H2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="I18" s="5">
-        <f>IF(I2="",0,IFERROR((TIMEVALUE(MID(I2,FIND("-",I2)+1,10))-TIMEVALUE(LEFT(I2,FIND("-",I2)-1)))*24-1,0))</f>
+        <f>IF(I2="",0,IFERROR((TIMEVALUE(MID(I2,FIND("-",I2)+1,10))-TIMEVALUE(LEFT(I2,FIND("-",I2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="J18" s="5">
@@ -2977,27 +2982,27 @@
         <v/>
       </c>
       <c r="K18" s="5">
-        <f>IF(K2="",0,IFERROR((TIMEVALUE(MID(K2,FIND("-",K2)+1,10))-TIMEVALUE(LEFT(K2,FIND("-",K2)-1)))*24-1,0))</f>
+        <f>IF(K2="",0,IFERROR((TIMEVALUE(MID(K2,FIND("-",K2)+1,10))-TIMEVALUE(LEFT(K2,FIND("-",K2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="L18" s="5">
-        <f>IF(L2="",0,IFERROR((TIMEVALUE(MID(L2,FIND("-",L2)+1,10))-TIMEVALUE(LEFT(L2,FIND("-",L2)-1)))*24-1,0))</f>
+        <f>IF(L2="",0,IFERROR((TIMEVALUE(MID(L2,FIND("-",L2)+1,10))-TIMEVALUE(LEFT(L2,FIND("-",L2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="M18" s="5">
-        <f>IF(M2="",0,IFERROR((TIMEVALUE(MID(M2,FIND("-",M2)+1,10))-TIMEVALUE(LEFT(M2,FIND("-",M2)-1)))*24-1,0))</f>
+        <f>IF(M2="",0,IFERROR((TIMEVALUE(MID(M2,FIND("-",M2)+1,10))-TIMEVALUE(LEFT(M2,FIND("-",M2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="N18" s="5">
-        <f>IF(N2="",0,IFERROR((TIMEVALUE(MID(N2,FIND("-",N2)+1,10))-TIMEVALUE(LEFT(N2,FIND("-",N2)-1)))*24-1,0))</f>
+        <f>IF(N2="",0,IFERROR((TIMEVALUE(MID(N2,FIND("-",N2)+1,10))-TIMEVALUE(LEFT(N2,FIND("-",N2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="O18" s="5">
-        <f>IF(O2="",0,IFERROR((TIMEVALUE(MID(O2,FIND("-",O2)+1,10))-TIMEVALUE(LEFT(O2,FIND("-",O2)-1)))*24-1,0))</f>
+        <f>IF(O2="",0,IFERROR((TIMEVALUE(MID(O2,FIND("-",O2)+1,10))-TIMEVALUE(LEFT(O2,FIND("-",O2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="P18" s="5">
-        <f>IF(P2="",0,IFERROR((TIMEVALUE(MID(P2,FIND("-",P2)+1,10))-TIMEVALUE(LEFT(P2,FIND("-",P2)-1)))*24-1,0))</f>
+        <f>IF(P2="",0,IFERROR((TIMEVALUE(MID(P2,FIND("-",P2)+1,10))-TIMEVALUE(LEFT(P2,FIND("-",P2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Q18" s="5">
@@ -3005,27 +3010,27 @@
         <v/>
       </c>
       <c r="R18" s="5">
-        <f>IF(R2="",0,IFERROR((TIMEVALUE(MID(R2,FIND("-",R2)+1,10))-TIMEVALUE(LEFT(R2,FIND("-",R2)-1)))*24-1,0))</f>
+        <f>IF(R2="",0,IFERROR((TIMEVALUE(MID(R2,FIND("-",R2)+1,10))-TIMEVALUE(LEFT(R2,FIND("-",R2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="S18" s="5">
-        <f>IF(S2="",0,IFERROR((TIMEVALUE(MID(S2,FIND("-",S2)+1,10))-TIMEVALUE(LEFT(S2,FIND("-",S2)-1)))*24-1,0))</f>
+        <f>IF(S2="",0,IFERROR((TIMEVALUE(MID(S2,FIND("-",S2)+1,10))-TIMEVALUE(LEFT(S2,FIND("-",S2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="T18" s="5">
-        <f>IF(T2="",0,IFERROR((TIMEVALUE(MID(T2,FIND("-",T2)+1,10))-TIMEVALUE(LEFT(T2,FIND("-",T2)-1)))*24-1,0))</f>
+        <f>IF(T2="",0,IFERROR((TIMEVALUE(MID(T2,FIND("-",T2)+1,10))-TIMEVALUE(LEFT(T2,FIND("-",T2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="U18" s="5">
-        <f>IF(U2="",0,IFERROR((TIMEVALUE(MID(U2,FIND("-",U2)+1,10))-TIMEVALUE(LEFT(U2,FIND("-",U2)-1)))*24-1,0))</f>
+        <f>IF(U2="",0,IFERROR((TIMEVALUE(MID(U2,FIND("-",U2)+1,10))-TIMEVALUE(LEFT(U2,FIND("-",U2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="V18" s="5">
-        <f>IF(V2="",0,IFERROR((TIMEVALUE(MID(V2,FIND("-",V2)+1,10))-TIMEVALUE(LEFT(V2,FIND("-",V2)-1)))*24-1,0))</f>
+        <f>IF(V2="",0,IFERROR((TIMEVALUE(MID(V2,FIND("-",V2)+1,10))-TIMEVALUE(LEFT(V2,FIND("-",V2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="W18" s="5">
-        <f>IF(W2="",0,IFERROR((TIMEVALUE(MID(W2,FIND("-",W2)+1,10))-TIMEVALUE(LEFT(W2,FIND("-",W2)-1)))*24-1,0))</f>
+        <f>IF(W2="",0,IFERROR((TIMEVALUE(MID(W2,FIND("-",W2)+1,10))-TIMEVALUE(LEFT(W2,FIND("-",W2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="X18" s="5">
@@ -3033,27 +3038,27 @@
         <v/>
       </c>
       <c r="Y18" s="5">
-        <f>IF(Y2="",0,IFERROR((TIMEVALUE(MID(Y2,FIND("-",Y2)+1,10))-TIMEVALUE(LEFT(Y2,FIND("-",Y2)-1)))*24-1,0))</f>
+        <f>IF(Y2="",0,IFERROR((TIMEVALUE(MID(Y2,FIND("-",Y2)+1,10))-TIMEVALUE(LEFT(Y2,FIND("-",Y2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Z18" s="5">
-        <f>IF(Z2="",0,IFERROR((TIMEVALUE(MID(Z2,FIND("-",Z2)+1,10))-TIMEVALUE(LEFT(Z2,FIND("-",Z2)-1)))*24-1,0))</f>
+        <f>IF(Z2="",0,IFERROR((TIMEVALUE(MID(Z2,FIND("-",Z2)+1,10))-TIMEVALUE(LEFT(Z2,FIND("-",Z2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AA18" s="5">
-        <f>IF(AA2="",0,IFERROR((TIMEVALUE(MID(AA2,FIND("-",AA2)+1,10))-TIMEVALUE(LEFT(AA2,FIND("-",AA2)-1)))*24-1,0))</f>
+        <f>IF(AA2="",0,IFERROR((TIMEVALUE(MID(AA2,FIND("-",AA2)+1,10))-TIMEVALUE(LEFT(AA2,FIND("-",AA2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AB18" s="5">
-        <f>IF(AB2="",0,IFERROR((TIMEVALUE(MID(AB2,FIND("-",AB2)+1,10))-TIMEVALUE(LEFT(AB2,FIND("-",AB2)-1)))*24-1,0))</f>
+        <f>IF(AB2="",0,IFERROR((TIMEVALUE(MID(AB2,FIND("-",AB2)+1,10))-TIMEVALUE(LEFT(AB2,FIND("-",AB2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AC18" s="5">
-        <f>IF(AC2="",0,IFERROR((TIMEVALUE(MID(AC2,FIND("-",AC2)+1,10))-TIMEVALUE(LEFT(AC2,FIND("-",AC2)-1)))*24-1,0))</f>
+        <f>IF(AC2="",0,IFERROR((TIMEVALUE(MID(AC2,FIND("-",AC2)+1,10))-TIMEVALUE(LEFT(AC2,FIND("-",AC2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AD18" s="5">
-        <f>IF(AD2="",0,IFERROR((TIMEVALUE(MID(AD2,FIND("-",AD2)+1,10))-TIMEVALUE(LEFT(AD2,FIND("-",AD2)-1)))*24-1,0))</f>
+        <f>IF(AD2="",0,IFERROR((TIMEVALUE(MID(AD2,FIND("-",AD2)+1,10))-TIMEVALUE(LEFT(AD2,FIND("-",AD2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AE18" s="5">
@@ -3061,11 +3066,11 @@
         <v/>
       </c>
       <c r="AF18" s="5">
-        <f>IF(AF2="",0,IFERROR((TIMEVALUE(MID(AF2,FIND("-",AF2)+1,10))-TIMEVALUE(LEFT(AF2,FIND("-",AF2)-1)))*24-1,0))</f>
+        <f>IF(AF2="",0,IFERROR((TIMEVALUE(MID(AF2,FIND("-",AF2)+1,10))-TIMEVALUE(LEFT(AF2,FIND("-",AF2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AG18" s="5">
-        <f>IF(AG2="",0,IFERROR((TIMEVALUE(MID(AG2,FIND("-",AG2)+1,10))-TIMEVALUE(LEFT(AG2,FIND("-",AG2)-1)))*24-1,0))</f>
+        <f>IF(AG2="",0,IFERROR((TIMEVALUE(MID(AG2,FIND("-",AG2)+1,10))-TIMEVALUE(LEFT(AG2,FIND("-",AG2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AH18" s="5">
@@ -3111,27 +3116,27 @@
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>IF(D3="",0,IFERROR((TIMEVALUE(MID(D3,FIND("-",D3)+1,10))-TIMEVALUE(LEFT(D3,FIND("-",D3)-1)))*24,0))</f>
+        <f>IF(D3="",0,IFERROR((TIMEVALUE(MID(D3,FIND("-",D3)+1,10))-TIMEVALUE(LEFT(D3,FIND("-",D3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>IF(E3="",0,IFERROR((TIMEVALUE(MID(E3,FIND("-",E3)+1,10))-TIMEVALUE(LEFT(E3,FIND("-",E3)-1)))*24,0))</f>
+        <f>IF(E3="",0,IFERROR((TIMEVALUE(MID(E3,FIND("-",E3)+1,10))-TIMEVALUE(LEFT(E3,FIND("-",E3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="F19" s="5">
-        <f>IF(F3="",0,IFERROR((TIMEVALUE(MID(F3,FIND("-",F3)+1,10))-TIMEVALUE(LEFT(F3,FIND("-",F3)-1)))*24,0))</f>
+        <f>IF(F3="",0,IFERROR((TIMEVALUE(MID(F3,FIND("-",F3)+1,10))-TIMEVALUE(LEFT(F3,FIND("-",F3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="G19" s="5">
-        <f>IF(G3="",0,IFERROR((TIMEVALUE(MID(G3,FIND("-",G3)+1,10))-TIMEVALUE(LEFT(G3,FIND("-",G3)-1)))*24,0))</f>
+        <f>IF(G3="",0,IFERROR((TIMEVALUE(MID(G3,FIND("-",G3)+1,10))-TIMEVALUE(LEFT(G3,FIND("-",G3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="H19" s="5">
-        <f>IF(H3="",0,IFERROR((TIMEVALUE(MID(H3,FIND("-",H3)+1,10))-TIMEVALUE(LEFT(H3,FIND("-",H3)-1)))*24,0))</f>
+        <f>IF(H3="",0,IFERROR((TIMEVALUE(MID(H3,FIND("-",H3)+1,10))-TIMEVALUE(LEFT(H3,FIND("-",H3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="I19" s="5">
-        <f>IF(I3="",0,IFERROR((TIMEVALUE(MID(I3,FIND("-",I3)+1,10))-TIMEVALUE(LEFT(I3,FIND("-",I3)-1)))*24,0))</f>
+        <f>IF(I3="",0,IFERROR((TIMEVALUE(MID(I3,FIND("-",I3)+1,10))-TIMEVALUE(LEFT(I3,FIND("-",I3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="J19" s="5">
@@ -3139,27 +3144,27 @@
         <v/>
       </c>
       <c r="K19" s="5">
-        <f>IF(K3="",0,IFERROR((TIMEVALUE(MID(K3,FIND("-",K3)+1,10))-TIMEVALUE(LEFT(K3,FIND("-",K3)-1)))*24,0))</f>
+        <f>IF(K3="",0,IFERROR((TIMEVALUE(MID(K3,FIND("-",K3)+1,10))-TIMEVALUE(LEFT(K3,FIND("-",K3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="L19" s="5">
-        <f>IF(L3="",0,IFERROR((TIMEVALUE(MID(L3,FIND("-",L3)+1,10))-TIMEVALUE(LEFT(L3,FIND("-",L3)-1)))*24,0))</f>
+        <f>IF(L3="",0,IFERROR((TIMEVALUE(MID(L3,FIND("-",L3)+1,10))-TIMEVALUE(LEFT(L3,FIND("-",L3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="M19" s="5">
-        <f>IF(M3="",0,IFERROR((TIMEVALUE(MID(M3,FIND("-",M3)+1,10))-TIMEVALUE(LEFT(M3,FIND("-",M3)-1)))*24,0))</f>
+        <f>IF(M3="",0,IFERROR((TIMEVALUE(MID(M3,FIND("-",M3)+1,10))-TIMEVALUE(LEFT(M3,FIND("-",M3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="N19" s="5">
-        <f>IF(N3="",0,IFERROR((TIMEVALUE(MID(N3,FIND("-",N3)+1,10))-TIMEVALUE(LEFT(N3,FIND("-",N3)-1)))*24,0))</f>
+        <f>IF(N3="",0,IFERROR((TIMEVALUE(MID(N3,FIND("-",N3)+1,10))-TIMEVALUE(LEFT(N3,FIND("-",N3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="O19" s="5">
-        <f>IF(O3="",0,IFERROR((TIMEVALUE(MID(O3,FIND("-",O3)+1,10))-TIMEVALUE(LEFT(O3,FIND("-",O3)-1)))*24,0))</f>
+        <f>IF(O3="",0,IFERROR((TIMEVALUE(MID(O3,FIND("-",O3)+1,10))-TIMEVALUE(LEFT(O3,FIND("-",O3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="P19" s="5">
-        <f>IF(P3="",0,IFERROR((TIMEVALUE(MID(P3,FIND("-",P3)+1,10))-TIMEVALUE(LEFT(P3,FIND("-",P3)-1)))*24,0))</f>
+        <f>IF(P3="",0,IFERROR((TIMEVALUE(MID(P3,FIND("-",P3)+1,10))-TIMEVALUE(LEFT(P3,FIND("-",P3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Q19" s="5">
@@ -3167,27 +3172,27 @@
         <v/>
       </c>
       <c r="R19" s="5">
-        <f>IF(R3="",0,IFERROR((TIMEVALUE(MID(R3,FIND("-",R3)+1,10))-TIMEVALUE(LEFT(R3,FIND("-",R3)-1)))*24,0))</f>
+        <f>IF(R3="",0,IFERROR((TIMEVALUE(MID(R3,FIND("-",R3)+1,10))-TIMEVALUE(LEFT(R3,FIND("-",R3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="S19" s="5">
-        <f>IF(S3="",0,IFERROR((TIMEVALUE(MID(S3,FIND("-",S3)+1,10))-TIMEVALUE(LEFT(S3,FIND("-",S3)-1)))*24,0))</f>
+        <f>IF(S3="",0,IFERROR((TIMEVALUE(MID(S3,FIND("-",S3)+1,10))-TIMEVALUE(LEFT(S3,FIND("-",S3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="T19" s="5">
-        <f>IF(T3="",0,IFERROR((TIMEVALUE(MID(T3,FIND("-",T3)+1,10))-TIMEVALUE(LEFT(T3,FIND("-",T3)-1)))*24,0))</f>
+        <f>IF(T3="",0,IFERROR((TIMEVALUE(MID(T3,FIND("-",T3)+1,10))-TIMEVALUE(LEFT(T3,FIND("-",T3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="U19" s="5">
-        <f>IF(U3="",0,IFERROR((TIMEVALUE(MID(U3,FIND("-",U3)+1,10))-TIMEVALUE(LEFT(U3,FIND("-",U3)-1)))*24,0))</f>
+        <f>IF(U3="",0,IFERROR((TIMEVALUE(MID(U3,FIND("-",U3)+1,10))-TIMEVALUE(LEFT(U3,FIND("-",U3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="V19" s="5">
-        <f>IF(V3="",0,IFERROR((TIMEVALUE(MID(V3,FIND("-",V3)+1,10))-TIMEVALUE(LEFT(V3,FIND("-",V3)-1)))*24,0))</f>
+        <f>IF(V3="",0,IFERROR((TIMEVALUE(MID(V3,FIND("-",V3)+1,10))-TIMEVALUE(LEFT(V3,FIND("-",V3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="W19" s="5">
-        <f>IF(W3="",0,IFERROR((TIMEVALUE(MID(W3,FIND("-",W3)+1,10))-TIMEVALUE(LEFT(W3,FIND("-",W3)-1)))*24,0))</f>
+        <f>IF(W3="",0,IFERROR((TIMEVALUE(MID(W3,FIND("-",W3)+1,10))-TIMEVALUE(LEFT(W3,FIND("-",W3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="X19" s="5">
@@ -3195,27 +3200,27 @@
         <v/>
       </c>
       <c r="Y19" s="5">
-        <f>IF(Y3="",0,IFERROR((TIMEVALUE(MID(Y3,FIND("-",Y3)+1,10))-TIMEVALUE(LEFT(Y3,FIND("-",Y3)-1)))*24,0))</f>
+        <f>IF(Y3="",0,IFERROR((TIMEVALUE(MID(Y3,FIND("-",Y3)+1,10))-TIMEVALUE(LEFT(Y3,FIND("-",Y3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Z19" s="5">
-        <f>IF(Z3="",0,IFERROR((TIMEVALUE(MID(Z3,FIND("-",Z3)+1,10))-TIMEVALUE(LEFT(Z3,FIND("-",Z3)-1)))*24,0))</f>
+        <f>IF(Z3="",0,IFERROR((TIMEVALUE(MID(Z3,FIND("-",Z3)+1,10))-TIMEVALUE(LEFT(Z3,FIND("-",Z3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AA19" s="5">
-        <f>IF(AA3="",0,IFERROR((TIMEVALUE(MID(AA3,FIND("-",AA3)+1,10))-TIMEVALUE(LEFT(AA3,FIND("-",AA3)-1)))*24,0))</f>
+        <f>IF(AA3="",0,IFERROR((TIMEVALUE(MID(AA3,FIND("-",AA3)+1,10))-TIMEVALUE(LEFT(AA3,FIND("-",AA3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AB19" s="5">
-        <f>IF(AB3="",0,IFERROR((TIMEVALUE(MID(AB3,FIND("-",AB3)+1,10))-TIMEVALUE(LEFT(AB3,FIND("-",AB3)-1)))*24,0))</f>
+        <f>IF(AB3="",0,IFERROR((TIMEVALUE(MID(AB3,FIND("-",AB3)+1,10))-TIMEVALUE(LEFT(AB3,FIND("-",AB3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AC19" s="5">
-        <f>IF(AC3="",0,IFERROR((TIMEVALUE(MID(AC3,FIND("-",AC3)+1,10))-TIMEVALUE(LEFT(AC3,FIND("-",AC3)-1)))*24,0))</f>
+        <f>IF(AC3="",0,IFERROR((TIMEVALUE(MID(AC3,FIND("-",AC3)+1,10))-TIMEVALUE(LEFT(AC3,FIND("-",AC3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AD19" s="5">
-        <f>IF(AD3="",0,IFERROR((TIMEVALUE(MID(AD3,FIND("-",AD3)+1,10))-TIMEVALUE(LEFT(AD3,FIND("-",AD3)-1)))*24,0))</f>
+        <f>IF(AD3="",0,IFERROR((TIMEVALUE(MID(AD3,FIND("-",AD3)+1,10))-TIMEVALUE(LEFT(AD3,FIND("-",AD3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AE19" s="5">
@@ -3223,11 +3228,11 @@
         <v/>
       </c>
       <c r="AF19" s="5">
-        <f>IF(AF3="",0,IFERROR((TIMEVALUE(MID(AF3,FIND("-",AF3)+1,10))-TIMEVALUE(LEFT(AF3,FIND("-",AF3)-1)))*24,0))</f>
+        <f>IF(AF3="",0,IFERROR((TIMEVALUE(MID(AF3,FIND("-",AF3)+1,10))-TIMEVALUE(LEFT(AF3,FIND("-",AF3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AG19" s="5">
-        <f>IF(AG3="",0,IFERROR((TIMEVALUE(MID(AG3,FIND("-",AG3)+1,10))-TIMEVALUE(LEFT(AG3,FIND("-",AG3)-1)))*24,0))</f>
+        <f>IF(AG3="",0,IFERROR((TIMEVALUE(MID(AG3,FIND("-",AG3)+1,10))-TIMEVALUE(LEFT(AG3,FIND("-",AG3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AH19" s="5">
@@ -3273,27 +3278,27 @@
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>IF(D4="",0,IFERROR((TIMEVALUE(MID(D4,FIND("-",D4)+1,10))-TIMEVALUE(LEFT(D4,FIND("-",D4)-1)))*24-1,0))</f>
+        <f>IF(D4="",0,IFERROR((TIMEVALUE(MID(D4,FIND("-",D4)+1,10))-TIMEVALUE(LEFT(D4,FIND("-",D4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>IF(E4="",0,IFERROR((TIMEVALUE(MID(E4,FIND("-",E4)+1,10))-TIMEVALUE(LEFT(E4,FIND("-",E4)-1)))*24-1,0))</f>
+        <f>IF(E4="",0,IFERROR((TIMEVALUE(MID(E4,FIND("-",E4)+1,10))-TIMEVALUE(LEFT(E4,FIND("-",E4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="F20" s="5">
-        <f>IF(F4="",0,IFERROR((TIMEVALUE(MID(F4,FIND("-",F4)+1,10))-TIMEVALUE(LEFT(F4,FIND("-",F4)-1)))*24-1,0))</f>
+        <f>IF(F4="",0,IFERROR((TIMEVALUE(MID(F4,FIND("-",F4)+1,10))-TIMEVALUE(LEFT(F4,FIND("-",F4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="G20" s="5">
-        <f>IF(G4="",0,IFERROR((TIMEVALUE(MID(G4,FIND("-",G4)+1,10))-TIMEVALUE(LEFT(G4,FIND("-",G4)-1)))*24-1,0))</f>
+        <f>IF(G4="",0,IFERROR((TIMEVALUE(MID(G4,FIND("-",G4)+1,10))-TIMEVALUE(LEFT(G4,FIND("-",G4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="H20" s="5">
-        <f>IF(H4="",0,IFERROR((TIMEVALUE(MID(H4,FIND("-",H4)+1,10))-TIMEVALUE(LEFT(H4,FIND("-",H4)-1)))*24-1,0))</f>
+        <f>IF(H4="",0,IFERROR((TIMEVALUE(MID(H4,FIND("-",H4)+1,10))-TIMEVALUE(LEFT(H4,FIND("-",H4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="I20" s="5">
-        <f>IF(I4="",0,IFERROR((TIMEVALUE(MID(I4,FIND("-",I4)+1,10))-TIMEVALUE(LEFT(I4,FIND("-",I4)-1)))*24-1,0))</f>
+        <f>IF(I4="",0,IFERROR((TIMEVALUE(MID(I4,FIND("-",I4)+1,10))-TIMEVALUE(LEFT(I4,FIND("-",I4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="J20" s="5">
@@ -3301,27 +3306,27 @@
         <v/>
       </c>
       <c r="K20" s="5">
-        <f>IF(K4="",0,IFERROR((TIMEVALUE(MID(K4,FIND("-",K4)+1,10))-TIMEVALUE(LEFT(K4,FIND("-",K4)-1)))*24-1,0))</f>
+        <f>IF(K4="",0,IFERROR((TIMEVALUE(MID(K4,FIND("-",K4)+1,10))-TIMEVALUE(LEFT(K4,FIND("-",K4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="L20" s="5">
-        <f>IF(L4="",0,IFERROR((TIMEVALUE(MID(L4,FIND("-",L4)+1,10))-TIMEVALUE(LEFT(L4,FIND("-",L4)-1)))*24-1,0))</f>
+        <f>IF(L4="",0,IFERROR((TIMEVALUE(MID(L4,FIND("-",L4)+1,10))-TIMEVALUE(LEFT(L4,FIND("-",L4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="M20" s="5">
-        <f>IF(M4="",0,IFERROR((TIMEVALUE(MID(M4,FIND("-",M4)+1,10))-TIMEVALUE(LEFT(M4,FIND("-",M4)-1)))*24-1,0))</f>
+        <f>IF(M4="",0,IFERROR((TIMEVALUE(MID(M4,FIND("-",M4)+1,10))-TIMEVALUE(LEFT(M4,FIND("-",M4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="N20" s="5">
-        <f>IF(N4="",0,IFERROR((TIMEVALUE(MID(N4,FIND("-",N4)+1,10))-TIMEVALUE(LEFT(N4,FIND("-",N4)-1)))*24-1,0))</f>
+        <f>IF(N4="",0,IFERROR((TIMEVALUE(MID(N4,FIND("-",N4)+1,10))-TIMEVALUE(LEFT(N4,FIND("-",N4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="O20" s="5">
-        <f>IF(O4="",0,IFERROR((TIMEVALUE(MID(O4,FIND("-",O4)+1,10))-TIMEVALUE(LEFT(O4,FIND("-",O4)-1)))*24-1,0))</f>
+        <f>IF(O4="",0,IFERROR((TIMEVALUE(MID(O4,FIND("-",O4)+1,10))-TIMEVALUE(LEFT(O4,FIND("-",O4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="P20" s="5">
-        <f>IF(P4="",0,IFERROR((TIMEVALUE(MID(P4,FIND("-",P4)+1,10))-TIMEVALUE(LEFT(P4,FIND("-",P4)-1)))*24-1,0))</f>
+        <f>IF(P4="",0,IFERROR((TIMEVALUE(MID(P4,FIND("-",P4)+1,10))-TIMEVALUE(LEFT(P4,FIND("-",P4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Q20" s="5">
@@ -3329,27 +3334,27 @@
         <v/>
       </c>
       <c r="R20" s="5">
-        <f>IF(R4="",0,IFERROR((TIMEVALUE(MID(R4,FIND("-",R4)+1,10))-TIMEVALUE(LEFT(R4,FIND("-",R4)-1)))*24-1,0))</f>
+        <f>IF(R4="",0,IFERROR((TIMEVALUE(MID(R4,FIND("-",R4)+1,10))-TIMEVALUE(LEFT(R4,FIND("-",R4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="S20" s="5">
-        <f>IF(S4="",0,IFERROR((TIMEVALUE(MID(S4,FIND("-",S4)+1,10))-TIMEVALUE(LEFT(S4,FIND("-",S4)-1)))*24-1,0))</f>
+        <f>IF(S4="",0,IFERROR((TIMEVALUE(MID(S4,FIND("-",S4)+1,10))-TIMEVALUE(LEFT(S4,FIND("-",S4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="T20" s="5">
-        <f>IF(T4="",0,IFERROR((TIMEVALUE(MID(T4,FIND("-",T4)+1,10))-TIMEVALUE(LEFT(T4,FIND("-",T4)-1)))*24-1,0))</f>
+        <f>IF(T4="",0,IFERROR((TIMEVALUE(MID(T4,FIND("-",T4)+1,10))-TIMEVALUE(LEFT(T4,FIND("-",T4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="U20" s="5">
-        <f>IF(U4="",0,IFERROR((TIMEVALUE(MID(U4,FIND("-",U4)+1,10))-TIMEVALUE(LEFT(U4,FIND("-",U4)-1)))*24-1,0))</f>
+        <f>IF(U4="",0,IFERROR((TIMEVALUE(MID(U4,FIND("-",U4)+1,10))-TIMEVALUE(LEFT(U4,FIND("-",U4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="V20" s="5">
-        <f>IF(V4="",0,IFERROR((TIMEVALUE(MID(V4,FIND("-",V4)+1,10))-TIMEVALUE(LEFT(V4,FIND("-",V4)-1)))*24-1,0))</f>
+        <f>IF(V4="",0,IFERROR((TIMEVALUE(MID(V4,FIND("-",V4)+1,10))-TIMEVALUE(LEFT(V4,FIND("-",V4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="W20" s="5">
-        <f>IF(W4="",0,IFERROR((TIMEVALUE(MID(W4,FIND("-",W4)+1,10))-TIMEVALUE(LEFT(W4,FIND("-",W4)-1)))*24-1,0))</f>
+        <f>IF(W4="",0,IFERROR((TIMEVALUE(MID(W4,FIND("-",W4)+1,10))-TIMEVALUE(LEFT(W4,FIND("-",W4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="X20" s="5">
@@ -3357,27 +3362,27 @@
         <v/>
       </c>
       <c r="Y20" s="5">
-        <f>IF(Y4="",0,IFERROR((TIMEVALUE(MID(Y4,FIND("-",Y4)+1,10))-TIMEVALUE(LEFT(Y4,FIND("-",Y4)-1)))*24-1,0))</f>
+        <f>IF(Y4="",0,IFERROR((TIMEVALUE(MID(Y4,FIND("-",Y4)+1,10))-TIMEVALUE(LEFT(Y4,FIND("-",Y4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Z20" s="5">
-        <f>IF(Z4="",0,IFERROR((TIMEVALUE(MID(Z4,FIND("-",Z4)+1,10))-TIMEVALUE(LEFT(Z4,FIND("-",Z4)-1)))*24-1,0))</f>
+        <f>IF(Z4="",0,IFERROR((TIMEVALUE(MID(Z4,FIND("-",Z4)+1,10))-TIMEVALUE(LEFT(Z4,FIND("-",Z4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AA20" s="5">
-        <f>IF(AA4="",0,IFERROR((TIMEVALUE(MID(AA4,FIND("-",AA4)+1,10))-TIMEVALUE(LEFT(AA4,FIND("-",AA4)-1)))*24-1,0))</f>
+        <f>IF(AA4="",0,IFERROR((TIMEVALUE(MID(AA4,FIND("-",AA4)+1,10))-TIMEVALUE(LEFT(AA4,FIND("-",AA4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AB20" s="5">
-        <f>IF(AB4="",0,IFERROR((TIMEVALUE(MID(AB4,FIND("-",AB4)+1,10))-TIMEVALUE(LEFT(AB4,FIND("-",AB4)-1)))*24-1,0))</f>
+        <f>IF(AB4="",0,IFERROR((TIMEVALUE(MID(AB4,FIND("-",AB4)+1,10))-TIMEVALUE(LEFT(AB4,FIND("-",AB4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AC20" s="5">
-        <f>IF(AC4="",0,IFERROR((TIMEVALUE(MID(AC4,FIND("-",AC4)+1,10))-TIMEVALUE(LEFT(AC4,FIND("-",AC4)-1)))*24-1,0))</f>
+        <f>IF(AC4="",0,IFERROR((TIMEVALUE(MID(AC4,FIND("-",AC4)+1,10))-TIMEVALUE(LEFT(AC4,FIND("-",AC4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AD20" s="5">
-        <f>IF(AD4="",0,IFERROR((TIMEVALUE(MID(AD4,FIND("-",AD4)+1,10))-TIMEVALUE(LEFT(AD4,FIND("-",AD4)-1)))*24-1,0))</f>
+        <f>IF(AD4="",0,IFERROR((TIMEVALUE(MID(AD4,FIND("-",AD4)+1,10))-TIMEVALUE(LEFT(AD4,FIND("-",AD4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AE20" s="5">
@@ -3385,11 +3390,11 @@
         <v/>
       </c>
       <c r="AF20" s="5">
-        <f>IF(AF4="",0,IFERROR((TIMEVALUE(MID(AF4,FIND("-",AF4)+1,10))-TIMEVALUE(LEFT(AF4,FIND("-",AF4)-1)))*24-1,0))</f>
+        <f>IF(AF4="",0,IFERROR((TIMEVALUE(MID(AF4,FIND("-",AF4)+1,10))-TIMEVALUE(LEFT(AF4,FIND("-",AF4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AG20" s="5">
-        <f>IF(AG4="",0,IFERROR((TIMEVALUE(MID(AG4,FIND("-",AG4)+1,10))-TIMEVALUE(LEFT(AG4,FIND("-",AG4)-1)))*24-1,0))</f>
+        <f>IF(AG4="",0,IFERROR((TIMEVALUE(MID(AG4,FIND("-",AG4)+1,10))-TIMEVALUE(LEFT(AG4,FIND("-",AG4)-1)))*24-IF(ISNUMBER(FIND("-",$C4)),IFERROR((TIMEVALUE(MID($C4,FIND("-",$C4)+1,10))-TIMEVALUE(LEFT($C4,FIND("-",$C4)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AH20" s="5">
@@ -3435,27 +3440,27 @@
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>IF(D5="",0,IFERROR((TIMEVALUE(MID(D5,FIND("-",D5)+1,10))-TIMEVALUE(LEFT(D5,FIND("-",D5)-1)))*24-1,0))</f>
+        <f>IF(D5="",0,IFERROR((TIMEVALUE(MID(D5,FIND("-",D5)+1,10))-TIMEVALUE(LEFT(D5,FIND("-",D5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>IF(E5="",0,IFERROR((TIMEVALUE(MID(E5,FIND("-",E5)+1,10))-TIMEVALUE(LEFT(E5,FIND("-",E5)-1)))*24-1,0))</f>
+        <f>IF(E5="",0,IFERROR((TIMEVALUE(MID(E5,FIND("-",E5)+1,10))-TIMEVALUE(LEFT(E5,FIND("-",E5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="F21" s="5">
-        <f>IF(F5="",0,IFERROR((TIMEVALUE(MID(F5,FIND("-",F5)+1,10))-TIMEVALUE(LEFT(F5,FIND("-",F5)-1)))*24-1,0))</f>
+        <f>IF(F5="",0,IFERROR((TIMEVALUE(MID(F5,FIND("-",F5)+1,10))-TIMEVALUE(LEFT(F5,FIND("-",F5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="G21" s="5">
-        <f>IF(G5="",0,IFERROR((TIMEVALUE(MID(G5,FIND("-",G5)+1,10))-TIMEVALUE(LEFT(G5,FIND("-",G5)-1)))*24-1,0))</f>
+        <f>IF(G5="",0,IFERROR((TIMEVALUE(MID(G5,FIND("-",G5)+1,10))-TIMEVALUE(LEFT(G5,FIND("-",G5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="H21" s="5">
-        <f>IF(H5="",0,IFERROR((TIMEVALUE(MID(H5,FIND("-",H5)+1,10))-TIMEVALUE(LEFT(H5,FIND("-",H5)-1)))*24-1,0))</f>
+        <f>IF(H5="",0,IFERROR((TIMEVALUE(MID(H5,FIND("-",H5)+1,10))-TIMEVALUE(LEFT(H5,FIND("-",H5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="I21" s="5">
-        <f>IF(I5="",0,IFERROR((TIMEVALUE(MID(I5,FIND("-",I5)+1,10))-TIMEVALUE(LEFT(I5,FIND("-",I5)-1)))*24-1,0))</f>
+        <f>IF(I5="",0,IFERROR((TIMEVALUE(MID(I5,FIND("-",I5)+1,10))-TIMEVALUE(LEFT(I5,FIND("-",I5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="J21" s="5">
@@ -3463,27 +3468,27 @@
         <v/>
       </c>
       <c r="K21" s="5">
-        <f>IF(K5="",0,IFERROR((TIMEVALUE(MID(K5,FIND("-",K5)+1,10))-TIMEVALUE(LEFT(K5,FIND("-",K5)-1)))*24-1,0))</f>
+        <f>IF(K5="",0,IFERROR((TIMEVALUE(MID(K5,FIND("-",K5)+1,10))-TIMEVALUE(LEFT(K5,FIND("-",K5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="L21" s="5">
-        <f>IF(L5="",0,IFERROR((TIMEVALUE(MID(L5,FIND("-",L5)+1,10))-TIMEVALUE(LEFT(L5,FIND("-",L5)-1)))*24-1,0))</f>
+        <f>IF(L5="",0,IFERROR((TIMEVALUE(MID(L5,FIND("-",L5)+1,10))-TIMEVALUE(LEFT(L5,FIND("-",L5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="M21" s="5">
-        <f>IF(M5="",0,IFERROR((TIMEVALUE(MID(M5,FIND("-",M5)+1,10))-TIMEVALUE(LEFT(M5,FIND("-",M5)-1)))*24-1,0))</f>
+        <f>IF(M5="",0,IFERROR((TIMEVALUE(MID(M5,FIND("-",M5)+1,10))-TIMEVALUE(LEFT(M5,FIND("-",M5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="N21" s="5">
-        <f>IF(N5="",0,IFERROR((TIMEVALUE(MID(N5,FIND("-",N5)+1,10))-TIMEVALUE(LEFT(N5,FIND("-",N5)-1)))*24-1,0))</f>
+        <f>IF(N5="",0,IFERROR((TIMEVALUE(MID(N5,FIND("-",N5)+1,10))-TIMEVALUE(LEFT(N5,FIND("-",N5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="O21" s="5">
-        <f>IF(O5="",0,IFERROR((TIMEVALUE(MID(O5,FIND("-",O5)+1,10))-TIMEVALUE(LEFT(O5,FIND("-",O5)-1)))*24-1,0))</f>
+        <f>IF(O5="",0,IFERROR((TIMEVALUE(MID(O5,FIND("-",O5)+1,10))-TIMEVALUE(LEFT(O5,FIND("-",O5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="P21" s="5">
-        <f>IF(P5="",0,IFERROR((TIMEVALUE(MID(P5,FIND("-",P5)+1,10))-TIMEVALUE(LEFT(P5,FIND("-",P5)-1)))*24-1,0))</f>
+        <f>IF(P5="",0,IFERROR((TIMEVALUE(MID(P5,FIND("-",P5)+1,10))-TIMEVALUE(LEFT(P5,FIND("-",P5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Q21" s="5">
@@ -3491,27 +3496,27 @@
         <v/>
       </c>
       <c r="R21" s="5">
-        <f>IF(R5="",0,IFERROR((TIMEVALUE(MID(R5,FIND("-",R5)+1,10))-TIMEVALUE(LEFT(R5,FIND("-",R5)-1)))*24-1,0))</f>
+        <f>IF(R5="",0,IFERROR((TIMEVALUE(MID(R5,FIND("-",R5)+1,10))-TIMEVALUE(LEFT(R5,FIND("-",R5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="S21" s="5">
-        <f>IF(S5="",0,IFERROR((TIMEVALUE(MID(S5,FIND("-",S5)+1,10))-TIMEVALUE(LEFT(S5,FIND("-",S5)-1)))*24-1,0))</f>
+        <f>IF(S5="",0,IFERROR((TIMEVALUE(MID(S5,FIND("-",S5)+1,10))-TIMEVALUE(LEFT(S5,FIND("-",S5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="T21" s="5">
-        <f>IF(T5="",0,IFERROR((TIMEVALUE(MID(T5,FIND("-",T5)+1,10))-TIMEVALUE(LEFT(T5,FIND("-",T5)-1)))*24-1,0))</f>
+        <f>IF(T5="",0,IFERROR((TIMEVALUE(MID(T5,FIND("-",T5)+1,10))-TIMEVALUE(LEFT(T5,FIND("-",T5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="U21" s="5">
-        <f>IF(U5="",0,IFERROR((TIMEVALUE(MID(U5,FIND("-",U5)+1,10))-TIMEVALUE(LEFT(U5,FIND("-",U5)-1)))*24-1,0))</f>
+        <f>IF(U5="",0,IFERROR((TIMEVALUE(MID(U5,FIND("-",U5)+1,10))-TIMEVALUE(LEFT(U5,FIND("-",U5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="V21" s="5">
-        <f>IF(V5="",0,IFERROR((TIMEVALUE(MID(V5,FIND("-",V5)+1,10))-TIMEVALUE(LEFT(V5,FIND("-",V5)-1)))*24-1,0))</f>
+        <f>IF(V5="",0,IFERROR((TIMEVALUE(MID(V5,FIND("-",V5)+1,10))-TIMEVALUE(LEFT(V5,FIND("-",V5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="W21" s="5">
-        <f>IF(W5="",0,IFERROR((TIMEVALUE(MID(W5,FIND("-",W5)+1,10))-TIMEVALUE(LEFT(W5,FIND("-",W5)-1)))*24-1,0))</f>
+        <f>IF(W5="",0,IFERROR((TIMEVALUE(MID(W5,FIND("-",W5)+1,10))-TIMEVALUE(LEFT(W5,FIND("-",W5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="X21" s="5">
@@ -3519,27 +3524,27 @@
         <v/>
       </c>
       <c r="Y21" s="5">
-        <f>IF(Y5="",0,IFERROR((TIMEVALUE(MID(Y5,FIND("-",Y5)+1,10))-TIMEVALUE(LEFT(Y5,FIND("-",Y5)-1)))*24-1,0))</f>
+        <f>IF(Y5="",0,IFERROR((TIMEVALUE(MID(Y5,FIND("-",Y5)+1,10))-TIMEVALUE(LEFT(Y5,FIND("-",Y5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Z21" s="5">
-        <f>IF(Z5="",0,IFERROR((TIMEVALUE(MID(Z5,FIND("-",Z5)+1,10))-TIMEVALUE(LEFT(Z5,FIND("-",Z5)-1)))*24-1,0))</f>
+        <f>IF(Z5="",0,IFERROR((TIMEVALUE(MID(Z5,FIND("-",Z5)+1,10))-TIMEVALUE(LEFT(Z5,FIND("-",Z5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AA21" s="5">
-        <f>IF(AA5="",0,IFERROR((TIMEVALUE(MID(AA5,FIND("-",AA5)+1,10))-TIMEVALUE(LEFT(AA5,FIND("-",AA5)-1)))*24-1,0))</f>
+        <f>IF(AA5="",0,IFERROR((TIMEVALUE(MID(AA5,FIND("-",AA5)+1,10))-TIMEVALUE(LEFT(AA5,FIND("-",AA5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AB21" s="5">
-        <f>IF(AB5="",0,IFERROR((TIMEVALUE(MID(AB5,FIND("-",AB5)+1,10))-TIMEVALUE(LEFT(AB5,FIND("-",AB5)-1)))*24-1,0))</f>
+        <f>IF(AB5="",0,IFERROR((TIMEVALUE(MID(AB5,FIND("-",AB5)+1,10))-TIMEVALUE(LEFT(AB5,FIND("-",AB5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AC21" s="5">
-        <f>IF(AC5="",0,IFERROR((TIMEVALUE(MID(AC5,FIND("-",AC5)+1,10))-TIMEVALUE(LEFT(AC5,FIND("-",AC5)-1)))*24-1,0))</f>
+        <f>IF(AC5="",0,IFERROR((TIMEVALUE(MID(AC5,FIND("-",AC5)+1,10))-TIMEVALUE(LEFT(AC5,FIND("-",AC5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AD21" s="5">
-        <f>IF(AD5="",0,IFERROR((TIMEVALUE(MID(AD5,FIND("-",AD5)+1,10))-TIMEVALUE(LEFT(AD5,FIND("-",AD5)-1)))*24-1,0))</f>
+        <f>IF(AD5="",0,IFERROR((TIMEVALUE(MID(AD5,FIND("-",AD5)+1,10))-TIMEVALUE(LEFT(AD5,FIND("-",AD5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AE21" s="5">
@@ -3547,11 +3552,11 @@
         <v/>
       </c>
       <c r="AF21" s="5">
-        <f>IF(AF5="",0,IFERROR((TIMEVALUE(MID(AF5,FIND("-",AF5)+1,10))-TIMEVALUE(LEFT(AF5,FIND("-",AF5)-1)))*24-1,0))</f>
+        <f>IF(AF5="",0,IFERROR((TIMEVALUE(MID(AF5,FIND("-",AF5)+1,10))-TIMEVALUE(LEFT(AF5,FIND("-",AF5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AG21" s="5">
-        <f>IF(AG5="",0,IFERROR((TIMEVALUE(MID(AG5,FIND("-",AG5)+1,10))-TIMEVALUE(LEFT(AG5,FIND("-",AG5)-1)))*24-1,0))</f>
+        <f>IF(AG5="",0,IFERROR((TIMEVALUE(MID(AG5,FIND("-",AG5)+1,10))-TIMEVALUE(LEFT(AG5,FIND("-",AG5)-1)))*24-IF(ISNUMBER(FIND("-",$C5)),IFERROR((TIMEVALUE(MID($C5,FIND("-",$C5)+1,10))-TIMEVALUE(LEFT($C5,FIND("-",$C5)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AH21" s="5">
@@ -3598,27 +3603,27 @@
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>IF(D6="",0,IFERROR((TIMEVALUE(MID(D6,FIND("-",D6)+1,10))-TIMEVALUE(LEFT(D6,FIND("-",D6)-1)))*24-1,0))</f>
+        <f>IF(D6="",0,IFERROR((TIMEVALUE(MID(D6,FIND("-",D6)+1,10))-TIMEVALUE(LEFT(D6,FIND("-",D6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>IF(E6="",0,IFERROR((TIMEVALUE(MID(E6,FIND("-",E6)+1,10))-TIMEVALUE(LEFT(E6,FIND("-",E6)-1)))*24-1,0))</f>
+        <f>IF(E6="",0,IFERROR((TIMEVALUE(MID(E6,FIND("-",E6)+1,10))-TIMEVALUE(LEFT(E6,FIND("-",E6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="F22" s="5">
-        <f>IF(F6="",0,IFERROR((TIMEVALUE(MID(F6,FIND("-",F6)+1,10))-TIMEVALUE(LEFT(F6,FIND("-",F6)-1)))*24-1,0))</f>
+        <f>IF(F6="",0,IFERROR((TIMEVALUE(MID(F6,FIND("-",F6)+1,10))-TIMEVALUE(LEFT(F6,FIND("-",F6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="G22" s="5">
-        <f>IF(G6="",0,IFERROR((TIMEVALUE(MID(G6,FIND("-",G6)+1,10))-TIMEVALUE(LEFT(G6,FIND("-",G6)-1)))*24-1,0))</f>
+        <f>IF(G6="",0,IFERROR((TIMEVALUE(MID(G6,FIND("-",G6)+1,10))-TIMEVALUE(LEFT(G6,FIND("-",G6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="H22" s="5">
-        <f>IF(H6="",0,IFERROR((TIMEVALUE(MID(H6,FIND("-",H6)+1,10))-TIMEVALUE(LEFT(H6,FIND("-",H6)-1)))*24-1,0))</f>
+        <f>IF(H6="",0,IFERROR((TIMEVALUE(MID(H6,FIND("-",H6)+1,10))-TIMEVALUE(LEFT(H6,FIND("-",H6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="I22" s="5">
-        <f>IF(I6="",0,IFERROR((TIMEVALUE(MID(I6,FIND("-",I6)+1,10))-TIMEVALUE(LEFT(I6,FIND("-",I6)-1)))*24-1,0))</f>
+        <f>IF(I6="",0,IFERROR((TIMEVALUE(MID(I6,FIND("-",I6)+1,10))-TIMEVALUE(LEFT(I6,FIND("-",I6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="J22" s="5">
@@ -3626,27 +3631,27 @@
         <v/>
       </c>
       <c r="K22" s="5">
-        <f>IF(K6="",0,IFERROR((TIMEVALUE(MID(K6,FIND("-",K6)+1,10))-TIMEVALUE(LEFT(K6,FIND("-",K6)-1)))*24-1,0))</f>
+        <f>IF(K6="",0,IFERROR((TIMEVALUE(MID(K6,FIND("-",K6)+1,10))-TIMEVALUE(LEFT(K6,FIND("-",K6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="L22" s="5">
-        <f>IF(L6="",0,IFERROR((TIMEVALUE(MID(L6,FIND("-",L6)+1,10))-TIMEVALUE(LEFT(L6,FIND("-",L6)-1)))*24-1,0))</f>
+        <f>IF(L6="",0,IFERROR((TIMEVALUE(MID(L6,FIND("-",L6)+1,10))-TIMEVALUE(LEFT(L6,FIND("-",L6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="M22" s="5">
-        <f>IF(M6="",0,IFERROR((TIMEVALUE(MID(M6,FIND("-",M6)+1,10))-TIMEVALUE(LEFT(M6,FIND("-",M6)-1)))*24-1,0))</f>
+        <f>IF(M6="",0,IFERROR((TIMEVALUE(MID(M6,FIND("-",M6)+1,10))-TIMEVALUE(LEFT(M6,FIND("-",M6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="N22" s="5">
-        <f>IF(N6="",0,IFERROR((TIMEVALUE(MID(N6,FIND("-",N6)+1,10))-TIMEVALUE(LEFT(N6,FIND("-",N6)-1)))*24-1,0))</f>
+        <f>IF(N6="",0,IFERROR((TIMEVALUE(MID(N6,FIND("-",N6)+1,10))-TIMEVALUE(LEFT(N6,FIND("-",N6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="O22" s="5">
-        <f>IF(O6="",0,IFERROR((TIMEVALUE(MID(O6,FIND("-",O6)+1,10))-TIMEVALUE(LEFT(O6,FIND("-",O6)-1)))*24-1,0))</f>
+        <f>IF(O6="",0,IFERROR((TIMEVALUE(MID(O6,FIND("-",O6)+1,10))-TIMEVALUE(LEFT(O6,FIND("-",O6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="P22" s="5">
-        <f>IF(P6="",0,IFERROR((TIMEVALUE(MID(P6,FIND("-",P6)+1,10))-TIMEVALUE(LEFT(P6,FIND("-",P6)-1)))*24-1,0))</f>
+        <f>IF(P6="",0,IFERROR((TIMEVALUE(MID(P6,FIND("-",P6)+1,10))-TIMEVALUE(LEFT(P6,FIND("-",P6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Q22" s="5">
@@ -3654,27 +3659,27 @@
         <v/>
       </c>
       <c r="R22" s="5">
-        <f>IF(R6="",0,IFERROR((TIMEVALUE(MID(R6,FIND("-",R6)+1,10))-TIMEVALUE(LEFT(R6,FIND("-",R6)-1)))*24-1,0))</f>
+        <f>IF(R6="",0,IFERROR((TIMEVALUE(MID(R6,FIND("-",R6)+1,10))-TIMEVALUE(LEFT(R6,FIND("-",R6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="S22" s="5">
-        <f>IF(S6="",0,IFERROR((TIMEVALUE(MID(S6,FIND("-",S6)+1,10))-TIMEVALUE(LEFT(S6,FIND("-",S6)-1)))*24-1,0))</f>
+        <f>IF(S6="",0,IFERROR((TIMEVALUE(MID(S6,FIND("-",S6)+1,10))-TIMEVALUE(LEFT(S6,FIND("-",S6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="T22" s="5">
-        <f>IF(T6="",0,IFERROR((TIMEVALUE(MID(T6,FIND("-",T6)+1,10))-TIMEVALUE(LEFT(T6,FIND("-",T6)-1)))*24-1,0))</f>
+        <f>IF(T6="",0,IFERROR((TIMEVALUE(MID(T6,FIND("-",T6)+1,10))-TIMEVALUE(LEFT(T6,FIND("-",T6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="U22" s="5">
-        <f>IF(U6="",0,IFERROR((TIMEVALUE(MID(U6,FIND("-",U6)+1,10))-TIMEVALUE(LEFT(U6,FIND("-",U6)-1)))*24-1,0))</f>
+        <f>IF(U6="",0,IFERROR((TIMEVALUE(MID(U6,FIND("-",U6)+1,10))-TIMEVALUE(LEFT(U6,FIND("-",U6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="V22" s="5">
-        <f>IF(V6="",0,IFERROR((TIMEVALUE(MID(V6,FIND("-",V6)+1,10))-TIMEVALUE(LEFT(V6,FIND("-",V6)-1)))*24-1,0))</f>
+        <f>IF(V6="",0,IFERROR((TIMEVALUE(MID(V6,FIND("-",V6)+1,10))-TIMEVALUE(LEFT(V6,FIND("-",V6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="W22" s="5">
-        <f>IF(W6="",0,IFERROR((TIMEVALUE(MID(W6,FIND("-",W6)+1,10))-TIMEVALUE(LEFT(W6,FIND("-",W6)-1)))*24-1,0))</f>
+        <f>IF(W6="",0,IFERROR((TIMEVALUE(MID(W6,FIND("-",W6)+1,10))-TIMEVALUE(LEFT(W6,FIND("-",W6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="X22" s="5">
@@ -3682,27 +3687,27 @@
         <v/>
       </c>
       <c r="Y22" s="5">
-        <f>IF(Y6="",0,IFERROR((TIMEVALUE(MID(Y6,FIND("-",Y6)+1,10))-TIMEVALUE(LEFT(Y6,FIND("-",Y6)-1)))*24-1,0))</f>
+        <f>IF(Y6="",0,IFERROR((TIMEVALUE(MID(Y6,FIND("-",Y6)+1,10))-TIMEVALUE(LEFT(Y6,FIND("-",Y6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Z22" s="5">
-        <f>IF(Z6="",0,IFERROR((TIMEVALUE(MID(Z6,FIND("-",Z6)+1,10))-TIMEVALUE(LEFT(Z6,FIND("-",Z6)-1)))*24-1,0))</f>
+        <f>IF(Z6="",0,IFERROR((TIMEVALUE(MID(Z6,FIND("-",Z6)+1,10))-TIMEVALUE(LEFT(Z6,FIND("-",Z6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AA22" s="5">
-        <f>IF(AA6="",0,IFERROR((TIMEVALUE(MID(AA6,FIND("-",AA6)+1,10))-TIMEVALUE(LEFT(AA6,FIND("-",AA6)-1)))*24-1,0))</f>
+        <f>IF(AA6="",0,IFERROR((TIMEVALUE(MID(AA6,FIND("-",AA6)+1,10))-TIMEVALUE(LEFT(AA6,FIND("-",AA6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AB22" s="5">
-        <f>IF(AB6="",0,IFERROR((TIMEVALUE(MID(AB6,FIND("-",AB6)+1,10))-TIMEVALUE(LEFT(AB6,FIND("-",AB6)-1)))*24-1,0))</f>
+        <f>IF(AB6="",0,IFERROR((TIMEVALUE(MID(AB6,FIND("-",AB6)+1,10))-TIMEVALUE(LEFT(AB6,FIND("-",AB6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AC22" s="5">
-        <f>IF(AC6="",0,IFERROR((TIMEVALUE(MID(AC6,FIND("-",AC6)+1,10))-TIMEVALUE(LEFT(AC6,FIND("-",AC6)-1)))*24-1,0))</f>
+        <f>IF(AC6="",0,IFERROR((TIMEVALUE(MID(AC6,FIND("-",AC6)+1,10))-TIMEVALUE(LEFT(AC6,FIND("-",AC6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AD22" s="5">
-        <f>IF(AD6="",0,IFERROR((TIMEVALUE(MID(AD6,FIND("-",AD6)+1,10))-TIMEVALUE(LEFT(AD6,FIND("-",AD6)-1)))*24-1,0))</f>
+        <f>IF(AD6="",0,IFERROR((TIMEVALUE(MID(AD6,FIND("-",AD6)+1,10))-TIMEVALUE(LEFT(AD6,FIND("-",AD6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AE22" s="5">
@@ -3710,11 +3715,11 @@
         <v/>
       </c>
       <c r="AF22" s="5">
-        <f>IF(AF6="",0,IFERROR((TIMEVALUE(MID(AF6,FIND("-",AF6)+1,10))-TIMEVALUE(LEFT(AF6,FIND("-",AF6)-1)))*24-1,0))</f>
+        <f>IF(AF6="",0,IFERROR((TIMEVALUE(MID(AF6,FIND("-",AF6)+1,10))-TIMEVALUE(LEFT(AF6,FIND("-",AF6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AG22" s="5">
-        <f>IF(AG6="",0,IFERROR((TIMEVALUE(MID(AG6,FIND("-",AG6)+1,10))-TIMEVALUE(LEFT(AG6,FIND("-",AG6)-1)))*24-1,0))</f>
+        <f>IF(AG6="",0,IFERROR((TIMEVALUE(MID(AG6,FIND("-",AG6)+1,10))-TIMEVALUE(LEFT(AG6,FIND("-",AG6)-1)))*24-IF(ISNUMBER(FIND("-",$C6)),IFERROR((TIMEVALUE(MID($C6,FIND("-",$C6)+1,10))-TIMEVALUE(LEFT($C6,FIND("-",$C6)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AH22" s="5">
@@ -3761,27 +3766,27 @@
         <v/>
       </c>
       <c r="D23" s="5">
-        <f>IF(D7="",0,IFERROR((TIMEVALUE(MID(D7,FIND("-",D7)+1,10))-TIMEVALUE(LEFT(D7,FIND("-",D7)-1)))*24-1,0))</f>
+        <f>IF(D7="",0,IFERROR((TIMEVALUE(MID(D7,FIND("-",D7)+1,10))-TIMEVALUE(LEFT(D7,FIND("-",D7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="E23" s="5">
-        <f>IF(E7="",0,IFERROR((TIMEVALUE(MID(E7,FIND("-",E7)+1,10))-TIMEVALUE(LEFT(E7,FIND("-",E7)-1)))*24-1,0))</f>
+        <f>IF(E7="",0,IFERROR((TIMEVALUE(MID(E7,FIND("-",E7)+1,10))-TIMEVALUE(LEFT(E7,FIND("-",E7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="F23" s="5">
-        <f>IF(F7="",0,IFERROR((TIMEVALUE(MID(F7,FIND("-",F7)+1,10))-TIMEVALUE(LEFT(F7,FIND("-",F7)-1)))*24-1,0))</f>
+        <f>IF(F7="",0,IFERROR((TIMEVALUE(MID(F7,FIND("-",F7)+1,10))-TIMEVALUE(LEFT(F7,FIND("-",F7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="G23" s="5">
-        <f>IF(G7="",0,IFERROR((TIMEVALUE(MID(G7,FIND("-",G7)+1,10))-TIMEVALUE(LEFT(G7,FIND("-",G7)-1)))*24-1,0))</f>
+        <f>IF(G7="",0,IFERROR((TIMEVALUE(MID(G7,FIND("-",G7)+1,10))-TIMEVALUE(LEFT(G7,FIND("-",G7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="H23" s="5">
-        <f>IF(H7="",0,IFERROR((TIMEVALUE(MID(H7,FIND("-",H7)+1,10))-TIMEVALUE(LEFT(H7,FIND("-",H7)-1)))*24-1,0))</f>
+        <f>IF(H7="",0,IFERROR((TIMEVALUE(MID(H7,FIND("-",H7)+1,10))-TIMEVALUE(LEFT(H7,FIND("-",H7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="I23" s="5">
-        <f>IF(I7="",0,IFERROR((TIMEVALUE(MID(I7,FIND("-",I7)+1,10))-TIMEVALUE(LEFT(I7,FIND("-",I7)-1)))*24-1,0))</f>
+        <f>IF(I7="",0,IFERROR((TIMEVALUE(MID(I7,FIND("-",I7)+1,10))-TIMEVALUE(LEFT(I7,FIND("-",I7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="J23" s="5">
@@ -3789,27 +3794,27 @@
         <v/>
       </c>
       <c r="K23" s="5">
-        <f>IF(K7="",0,IFERROR((TIMEVALUE(MID(K7,FIND("-",K7)+1,10))-TIMEVALUE(LEFT(K7,FIND("-",K7)-1)))*24-1,0))</f>
+        <f>IF(K7="",0,IFERROR((TIMEVALUE(MID(K7,FIND("-",K7)+1,10))-TIMEVALUE(LEFT(K7,FIND("-",K7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="L23" s="5">
-        <f>IF(L7="",0,IFERROR((TIMEVALUE(MID(L7,FIND("-",L7)+1,10))-TIMEVALUE(LEFT(L7,FIND("-",L7)-1)))*24-1,0))</f>
+        <f>IF(L7="",0,IFERROR((TIMEVALUE(MID(L7,FIND("-",L7)+1,10))-TIMEVALUE(LEFT(L7,FIND("-",L7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="M23" s="5">
-        <f>IF(M7="",0,IFERROR((TIMEVALUE(MID(M7,FIND("-",M7)+1,10))-TIMEVALUE(LEFT(M7,FIND("-",M7)-1)))*24-1,0))</f>
+        <f>IF(M7="",0,IFERROR((TIMEVALUE(MID(M7,FIND("-",M7)+1,10))-TIMEVALUE(LEFT(M7,FIND("-",M7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="N23" s="5">
-        <f>IF(N7="",0,IFERROR((TIMEVALUE(MID(N7,FIND("-",N7)+1,10))-TIMEVALUE(LEFT(N7,FIND("-",N7)-1)))*24-1,0))</f>
+        <f>IF(N7="",0,IFERROR((TIMEVALUE(MID(N7,FIND("-",N7)+1,10))-TIMEVALUE(LEFT(N7,FIND("-",N7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="O23" s="5">
-        <f>IF(O7="",0,IFERROR((TIMEVALUE(MID(O7,FIND("-",O7)+1,10))-TIMEVALUE(LEFT(O7,FIND("-",O7)-1)))*24-1,0))</f>
+        <f>IF(O7="",0,IFERROR((TIMEVALUE(MID(O7,FIND("-",O7)+1,10))-TIMEVALUE(LEFT(O7,FIND("-",O7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="P23" s="5">
-        <f>IF(P7="",0,IFERROR((TIMEVALUE(MID(P7,FIND("-",P7)+1,10))-TIMEVALUE(LEFT(P7,FIND("-",P7)-1)))*24-1,0))</f>
+        <f>IF(P7="",0,IFERROR((TIMEVALUE(MID(P7,FIND("-",P7)+1,10))-TIMEVALUE(LEFT(P7,FIND("-",P7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Q23" s="5">
@@ -3817,27 +3822,27 @@
         <v/>
       </c>
       <c r="R23" s="5">
-        <f>IF(R7="",0,IFERROR((TIMEVALUE(MID(R7,FIND("-",R7)+1,10))-TIMEVALUE(LEFT(R7,FIND("-",R7)-1)))*24-1,0))</f>
+        <f>IF(R7="",0,IFERROR((TIMEVALUE(MID(R7,FIND("-",R7)+1,10))-TIMEVALUE(LEFT(R7,FIND("-",R7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="S23" s="5">
-        <f>IF(S7="",0,IFERROR((TIMEVALUE(MID(S7,FIND("-",S7)+1,10))-TIMEVALUE(LEFT(S7,FIND("-",S7)-1)))*24-1,0))</f>
+        <f>IF(S7="",0,IFERROR((TIMEVALUE(MID(S7,FIND("-",S7)+1,10))-TIMEVALUE(LEFT(S7,FIND("-",S7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="T23" s="5">
-        <f>IF(T7="",0,IFERROR((TIMEVALUE(MID(T7,FIND("-",T7)+1,10))-TIMEVALUE(LEFT(T7,FIND("-",T7)-1)))*24-1,0))</f>
+        <f>IF(T7="",0,IFERROR((TIMEVALUE(MID(T7,FIND("-",T7)+1,10))-TIMEVALUE(LEFT(T7,FIND("-",T7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="U23" s="5">
-        <f>IF(U7="",0,IFERROR((TIMEVALUE(MID(U7,FIND("-",U7)+1,10))-TIMEVALUE(LEFT(U7,FIND("-",U7)-1)))*24-1,0))</f>
+        <f>IF(U7="",0,IFERROR((TIMEVALUE(MID(U7,FIND("-",U7)+1,10))-TIMEVALUE(LEFT(U7,FIND("-",U7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="V23" s="5">
-        <f>IF(V7="",0,IFERROR((TIMEVALUE(MID(V7,FIND("-",V7)+1,10))-TIMEVALUE(LEFT(V7,FIND("-",V7)-1)))*24-1,0))</f>
+        <f>IF(V7="",0,IFERROR((TIMEVALUE(MID(V7,FIND("-",V7)+1,10))-TIMEVALUE(LEFT(V7,FIND("-",V7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="W23" s="5">
-        <f>IF(W7="",0,IFERROR((TIMEVALUE(MID(W7,FIND("-",W7)+1,10))-TIMEVALUE(LEFT(W7,FIND("-",W7)-1)))*24-1,0))</f>
+        <f>IF(W7="",0,IFERROR((TIMEVALUE(MID(W7,FIND("-",W7)+1,10))-TIMEVALUE(LEFT(W7,FIND("-",W7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="X23" s="5">
@@ -3845,27 +3850,27 @@
         <v/>
       </c>
       <c r="Y23" s="5">
-        <f>IF(Y7="",0,IFERROR((TIMEVALUE(MID(Y7,FIND("-",Y7)+1,10))-TIMEVALUE(LEFT(Y7,FIND("-",Y7)-1)))*24-1,0))</f>
+        <f>IF(Y7="",0,IFERROR((TIMEVALUE(MID(Y7,FIND("-",Y7)+1,10))-TIMEVALUE(LEFT(Y7,FIND("-",Y7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Z23" s="5">
-        <f>IF(Z7="",0,IFERROR((TIMEVALUE(MID(Z7,FIND("-",Z7)+1,10))-TIMEVALUE(LEFT(Z7,FIND("-",Z7)-1)))*24-1,0))</f>
+        <f>IF(Z7="",0,IFERROR((TIMEVALUE(MID(Z7,FIND("-",Z7)+1,10))-TIMEVALUE(LEFT(Z7,FIND("-",Z7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AA23" s="5">
-        <f>IF(AA7="",0,IFERROR((TIMEVALUE(MID(AA7,FIND("-",AA7)+1,10))-TIMEVALUE(LEFT(AA7,FIND("-",AA7)-1)))*24-1,0))</f>
+        <f>IF(AA7="",0,IFERROR((TIMEVALUE(MID(AA7,FIND("-",AA7)+1,10))-TIMEVALUE(LEFT(AA7,FIND("-",AA7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AB23" s="5">
-        <f>IF(AB7="",0,IFERROR((TIMEVALUE(MID(AB7,FIND("-",AB7)+1,10))-TIMEVALUE(LEFT(AB7,FIND("-",AB7)-1)))*24-1,0))</f>
+        <f>IF(AB7="",0,IFERROR((TIMEVALUE(MID(AB7,FIND("-",AB7)+1,10))-TIMEVALUE(LEFT(AB7,FIND("-",AB7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AC23" s="5">
-        <f>IF(AC7="",0,IFERROR((TIMEVALUE(MID(AC7,FIND("-",AC7)+1,10))-TIMEVALUE(LEFT(AC7,FIND("-",AC7)-1)))*24-1,0))</f>
+        <f>IF(AC7="",0,IFERROR((TIMEVALUE(MID(AC7,FIND("-",AC7)+1,10))-TIMEVALUE(LEFT(AC7,FIND("-",AC7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AD23" s="5">
-        <f>IF(AD7="",0,IFERROR((TIMEVALUE(MID(AD7,FIND("-",AD7)+1,10))-TIMEVALUE(LEFT(AD7,FIND("-",AD7)-1)))*24-1,0))</f>
+        <f>IF(AD7="",0,IFERROR((TIMEVALUE(MID(AD7,FIND("-",AD7)+1,10))-TIMEVALUE(LEFT(AD7,FIND("-",AD7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AE23" s="5">
@@ -3873,11 +3878,11 @@
         <v/>
       </c>
       <c r="AF23" s="5">
-        <f>IF(AF7="",0,IFERROR((TIMEVALUE(MID(AF7,FIND("-",AF7)+1,10))-TIMEVALUE(LEFT(AF7,FIND("-",AF7)-1)))*24-1,0))</f>
+        <f>IF(AF7="",0,IFERROR((TIMEVALUE(MID(AF7,FIND("-",AF7)+1,10))-TIMEVALUE(LEFT(AF7,FIND("-",AF7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AG23" s="5">
-        <f>IF(AG7="",0,IFERROR((TIMEVALUE(MID(AG7,FIND("-",AG7)+1,10))-TIMEVALUE(LEFT(AG7,FIND("-",AG7)-1)))*24-1,0))</f>
+        <f>IF(AG7="",0,IFERROR((TIMEVALUE(MID(AG7,FIND("-",AG7)+1,10))-TIMEVALUE(LEFT(AG7,FIND("-",AG7)-1)))*24-IF(ISNUMBER(FIND("-",$C7)),IFERROR((TIMEVALUE(MID($C7,FIND("-",$C7)+1,10))-TIMEVALUE(LEFT($C7,FIND("-",$C7)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AH23" s="5">
@@ -3924,27 +3929,27 @@
         <v/>
       </c>
       <c r="D24" s="5">
-        <f>IF(D8="",0,IFERROR((TIMEVALUE(MID(D8,FIND("-",D8)+1,10))-TIMEVALUE(LEFT(D8,FIND("-",D8)-1)))*24-1,0))</f>
+        <f>IF(D8="",0,IFERROR((TIMEVALUE(MID(D8,FIND("-",D8)+1,10))-TIMEVALUE(LEFT(D8,FIND("-",D8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="E24" s="5">
-        <f>IF(E8="",0,IFERROR((TIMEVALUE(MID(E8,FIND("-",E8)+1,10))-TIMEVALUE(LEFT(E8,FIND("-",E8)-1)))*24-1,0))</f>
+        <f>IF(E8="",0,IFERROR((TIMEVALUE(MID(E8,FIND("-",E8)+1,10))-TIMEVALUE(LEFT(E8,FIND("-",E8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="F24" s="5">
-        <f>IF(F8="",0,IFERROR((TIMEVALUE(MID(F8,FIND("-",F8)+1,10))-TIMEVALUE(LEFT(F8,FIND("-",F8)-1)))*24-1,0))</f>
+        <f>IF(F8="",0,IFERROR((TIMEVALUE(MID(F8,FIND("-",F8)+1,10))-TIMEVALUE(LEFT(F8,FIND("-",F8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="G24" s="5">
-        <f>IF(G8="",0,IFERROR((TIMEVALUE(MID(G8,FIND("-",G8)+1,10))-TIMEVALUE(LEFT(G8,FIND("-",G8)-1)))*24-1,0))</f>
+        <f>IF(G8="",0,IFERROR((TIMEVALUE(MID(G8,FIND("-",G8)+1,10))-TIMEVALUE(LEFT(G8,FIND("-",G8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="H24" s="5">
-        <f>IF(H8="",0,IFERROR((TIMEVALUE(MID(H8,FIND("-",H8)+1,10))-TIMEVALUE(LEFT(H8,FIND("-",H8)-1)))*24-1,0))</f>
+        <f>IF(H8="",0,IFERROR((TIMEVALUE(MID(H8,FIND("-",H8)+1,10))-TIMEVALUE(LEFT(H8,FIND("-",H8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="I24" s="5">
-        <f>IF(I8="",0,IFERROR((TIMEVALUE(MID(I8,FIND("-",I8)+1,10))-TIMEVALUE(LEFT(I8,FIND("-",I8)-1)))*24-1,0))</f>
+        <f>IF(I8="",0,IFERROR((TIMEVALUE(MID(I8,FIND("-",I8)+1,10))-TIMEVALUE(LEFT(I8,FIND("-",I8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="J24" s="5">
@@ -3952,27 +3957,27 @@
         <v/>
       </c>
       <c r="K24" s="5">
-        <f>IF(K8="",0,IFERROR((TIMEVALUE(MID(K8,FIND("-",K8)+1,10))-TIMEVALUE(LEFT(K8,FIND("-",K8)-1)))*24-1,0))</f>
+        <f>IF(K8="",0,IFERROR((TIMEVALUE(MID(K8,FIND("-",K8)+1,10))-TIMEVALUE(LEFT(K8,FIND("-",K8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="L24" s="5">
-        <f>IF(L8="",0,IFERROR((TIMEVALUE(MID(L8,FIND("-",L8)+1,10))-TIMEVALUE(LEFT(L8,FIND("-",L8)-1)))*24-1,0))</f>
+        <f>IF(L8="",0,IFERROR((TIMEVALUE(MID(L8,FIND("-",L8)+1,10))-TIMEVALUE(LEFT(L8,FIND("-",L8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="M24" s="5">
-        <f>IF(M8="",0,IFERROR((TIMEVALUE(MID(M8,FIND("-",M8)+1,10))-TIMEVALUE(LEFT(M8,FIND("-",M8)-1)))*24-1,0))</f>
+        <f>IF(M8="",0,IFERROR((TIMEVALUE(MID(M8,FIND("-",M8)+1,10))-TIMEVALUE(LEFT(M8,FIND("-",M8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="N24" s="5">
-        <f>IF(N8="",0,IFERROR((TIMEVALUE(MID(N8,FIND("-",N8)+1,10))-TIMEVALUE(LEFT(N8,FIND("-",N8)-1)))*24-1,0))</f>
+        <f>IF(N8="",0,IFERROR((TIMEVALUE(MID(N8,FIND("-",N8)+1,10))-TIMEVALUE(LEFT(N8,FIND("-",N8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="O24" s="5">
-        <f>IF(O8="",0,IFERROR((TIMEVALUE(MID(O8,FIND("-",O8)+1,10))-TIMEVALUE(LEFT(O8,FIND("-",O8)-1)))*24-1,0))</f>
+        <f>IF(O8="",0,IFERROR((TIMEVALUE(MID(O8,FIND("-",O8)+1,10))-TIMEVALUE(LEFT(O8,FIND("-",O8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="P24" s="5">
-        <f>IF(P8="",0,IFERROR((TIMEVALUE(MID(P8,FIND("-",P8)+1,10))-TIMEVALUE(LEFT(P8,FIND("-",P8)-1)))*24-1,0))</f>
+        <f>IF(P8="",0,IFERROR((TIMEVALUE(MID(P8,FIND("-",P8)+1,10))-TIMEVALUE(LEFT(P8,FIND("-",P8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Q24" s="5">
@@ -3980,27 +3985,27 @@
         <v/>
       </c>
       <c r="R24" s="5">
-        <f>IF(R8="",0,IFERROR((TIMEVALUE(MID(R8,FIND("-",R8)+1,10))-TIMEVALUE(LEFT(R8,FIND("-",R8)-1)))*24-1,0))</f>
+        <f>IF(R8="",0,IFERROR((TIMEVALUE(MID(R8,FIND("-",R8)+1,10))-TIMEVALUE(LEFT(R8,FIND("-",R8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="S24" s="5">
-        <f>IF(S8="",0,IFERROR((TIMEVALUE(MID(S8,FIND("-",S8)+1,10))-TIMEVALUE(LEFT(S8,FIND("-",S8)-1)))*24-1,0))</f>
+        <f>IF(S8="",0,IFERROR((TIMEVALUE(MID(S8,FIND("-",S8)+1,10))-TIMEVALUE(LEFT(S8,FIND("-",S8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="T24" s="5">
-        <f>IF(T8="",0,IFERROR((TIMEVALUE(MID(T8,FIND("-",T8)+1,10))-TIMEVALUE(LEFT(T8,FIND("-",T8)-1)))*24-1,0))</f>
+        <f>IF(T8="",0,IFERROR((TIMEVALUE(MID(T8,FIND("-",T8)+1,10))-TIMEVALUE(LEFT(T8,FIND("-",T8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="U24" s="5">
-        <f>IF(U8="",0,IFERROR((TIMEVALUE(MID(U8,FIND("-",U8)+1,10))-TIMEVALUE(LEFT(U8,FIND("-",U8)-1)))*24-1,0))</f>
+        <f>IF(U8="",0,IFERROR((TIMEVALUE(MID(U8,FIND("-",U8)+1,10))-TIMEVALUE(LEFT(U8,FIND("-",U8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="V24" s="5">
-        <f>IF(V8="",0,IFERROR((TIMEVALUE(MID(V8,FIND("-",V8)+1,10))-TIMEVALUE(LEFT(V8,FIND("-",V8)-1)))*24-1,0))</f>
+        <f>IF(V8="",0,IFERROR((TIMEVALUE(MID(V8,FIND("-",V8)+1,10))-TIMEVALUE(LEFT(V8,FIND("-",V8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="W24" s="5">
-        <f>IF(W8="",0,IFERROR((TIMEVALUE(MID(W8,FIND("-",W8)+1,10))-TIMEVALUE(LEFT(W8,FIND("-",W8)-1)))*24-1,0))</f>
+        <f>IF(W8="",0,IFERROR((TIMEVALUE(MID(W8,FIND("-",W8)+1,10))-TIMEVALUE(LEFT(W8,FIND("-",W8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="X24" s="5">
@@ -4008,27 +4013,27 @@
         <v/>
       </c>
       <c r="Y24" s="5">
-        <f>IF(Y8="",0,IFERROR((TIMEVALUE(MID(Y8,FIND("-",Y8)+1,10))-TIMEVALUE(LEFT(Y8,FIND("-",Y8)-1)))*24-1,0))</f>
+        <f>IF(Y8="",0,IFERROR((TIMEVALUE(MID(Y8,FIND("-",Y8)+1,10))-TIMEVALUE(LEFT(Y8,FIND("-",Y8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Z24" s="5">
-        <f>IF(Z8="",0,IFERROR((TIMEVALUE(MID(Z8,FIND("-",Z8)+1,10))-TIMEVALUE(LEFT(Z8,FIND("-",Z8)-1)))*24-1,0))</f>
+        <f>IF(Z8="",0,IFERROR((TIMEVALUE(MID(Z8,FIND("-",Z8)+1,10))-TIMEVALUE(LEFT(Z8,FIND("-",Z8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AA24" s="5">
-        <f>IF(AA8="",0,IFERROR((TIMEVALUE(MID(AA8,FIND("-",AA8)+1,10))-TIMEVALUE(LEFT(AA8,FIND("-",AA8)-1)))*24-1,0))</f>
+        <f>IF(AA8="",0,IFERROR((TIMEVALUE(MID(AA8,FIND("-",AA8)+1,10))-TIMEVALUE(LEFT(AA8,FIND("-",AA8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AB24" s="5">
-        <f>IF(AB8="",0,IFERROR((TIMEVALUE(MID(AB8,FIND("-",AB8)+1,10))-TIMEVALUE(LEFT(AB8,FIND("-",AB8)-1)))*24-1,0))</f>
+        <f>IF(AB8="",0,IFERROR((TIMEVALUE(MID(AB8,FIND("-",AB8)+1,10))-TIMEVALUE(LEFT(AB8,FIND("-",AB8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AC24" s="5">
-        <f>IF(AC8="",0,IFERROR((TIMEVALUE(MID(AC8,FIND("-",AC8)+1,10))-TIMEVALUE(LEFT(AC8,FIND("-",AC8)-1)))*24-1,0))</f>
+        <f>IF(AC8="",0,IFERROR((TIMEVALUE(MID(AC8,FIND("-",AC8)+1,10))-TIMEVALUE(LEFT(AC8,FIND("-",AC8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AD24" s="5">
-        <f>IF(AD8="",0,IFERROR((TIMEVALUE(MID(AD8,FIND("-",AD8)+1,10))-TIMEVALUE(LEFT(AD8,FIND("-",AD8)-1)))*24-1,0))</f>
+        <f>IF(AD8="",0,IFERROR((TIMEVALUE(MID(AD8,FIND("-",AD8)+1,10))-TIMEVALUE(LEFT(AD8,FIND("-",AD8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AE24" s="5">
@@ -4036,11 +4041,11 @@
         <v/>
       </c>
       <c r="AF24" s="5">
-        <f>IF(AF8="",0,IFERROR((TIMEVALUE(MID(AF8,FIND("-",AF8)+1,10))-TIMEVALUE(LEFT(AF8,FIND("-",AF8)-1)))*24-1,0))</f>
+        <f>IF(AF8="",0,IFERROR((TIMEVALUE(MID(AF8,FIND("-",AF8)+1,10))-TIMEVALUE(LEFT(AF8,FIND("-",AF8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AG24" s="5">
-        <f>IF(AG8="",0,IFERROR((TIMEVALUE(MID(AG8,FIND("-",AG8)+1,10))-TIMEVALUE(LEFT(AG8,FIND("-",AG8)-1)))*24-1,0))</f>
+        <f>IF(AG8="",0,IFERROR((TIMEVALUE(MID(AG8,FIND("-",AG8)+1,10))-TIMEVALUE(LEFT(AG8,FIND("-",AG8)-1)))*24-IF(ISNUMBER(FIND("-",$C8)),IFERROR((TIMEVALUE(MID($C8,FIND("-",$C8)+1,10))-TIMEVALUE(LEFT($C8,FIND("-",$C8)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AH24" s="5">
@@ -4086,27 +4091,27 @@
         <v/>
       </c>
       <c r="D25" s="5">
-        <f>IF(D9="",0,IFERROR((TIMEVALUE(MID(D9,FIND("-",D9)+1,10))-TIMEVALUE(LEFT(D9,FIND("-",D9)-1)))*24-1,0))</f>
+        <f>IF(D9="",0,IFERROR((TIMEVALUE(MID(D9,FIND("-",D9)+1,10))-TIMEVALUE(LEFT(D9,FIND("-",D9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="E25" s="5">
-        <f>IF(E9="",0,IFERROR((TIMEVALUE(MID(E9,FIND("-",E9)+1,10))-TIMEVALUE(LEFT(E9,FIND("-",E9)-1)))*24-1,0))</f>
+        <f>IF(E9="",0,IFERROR((TIMEVALUE(MID(E9,FIND("-",E9)+1,10))-TIMEVALUE(LEFT(E9,FIND("-",E9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="F25" s="5">
-        <f>IF(F9="",0,IFERROR((TIMEVALUE(MID(F9,FIND("-",F9)+1,10))-TIMEVALUE(LEFT(F9,FIND("-",F9)-1)))*24-1,0))</f>
+        <f>IF(F9="",0,IFERROR((TIMEVALUE(MID(F9,FIND("-",F9)+1,10))-TIMEVALUE(LEFT(F9,FIND("-",F9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="G25" s="5">
-        <f>IF(G9="",0,IFERROR((TIMEVALUE(MID(G9,FIND("-",G9)+1,10))-TIMEVALUE(LEFT(G9,FIND("-",G9)-1)))*24-1,0))</f>
+        <f>IF(G9="",0,IFERROR((TIMEVALUE(MID(G9,FIND("-",G9)+1,10))-TIMEVALUE(LEFT(G9,FIND("-",G9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="H25" s="5">
-        <f>IF(H9="",0,IFERROR((TIMEVALUE(MID(H9,FIND("-",H9)+1,10))-TIMEVALUE(LEFT(H9,FIND("-",H9)-1)))*24-1,0))</f>
+        <f>IF(H9="",0,IFERROR((TIMEVALUE(MID(H9,FIND("-",H9)+1,10))-TIMEVALUE(LEFT(H9,FIND("-",H9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="I25" s="5">
-        <f>IF(I9="",0,IFERROR((TIMEVALUE(MID(I9,FIND("-",I9)+1,10))-TIMEVALUE(LEFT(I9,FIND("-",I9)-1)))*24-1,0))</f>
+        <f>IF(I9="",0,IFERROR((TIMEVALUE(MID(I9,FIND("-",I9)+1,10))-TIMEVALUE(LEFT(I9,FIND("-",I9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="J25" s="5">
@@ -4114,27 +4119,27 @@
         <v/>
       </c>
       <c r="K25" s="5">
-        <f>IF(K9="",0,IFERROR((TIMEVALUE(MID(K9,FIND("-",K9)+1,10))-TIMEVALUE(LEFT(K9,FIND("-",K9)-1)))*24-1,0))</f>
+        <f>IF(K9="",0,IFERROR((TIMEVALUE(MID(K9,FIND("-",K9)+1,10))-TIMEVALUE(LEFT(K9,FIND("-",K9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="L25" s="5">
-        <f>IF(L9="",0,IFERROR((TIMEVALUE(MID(L9,FIND("-",L9)+1,10))-TIMEVALUE(LEFT(L9,FIND("-",L9)-1)))*24-1,0))</f>
+        <f>IF(L9="",0,IFERROR((TIMEVALUE(MID(L9,FIND("-",L9)+1,10))-TIMEVALUE(LEFT(L9,FIND("-",L9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="M25" s="5">
-        <f>IF(M9="",0,IFERROR((TIMEVALUE(MID(M9,FIND("-",M9)+1,10))-TIMEVALUE(LEFT(M9,FIND("-",M9)-1)))*24-1,0))</f>
+        <f>IF(M9="",0,IFERROR((TIMEVALUE(MID(M9,FIND("-",M9)+1,10))-TIMEVALUE(LEFT(M9,FIND("-",M9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="N25" s="5">
-        <f>IF(N9="",0,IFERROR((TIMEVALUE(MID(N9,FIND("-",N9)+1,10))-TIMEVALUE(LEFT(N9,FIND("-",N9)-1)))*24-1,0))</f>
+        <f>IF(N9="",0,IFERROR((TIMEVALUE(MID(N9,FIND("-",N9)+1,10))-TIMEVALUE(LEFT(N9,FIND("-",N9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="O25" s="5">
-        <f>IF(O9="",0,IFERROR((TIMEVALUE(MID(O9,FIND("-",O9)+1,10))-TIMEVALUE(LEFT(O9,FIND("-",O9)-1)))*24-1,0))</f>
+        <f>IF(O9="",0,IFERROR((TIMEVALUE(MID(O9,FIND("-",O9)+1,10))-TIMEVALUE(LEFT(O9,FIND("-",O9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="P25" s="5">
-        <f>IF(P9="",0,IFERROR((TIMEVALUE(MID(P9,FIND("-",P9)+1,10))-TIMEVALUE(LEFT(P9,FIND("-",P9)-1)))*24-1,0))</f>
+        <f>IF(P9="",0,IFERROR((TIMEVALUE(MID(P9,FIND("-",P9)+1,10))-TIMEVALUE(LEFT(P9,FIND("-",P9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Q25" s="5">
@@ -4142,27 +4147,27 @@
         <v/>
       </c>
       <c r="R25" s="5">
-        <f>IF(R9="",0,IFERROR((TIMEVALUE(MID(R9,FIND("-",R9)+1,10))-TIMEVALUE(LEFT(R9,FIND("-",R9)-1)))*24-1,0))</f>
+        <f>IF(R9="",0,IFERROR((TIMEVALUE(MID(R9,FIND("-",R9)+1,10))-TIMEVALUE(LEFT(R9,FIND("-",R9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="S25" s="5">
-        <f>IF(S9="",0,IFERROR((TIMEVALUE(MID(S9,FIND("-",S9)+1,10))-TIMEVALUE(LEFT(S9,FIND("-",S9)-1)))*24-1,0))</f>
+        <f>IF(S9="",0,IFERROR((TIMEVALUE(MID(S9,FIND("-",S9)+1,10))-TIMEVALUE(LEFT(S9,FIND("-",S9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="T25" s="5">
-        <f>IF(T9="",0,IFERROR((TIMEVALUE(MID(T9,FIND("-",T9)+1,10))-TIMEVALUE(LEFT(T9,FIND("-",T9)-1)))*24-1,0))</f>
+        <f>IF(T9="",0,IFERROR((TIMEVALUE(MID(T9,FIND("-",T9)+1,10))-TIMEVALUE(LEFT(T9,FIND("-",T9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="U25" s="5">
-        <f>IF(U9="",0,IFERROR((TIMEVALUE(MID(U9,FIND("-",U9)+1,10))-TIMEVALUE(LEFT(U9,FIND("-",U9)-1)))*24-1,0))</f>
+        <f>IF(U9="",0,IFERROR((TIMEVALUE(MID(U9,FIND("-",U9)+1,10))-TIMEVALUE(LEFT(U9,FIND("-",U9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="V25" s="5">
-        <f>IF(V9="",0,IFERROR((TIMEVALUE(MID(V9,FIND("-",V9)+1,10))-TIMEVALUE(LEFT(V9,FIND("-",V9)-1)))*24-1,0))</f>
+        <f>IF(V9="",0,IFERROR((TIMEVALUE(MID(V9,FIND("-",V9)+1,10))-TIMEVALUE(LEFT(V9,FIND("-",V9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="W25" s="5">
-        <f>IF(W9="",0,IFERROR((TIMEVALUE(MID(W9,FIND("-",W9)+1,10))-TIMEVALUE(LEFT(W9,FIND("-",W9)-1)))*24-1,0))</f>
+        <f>IF(W9="",0,IFERROR((TIMEVALUE(MID(W9,FIND("-",W9)+1,10))-TIMEVALUE(LEFT(W9,FIND("-",W9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="X25" s="5">
@@ -4170,27 +4175,27 @@
         <v/>
       </c>
       <c r="Y25" s="5">
-        <f>IF(Y9="",0,IFERROR((TIMEVALUE(MID(Y9,FIND("-",Y9)+1,10))-TIMEVALUE(LEFT(Y9,FIND("-",Y9)-1)))*24-1,0))</f>
+        <f>IF(Y9="",0,IFERROR((TIMEVALUE(MID(Y9,FIND("-",Y9)+1,10))-TIMEVALUE(LEFT(Y9,FIND("-",Y9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Z25" s="5">
-        <f>IF(Z9="",0,IFERROR((TIMEVALUE(MID(Z9,FIND("-",Z9)+1,10))-TIMEVALUE(LEFT(Z9,FIND("-",Z9)-1)))*24-1,0))</f>
+        <f>IF(Z9="",0,IFERROR((TIMEVALUE(MID(Z9,FIND("-",Z9)+1,10))-TIMEVALUE(LEFT(Z9,FIND("-",Z9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AA25" s="5">
-        <f>IF(AA9="",0,IFERROR((TIMEVALUE(MID(AA9,FIND("-",AA9)+1,10))-TIMEVALUE(LEFT(AA9,FIND("-",AA9)-1)))*24-1,0))</f>
+        <f>IF(AA9="",0,IFERROR((TIMEVALUE(MID(AA9,FIND("-",AA9)+1,10))-TIMEVALUE(LEFT(AA9,FIND("-",AA9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AB25" s="5">
-        <f>IF(AB9="",0,IFERROR((TIMEVALUE(MID(AB9,FIND("-",AB9)+1,10))-TIMEVALUE(LEFT(AB9,FIND("-",AB9)-1)))*24-1,0))</f>
+        <f>IF(AB9="",0,IFERROR((TIMEVALUE(MID(AB9,FIND("-",AB9)+1,10))-TIMEVALUE(LEFT(AB9,FIND("-",AB9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AC25" s="5">
-        <f>IF(AC9="",0,IFERROR((TIMEVALUE(MID(AC9,FIND("-",AC9)+1,10))-TIMEVALUE(LEFT(AC9,FIND("-",AC9)-1)))*24-1,0))</f>
+        <f>IF(AC9="",0,IFERROR((TIMEVALUE(MID(AC9,FIND("-",AC9)+1,10))-TIMEVALUE(LEFT(AC9,FIND("-",AC9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AD25" s="5">
-        <f>IF(AD9="",0,IFERROR((TIMEVALUE(MID(AD9,FIND("-",AD9)+1,10))-TIMEVALUE(LEFT(AD9,FIND("-",AD9)-1)))*24-1,0))</f>
+        <f>IF(AD9="",0,IFERROR((TIMEVALUE(MID(AD9,FIND("-",AD9)+1,10))-TIMEVALUE(LEFT(AD9,FIND("-",AD9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AE25" s="5">
@@ -4198,11 +4203,11 @@
         <v/>
       </c>
       <c r="AF25" s="5">
-        <f>IF(AF9="",0,IFERROR((TIMEVALUE(MID(AF9,FIND("-",AF9)+1,10))-TIMEVALUE(LEFT(AF9,FIND("-",AF9)-1)))*24-1,0))</f>
+        <f>IF(AF9="",0,IFERROR((TIMEVALUE(MID(AF9,FIND("-",AF9)+1,10))-TIMEVALUE(LEFT(AF9,FIND("-",AF9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AG25" s="5">
-        <f>IF(AG9="",0,IFERROR((TIMEVALUE(MID(AG9,FIND("-",AG9)+1,10))-TIMEVALUE(LEFT(AG9,FIND("-",AG9)-1)))*24-1,0))</f>
+        <f>IF(AG9="",0,IFERROR((TIMEVALUE(MID(AG9,FIND("-",AG9)+1,10))-TIMEVALUE(LEFT(AG9,FIND("-",AG9)-1)))*24-IF(ISNUMBER(FIND("-",$C9)),IFERROR((TIMEVALUE(MID($C9,FIND("-",$C9)+1,10))-TIMEVALUE(LEFT($C9,FIND("-",$C9)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AH25" s="5">
@@ -4248,27 +4253,27 @@
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>IF(D10="",0,IFERROR((TIMEVALUE(MID(D10,FIND("-",D10)+1,10))-TIMEVALUE(LEFT(D10,FIND("-",D10)-1)))*24-1,0))</f>
+        <f>IF(D10="",0,IFERROR((TIMEVALUE(MID(D10,FIND("-",D10)+1,10))-TIMEVALUE(LEFT(D10,FIND("-",D10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>IF(E10="",0,IFERROR((TIMEVALUE(MID(E10,FIND("-",E10)+1,10))-TIMEVALUE(LEFT(E10,FIND("-",E10)-1)))*24-1,0))</f>
+        <f>IF(E10="",0,IFERROR((TIMEVALUE(MID(E10,FIND("-",E10)+1,10))-TIMEVALUE(LEFT(E10,FIND("-",E10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="F26" s="5">
-        <f>IF(F10="",0,IFERROR((TIMEVALUE(MID(F10,FIND("-",F10)+1,10))-TIMEVALUE(LEFT(F10,FIND("-",F10)-1)))*24-1,0))</f>
+        <f>IF(F10="",0,IFERROR((TIMEVALUE(MID(F10,FIND("-",F10)+1,10))-TIMEVALUE(LEFT(F10,FIND("-",F10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="G26" s="5">
-        <f>IF(G10="",0,IFERROR((TIMEVALUE(MID(G10,FIND("-",G10)+1,10))-TIMEVALUE(LEFT(G10,FIND("-",G10)-1)))*24-1,0))</f>
+        <f>IF(G10="",0,IFERROR((TIMEVALUE(MID(G10,FIND("-",G10)+1,10))-TIMEVALUE(LEFT(G10,FIND("-",G10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="H26" s="5">
-        <f>IF(H10="",0,IFERROR((TIMEVALUE(MID(H10,FIND("-",H10)+1,10))-TIMEVALUE(LEFT(H10,FIND("-",H10)-1)))*24-1,0))</f>
+        <f>IF(H10="",0,IFERROR((TIMEVALUE(MID(H10,FIND("-",H10)+1,10))-TIMEVALUE(LEFT(H10,FIND("-",H10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="I26" s="5">
-        <f>IF(I10="",0,IFERROR((TIMEVALUE(MID(I10,FIND("-",I10)+1,10))-TIMEVALUE(LEFT(I10,FIND("-",I10)-1)))*24-1,0))</f>
+        <f>IF(I10="",0,IFERROR((TIMEVALUE(MID(I10,FIND("-",I10)+1,10))-TIMEVALUE(LEFT(I10,FIND("-",I10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="J26" s="5">
@@ -4276,27 +4281,27 @@
         <v/>
       </c>
       <c r="K26" s="5">
-        <f>IF(K10="",0,IFERROR((TIMEVALUE(MID(K10,FIND("-",K10)+1,10))-TIMEVALUE(LEFT(K10,FIND("-",K10)-1)))*24-1,0))</f>
+        <f>IF(K10="",0,IFERROR((TIMEVALUE(MID(K10,FIND("-",K10)+1,10))-TIMEVALUE(LEFT(K10,FIND("-",K10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="L26" s="5">
-        <f>IF(L10="",0,IFERROR((TIMEVALUE(MID(L10,FIND("-",L10)+1,10))-TIMEVALUE(LEFT(L10,FIND("-",L10)-1)))*24-1,0))</f>
+        <f>IF(L10="",0,IFERROR((TIMEVALUE(MID(L10,FIND("-",L10)+1,10))-TIMEVALUE(LEFT(L10,FIND("-",L10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="M26" s="5">
-        <f>IF(M10="",0,IFERROR((TIMEVALUE(MID(M10,FIND("-",M10)+1,10))-TIMEVALUE(LEFT(M10,FIND("-",M10)-1)))*24-1,0))</f>
+        <f>IF(M10="",0,IFERROR((TIMEVALUE(MID(M10,FIND("-",M10)+1,10))-TIMEVALUE(LEFT(M10,FIND("-",M10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="N26" s="5">
-        <f>IF(N10="",0,IFERROR((TIMEVALUE(MID(N10,FIND("-",N10)+1,10))-TIMEVALUE(LEFT(N10,FIND("-",N10)-1)))*24-1,0))</f>
+        <f>IF(N10="",0,IFERROR((TIMEVALUE(MID(N10,FIND("-",N10)+1,10))-TIMEVALUE(LEFT(N10,FIND("-",N10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="O26" s="5">
-        <f>IF(O10="",0,IFERROR((TIMEVALUE(MID(O10,FIND("-",O10)+1,10))-TIMEVALUE(LEFT(O10,FIND("-",O10)-1)))*24-1,0))</f>
+        <f>IF(O10="",0,IFERROR((TIMEVALUE(MID(O10,FIND("-",O10)+1,10))-TIMEVALUE(LEFT(O10,FIND("-",O10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="P26" s="5">
-        <f>IF(P10="",0,IFERROR((TIMEVALUE(MID(P10,FIND("-",P10)+1,10))-TIMEVALUE(LEFT(P10,FIND("-",P10)-1)))*24-1,0))</f>
+        <f>IF(P10="",0,IFERROR((TIMEVALUE(MID(P10,FIND("-",P10)+1,10))-TIMEVALUE(LEFT(P10,FIND("-",P10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Q26" s="5">
@@ -4304,27 +4309,27 @@
         <v/>
       </c>
       <c r="R26" s="5">
-        <f>IF(R10="",0,IFERROR((TIMEVALUE(MID(R10,FIND("-",R10)+1,10))-TIMEVALUE(LEFT(R10,FIND("-",R10)-1)))*24-1,0))</f>
+        <f>IF(R10="",0,IFERROR((TIMEVALUE(MID(R10,FIND("-",R10)+1,10))-TIMEVALUE(LEFT(R10,FIND("-",R10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="S26" s="5">
-        <f>IF(S10="",0,IFERROR((TIMEVALUE(MID(S10,FIND("-",S10)+1,10))-TIMEVALUE(LEFT(S10,FIND("-",S10)-1)))*24-1,0))</f>
+        <f>IF(S10="",0,IFERROR((TIMEVALUE(MID(S10,FIND("-",S10)+1,10))-TIMEVALUE(LEFT(S10,FIND("-",S10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="T26" s="5">
-        <f>IF(T10="",0,IFERROR((TIMEVALUE(MID(T10,FIND("-",T10)+1,10))-TIMEVALUE(LEFT(T10,FIND("-",T10)-1)))*24-1,0))</f>
+        <f>IF(T10="",0,IFERROR((TIMEVALUE(MID(T10,FIND("-",T10)+1,10))-TIMEVALUE(LEFT(T10,FIND("-",T10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="U26" s="5">
-        <f>IF(U10="",0,IFERROR((TIMEVALUE(MID(U10,FIND("-",U10)+1,10))-TIMEVALUE(LEFT(U10,FIND("-",U10)-1)))*24-1,0))</f>
+        <f>IF(U10="",0,IFERROR((TIMEVALUE(MID(U10,FIND("-",U10)+1,10))-TIMEVALUE(LEFT(U10,FIND("-",U10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="V26" s="5">
-        <f>IF(V10="",0,IFERROR((TIMEVALUE(MID(V10,FIND("-",V10)+1,10))-TIMEVALUE(LEFT(V10,FIND("-",V10)-1)))*24-1,0))</f>
+        <f>IF(V10="",0,IFERROR((TIMEVALUE(MID(V10,FIND("-",V10)+1,10))-TIMEVALUE(LEFT(V10,FIND("-",V10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="W26" s="5">
-        <f>IF(W10="",0,IFERROR((TIMEVALUE(MID(W10,FIND("-",W10)+1,10))-TIMEVALUE(LEFT(W10,FIND("-",W10)-1)))*24-1,0))</f>
+        <f>IF(W10="",0,IFERROR((TIMEVALUE(MID(W10,FIND("-",W10)+1,10))-TIMEVALUE(LEFT(W10,FIND("-",W10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="X26" s="5">
@@ -4332,27 +4337,27 @@
         <v/>
       </c>
       <c r="Y26" s="5">
-        <f>IF(Y10="",0,IFERROR((TIMEVALUE(MID(Y10,FIND("-",Y10)+1,10))-TIMEVALUE(LEFT(Y10,FIND("-",Y10)-1)))*24-1,0))</f>
+        <f>IF(Y10="",0,IFERROR((TIMEVALUE(MID(Y10,FIND("-",Y10)+1,10))-TIMEVALUE(LEFT(Y10,FIND("-",Y10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Z26" s="5">
-        <f>IF(Z10="",0,IFERROR((TIMEVALUE(MID(Z10,FIND("-",Z10)+1,10))-TIMEVALUE(LEFT(Z10,FIND("-",Z10)-1)))*24-1,0))</f>
+        <f>IF(Z10="",0,IFERROR((TIMEVALUE(MID(Z10,FIND("-",Z10)+1,10))-TIMEVALUE(LEFT(Z10,FIND("-",Z10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AA26" s="5">
-        <f>IF(AA10="",0,IFERROR((TIMEVALUE(MID(AA10,FIND("-",AA10)+1,10))-TIMEVALUE(LEFT(AA10,FIND("-",AA10)-1)))*24-1,0))</f>
+        <f>IF(AA10="",0,IFERROR((TIMEVALUE(MID(AA10,FIND("-",AA10)+1,10))-TIMEVALUE(LEFT(AA10,FIND("-",AA10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AB26" s="5">
-        <f>IF(AB10="",0,IFERROR((TIMEVALUE(MID(AB10,FIND("-",AB10)+1,10))-TIMEVALUE(LEFT(AB10,FIND("-",AB10)-1)))*24-1,0))</f>
+        <f>IF(AB10="",0,IFERROR((TIMEVALUE(MID(AB10,FIND("-",AB10)+1,10))-TIMEVALUE(LEFT(AB10,FIND("-",AB10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AC26" s="5">
-        <f>IF(AC10="",0,IFERROR((TIMEVALUE(MID(AC10,FIND("-",AC10)+1,10))-TIMEVALUE(LEFT(AC10,FIND("-",AC10)-1)))*24-1,0))</f>
+        <f>IF(AC10="",0,IFERROR((TIMEVALUE(MID(AC10,FIND("-",AC10)+1,10))-TIMEVALUE(LEFT(AC10,FIND("-",AC10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AD26" s="5">
-        <f>IF(AD10="",0,IFERROR((TIMEVALUE(MID(AD10,FIND("-",AD10)+1,10))-TIMEVALUE(LEFT(AD10,FIND("-",AD10)-1)))*24-1,0))</f>
+        <f>IF(AD10="",0,IFERROR((TIMEVALUE(MID(AD10,FIND("-",AD10)+1,10))-TIMEVALUE(LEFT(AD10,FIND("-",AD10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AE26" s="5">
@@ -4360,11 +4365,11 @@
         <v/>
       </c>
       <c r="AF26" s="5">
-        <f>IF(AF10="",0,IFERROR((TIMEVALUE(MID(AF10,FIND("-",AF10)+1,10))-TIMEVALUE(LEFT(AF10,FIND("-",AF10)-1)))*24-1,0))</f>
+        <f>IF(AF10="",0,IFERROR((TIMEVALUE(MID(AF10,FIND("-",AF10)+1,10))-TIMEVALUE(LEFT(AF10,FIND("-",AF10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AG26" s="5">
-        <f>IF(AG10="",0,IFERROR((TIMEVALUE(MID(AG10,FIND("-",AG10)+1,10))-TIMEVALUE(LEFT(AG10,FIND("-",AG10)-1)))*24-1,0))</f>
+        <f>IF(AG10="",0,IFERROR((TIMEVALUE(MID(AG10,FIND("-",AG10)+1,10))-TIMEVALUE(LEFT(AG10,FIND("-",AG10)-1)))*24-IF(ISNUMBER(FIND("-",$C10)),IFERROR((TIMEVALUE(MID($C10,FIND("-",$C10)+1,10))-TIMEVALUE(LEFT($C10,FIND("-",$C10)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AH26" s="5">
@@ -4411,27 +4416,27 @@
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>IF(D11="",0,IFERROR((TIMEVALUE(MID(D11,FIND("-",D11)+1,10))-TIMEVALUE(LEFT(D11,FIND("-",D11)-1)))*24-1,0))</f>
+        <f>IF(D11="",0,IFERROR((TIMEVALUE(MID(D11,FIND("-",D11)+1,10))-TIMEVALUE(LEFT(D11,FIND("-",D11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>IF(E11="",0,IFERROR((TIMEVALUE(MID(E11,FIND("-",E11)+1,10))-TIMEVALUE(LEFT(E11,FIND("-",E11)-1)))*24-1,0))</f>
+        <f>IF(E11="",0,IFERROR((TIMEVALUE(MID(E11,FIND("-",E11)+1,10))-TIMEVALUE(LEFT(E11,FIND("-",E11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="F27" s="5">
-        <f>IF(F11="",0,IFERROR((TIMEVALUE(MID(F11,FIND("-",F11)+1,10))-TIMEVALUE(LEFT(F11,FIND("-",F11)-1)))*24-1,0))</f>
+        <f>IF(F11="",0,IFERROR((TIMEVALUE(MID(F11,FIND("-",F11)+1,10))-TIMEVALUE(LEFT(F11,FIND("-",F11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="G27" s="5">
-        <f>IF(G11="",0,IFERROR((TIMEVALUE(MID(G11,FIND("-",G11)+1,10))-TIMEVALUE(LEFT(G11,FIND("-",G11)-1)))*24-1,0))</f>
+        <f>IF(G11="",0,IFERROR((TIMEVALUE(MID(G11,FIND("-",G11)+1,10))-TIMEVALUE(LEFT(G11,FIND("-",G11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="H27" s="5">
-        <f>IF(H11="",0,IFERROR((TIMEVALUE(MID(H11,FIND("-",H11)+1,10))-TIMEVALUE(LEFT(H11,FIND("-",H11)-1)))*24-1,0))</f>
+        <f>IF(H11="",0,IFERROR((TIMEVALUE(MID(H11,FIND("-",H11)+1,10))-TIMEVALUE(LEFT(H11,FIND("-",H11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="I27" s="5">
-        <f>IF(I11="",0,IFERROR((TIMEVALUE(MID(I11,FIND("-",I11)+1,10))-TIMEVALUE(LEFT(I11,FIND("-",I11)-1)))*24-1,0))</f>
+        <f>IF(I11="",0,IFERROR((TIMEVALUE(MID(I11,FIND("-",I11)+1,10))-TIMEVALUE(LEFT(I11,FIND("-",I11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="J27" s="5">
@@ -4439,27 +4444,27 @@
         <v/>
       </c>
       <c r="K27" s="5">
-        <f>IF(K11="",0,IFERROR((TIMEVALUE(MID(K11,FIND("-",K11)+1,10))-TIMEVALUE(LEFT(K11,FIND("-",K11)-1)))*24-1,0))</f>
+        <f>IF(K11="",0,IFERROR((TIMEVALUE(MID(K11,FIND("-",K11)+1,10))-TIMEVALUE(LEFT(K11,FIND("-",K11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="L27" s="5">
-        <f>IF(L11="",0,IFERROR((TIMEVALUE(MID(L11,FIND("-",L11)+1,10))-TIMEVALUE(LEFT(L11,FIND("-",L11)-1)))*24-1,0))</f>
+        <f>IF(L11="",0,IFERROR((TIMEVALUE(MID(L11,FIND("-",L11)+1,10))-TIMEVALUE(LEFT(L11,FIND("-",L11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="M27" s="5">
-        <f>IF(M11="",0,IFERROR((TIMEVALUE(MID(M11,FIND("-",M11)+1,10))-TIMEVALUE(LEFT(M11,FIND("-",M11)-1)))*24-1,0))</f>
+        <f>IF(M11="",0,IFERROR((TIMEVALUE(MID(M11,FIND("-",M11)+1,10))-TIMEVALUE(LEFT(M11,FIND("-",M11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="N27" s="5">
-        <f>IF(N11="",0,IFERROR((TIMEVALUE(MID(N11,FIND("-",N11)+1,10))-TIMEVALUE(LEFT(N11,FIND("-",N11)-1)))*24-1,0))</f>
+        <f>IF(N11="",0,IFERROR((TIMEVALUE(MID(N11,FIND("-",N11)+1,10))-TIMEVALUE(LEFT(N11,FIND("-",N11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="O27" s="5">
-        <f>IF(O11="",0,IFERROR((TIMEVALUE(MID(O11,FIND("-",O11)+1,10))-TIMEVALUE(LEFT(O11,FIND("-",O11)-1)))*24-1,0))</f>
+        <f>IF(O11="",0,IFERROR((TIMEVALUE(MID(O11,FIND("-",O11)+1,10))-TIMEVALUE(LEFT(O11,FIND("-",O11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="P27" s="5">
-        <f>IF(P11="",0,IFERROR((TIMEVALUE(MID(P11,FIND("-",P11)+1,10))-TIMEVALUE(LEFT(P11,FIND("-",P11)-1)))*24-1,0))</f>
+        <f>IF(P11="",0,IFERROR((TIMEVALUE(MID(P11,FIND("-",P11)+1,10))-TIMEVALUE(LEFT(P11,FIND("-",P11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Q27" s="5">
@@ -4467,27 +4472,27 @@
         <v/>
       </c>
       <c r="R27" s="5">
-        <f>IF(R11="",0,IFERROR((TIMEVALUE(MID(R11,FIND("-",R11)+1,10))-TIMEVALUE(LEFT(R11,FIND("-",R11)-1)))*24-1,0))</f>
+        <f>IF(R11="",0,IFERROR((TIMEVALUE(MID(R11,FIND("-",R11)+1,10))-TIMEVALUE(LEFT(R11,FIND("-",R11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="S27" s="5">
-        <f>IF(S11="",0,IFERROR((TIMEVALUE(MID(S11,FIND("-",S11)+1,10))-TIMEVALUE(LEFT(S11,FIND("-",S11)-1)))*24-1,0))</f>
+        <f>IF(S11="",0,IFERROR((TIMEVALUE(MID(S11,FIND("-",S11)+1,10))-TIMEVALUE(LEFT(S11,FIND("-",S11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="T27" s="5">
-        <f>IF(T11="",0,IFERROR((TIMEVALUE(MID(T11,FIND("-",T11)+1,10))-TIMEVALUE(LEFT(T11,FIND("-",T11)-1)))*24-1,0))</f>
+        <f>IF(T11="",0,IFERROR((TIMEVALUE(MID(T11,FIND("-",T11)+1,10))-TIMEVALUE(LEFT(T11,FIND("-",T11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="U27" s="5">
-        <f>IF(U11="",0,IFERROR((TIMEVALUE(MID(U11,FIND("-",U11)+1,10))-TIMEVALUE(LEFT(U11,FIND("-",U11)-1)))*24-1,0))</f>
+        <f>IF(U11="",0,IFERROR((TIMEVALUE(MID(U11,FIND("-",U11)+1,10))-TIMEVALUE(LEFT(U11,FIND("-",U11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="V27" s="5">
-        <f>IF(V11="",0,IFERROR((TIMEVALUE(MID(V11,FIND("-",V11)+1,10))-TIMEVALUE(LEFT(V11,FIND("-",V11)-1)))*24-1,0))</f>
+        <f>IF(V11="",0,IFERROR((TIMEVALUE(MID(V11,FIND("-",V11)+1,10))-TIMEVALUE(LEFT(V11,FIND("-",V11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="W27" s="5">
-        <f>IF(W11="",0,IFERROR((TIMEVALUE(MID(W11,FIND("-",W11)+1,10))-TIMEVALUE(LEFT(W11,FIND("-",W11)-1)))*24-1,0))</f>
+        <f>IF(W11="",0,IFERROR((TIMEVALUE(MID(W11,FIND("-",W11)+1,10))-TIMEVALUE(LEFT(W11,FIND("-",W11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="X27" s="5">
@@ -4495,27 +4500,27 @@
         <v/>
       </c>
       <c r="Y27" s="5">
-        <f>IF(Y11="",0,IFERROR((TIMEVALUE(MID(Y11,FIND("-",Y11)+1,10))-TIMEVALUE(LEFT(Y11,FIND("-",Y11)-1)))*24-1,0))</f>
+        <f>IF(Y11="",0,IFERROR((TIMEVALUE(MID(Y11,FIND("-",Y11)+1,10))-TIMEVALUE(LEFT(Y11,FIND("-",Y11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Z27" s="5">
-        <f>IF(Z11="",0,IFERROR((TIMEVALUE(MID(Z11,FIND("-",Z11)+1,10))-TIMEVALUE(LEFT(Z11,FIND("-",Z11)-1)))*24-1,0))</f>
+        <f>IF(Z11="",0,IFERROR((TIMEVALUE(MID(Z11,FIND("-",Z11)+1,10))-TIMEVALUE(LEFT(Z11,FIND("-",Z11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AA27" s="5">
-        <f>IF(AA11="",0,IFERROR((TIMEVALUE(MID(AA11,FIND("-",AA11)+1,10))-TIMEVALUE(LEFT(AA11,FIND("-",AA11)-1)))*24-1,0))</f>
+        <f>IF(AA11="",0,IFERROR((TIMEVALUE(MID(AA11,FIND("-",AA11)+1,10))-TIMEVALUE(LEFT(AA11,FIND("-",AA11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AB27" s="5">
-        <f>IF(AB11="",0,IFERROR((TIMEVALUE(MID(AB11,FIND("-",AB11)+1,10))-TIMEVALUE(LEFT(AB11,FIND("-",AB11)-1)))*24-1,0))</f>
+        <f>IF(AB11="",0,IFERROR((TIMEVALUE(MID(AB11,FIND("-",AB11)+1,10))-TIMEVALUE(LEFT(AB11,FIND("-",AB11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AC27" s="5">
-        <f>IF(AC11="",0,IFERROR((TIMEVALUE(MID(AC11,FIND("-",AC11)+1,10))-TIMEVALUE(LEFT(AC11,FIND("-",AC11)-1)))*24-1,0))</f>
+        <f>IF(AC11="",0,IFERROR((TIMEVALUE(MID(AC11,FIND("-",AC11)+1,10))-TIMEVALUE(LEFT(AC11,FIND("-",AC11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AD27" s="5">
-        <f>IF(AD11="",0,IFERROR((TIMEVALUE(MID(AD11,FIND("-",AD11)+1,10))-TIMEVALUE(LEFT(AD11,FIND("-",AD11)-1)))*24-1,0))</f>
+        <f>IF(AD11="",0,IFERROR((TIMEVALUE(MID(AD11,FIND("-",AD11)+1,10))-TIMEVALUE(LEFT(AD11,FIND("-",AD11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AE27" s="5">
@@ -4523,11 +4528,11 @@
         <v/>
       </c>
       <c r="AF27" s="5">
-        <f>IF(AF11="",0,IFERROR((TIMEVALUE(MID(AF11,FIND("-",AF11)+1,10))-TIMEVALUE(LEFT(AF11,FIND("-",AF11)-1)))*24-1,0))</f>
+        <f>IF(AF11="",0,IFERROR((TIMEVALUE(MID(AF11,FIND("-",AF11)+1,10))-TIMEVALUE(LEFT(AF11,FIND("-",AF11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AG27" s="5">
-        <f>IF(AG11="",0,IFERROR((TIMEVALUE(MID(AG11,FIND("-",AG11)+1,10))-TIMEVALUE(LEFT(AG11,FIND("-",AG11)-1)))*24-1,0))</f>
+        <f>IF(AG11="",0,IFERROR((TIMEVALUE(MID(AG11,FIND("-",AG11)+1,10))-TIMEVALUE(LEFT(AG11,FIND("-",AG11)-1)))*24-IF(ISNUMBER(FIND("-",$C11)),IFERROR((TIMEVALUE(MID($C11,FIND("-",$C11)+1,10))-TIMEVALUE(LEFT($C11,FIND("-",$C11)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AH27" s="5">
@@ -4573,27 +4578,27 @@
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>IF(D12="",0,IFERROR((TIMEVALUE(MID(D12,FIND("-",D12)+1,10))-TIMEVALUE(LEFT(D12,FIND("-",D12)-1)))*24-1,0))</f>
+        <f>IF(D12="",0,IFERROR((TIMEVALUE(MID(D12,FIND("-",D12)+1,10))-TIMEVALUE(LEFT(D12,FIND("-",D12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>IF(E12="",0,IFERROR((TIMEVALUE(MID(E12,FIND("-",E12)+1,10))-TIMEVALUE(LEFT(E12,FIND("-",E12)-1)))*24-1,0))</f>
+        <f>IF(E12="",0,IFERROR((TIMEVALUE(MID(E12,FIND("-",E12)+1,10))-TIMEVALUE(LEFT(E12,FIND("-",E12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="F28" s="5">
-        <f>IF(F12="",0,IFERROR((TIMEVALUE(MID(F12,FIND("-",F12)+1,10))-TIMEVALUE(LEFT(F12,FIND("-",F12)-1)))*24-1,0))</f>
+        <f>IF(F12="",0,IFERROR((TIMEVALUE(MID(F12,FIND("-",F12)+1,10))-TIMEVALUE(LEFT(F12,FIND("-",F12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="G28" s="5">
-        <f>IF(G12="",0,IFERROR((TIMEVALUE(MID(G12,FIND("-",G12)+1,10))-TIMEVALUE(LEFT(G12,FIND("-",G12)-1)))*24-1,0))</f>
+        <f>IF(G12="",0,IFERROR((TIMEVALUE(MID(G12,FIND("-",G12)+1,10))-TIMEVALUE(LEFT(G12,FIND("-",G12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="H28" s="5">
-        <f>IF(H12="",0,IFERROR((TIMEVALUE(MID(H12,FIND("-",H12)+1,10))-TIMEVALUE(LEFT(H12,FIND("-",H12)-1)))*24-1,0))</f>
+        <f>IF(H12="",0,IFERROR((TIMEVALUE(MID(H12,FIND("-",H12)+1,10))-TIMEVALUE(LEFT(H12,FIND("-",H12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="I28" s="5">
-        <f>IF(I12="",0,IFERROR((TIMEVALUE(MID(I12,FIND("-",I12)+1,10))-TIMEVALUE(LEFT(I12,FIND("-",I12)-1)))*24-1,0))</f>
+        <f>IF(I12="",0,IFERROR((TIMEVALUE(MID(I12,FIND("-",I12)+1,10))-TIMEVALUE(LEFT(I12,FIND("-",I12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="J28" s="5">
@@ -4601,27 +4606,27 @@
         <v/>
       </c>
       <c r="K28" s="5">
-        <f>IF(K12="",0,IFERROR((TIMEVALUE(MID(K12,FIND("-",K12)+1,10))-TIMEVALUE(LEFT(K12,FIND("-",K12)-1)))*24-1,0))</f>
+        <f>IF(K12="",0,IFERROR((TIMEVALUE(MID(K12,FIND("-",K12)+1,10))-TIMEVALUE(LEFT(K12,FIND("-",K12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="L28" s="5">
-        <f>IF(L12="",0,IFERROR((TIMEVALUE(MID(L12,FIND("-",L12)+1,10))-TIMEVALUE(LEFT(L12,FIND("-",L12)-1)))*24-1,0))</f>
+        <f>IF(L12="",0,IFERROR((TIMEVALUE(MID(L12,FIND("-",L12)+1,10))-TIMEVALUE(LEFT(L12,FIND("-",L12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="M28" s="5">
-        <f>IF(M12="",0,IFERROR((TIMEVALUE(MID(M12,FIND("-",M12)+1,10))-TIMEVALUE(LEFT(M12,FIND("-",M12)-1)))*24-1,0))</f>
+        <f>IF(M12="",0,IFERROR((TIMEVALUE(MID(M12,FIND("-",M12)+1,10))-TIMEVALUE(LEFT(M12,FIND("-",M12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="N28" s="5">
-        <f>IF(N12="",0,IFERROR((TIMEVALUE(MID(N12,FIND("-",N12)+1,10))-TIMEVALUE(LEFT(N12,FIND("-",N12)-1)))*24-1,0))</f>
+        <f>IF(N12="",0,IFERROR((TIMEVALUE(MID(N12,FIND("-",N12)+1,10))-TIMEVALUE(LEFT(N12,FIND("-",N12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="O28" s="5">
-        <f>IF(O12="",0,IFERROR((TIMEVALUE(MID(O12,FIND("-",O12)+1,10))-TIMEVALUE(LEFT(O12,FIND("-",O12)-1)))*24-1,0))</f>
+        <f>IF(O12="",0,IFERROR((TIMEVALUE(MID(O12,FIND("-",O12)+1,10))-TIMEVALUE(LEFT(O12,FIND("-",O12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="P28" s="5">
-        <f>IF(P12="",0,IFERROR((TIMEVALUE(MID(P12,FIND("-",P12)+1,10))-TIMEVALUE(LEFT(P12,FIND("-",P12)-1)))*24-1,0))</f>
+        <f>IF(P12="",0,IFERROR((TIMEVALUE(MID(P12,FIND("-",P12)+1,10))-TIMEVALUE(LEFT(P12,FIND("-",P12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Q28" s="5">
@@ -4629,27 +4634,27 @@
         <v/>
       </c>
       <c r="R28" s="5">
-        <f>IF(R12="",0,IFERROR((TIMEVALUE(MID(R12,FIND("-",R12)+1,10))-TIMEVALUE(LEFT(R12,FIND("-",R12)-1)))*24-1,0))</f>
+        <f>IF(R12="",0,IFERROR((TIMEVALUE(MID(R12,FIND("-",R12)+1,10))-TIMEVALUE(LEFT(R12,FIND("-",R12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="S28" s="5">
-        <f>IF(S12="",0,IFERROR((TIMEVALUE(MID(S12,FIND("-",S12)+1,10))-TIMEVALUE(LEFT(S12,FIND("-",S12)-1)))*24-1,0))</f>
+        <f>IF(S12="",0,IFERROR((TIMEVALUE(MID(S12,FIND("-",S12)+1,10))-TIMEVALUE(LEFT(S12,FIND("-",S12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="T28" s="5">
-        <f>IF(T12="",0,IFERROR((TIMEVALUE(MID(T12,FIND("-",T12)+1,10))-TIMEVALUE(LEFT(T12,FIND("-",T12)-1)))*24-1,0))</f>
+        <f>IF(T12="",0,IFERROR((TIMEVALUE(MID(T12,FIND("-",T12)+1,10))-TIMEVALUE(LEFT(T12,FIND("-",T12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="U28" s="5">
-        <f>IF(U12="",0,IFERROR((TIMEVALUE(MID(U12,FIND("-",U12)+1,10))-TIMEVALUE(LEFT(U12,FIND("-",U12)-1)))*24-1,0))</f>
+        <f>IF(U12="",0,IFERROR((TIMEVALUE(MID(U12,FIND("-",U12)+1,10))-TIMEVALUE(LEFT(U12,FIND("-",U12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="V28" s="5">
-        <f>IF(V12="",0,IFERROR((TIMEVALUE(MID(V12,FIND("-",V12)+1,10))-TIMEVALUE(LEFT(V12,FIND("-",V12)-1)))*24-1,0))</f>
+        <f>IF(V12="",0,IFERROR((TIMEVALUE(MID(V12,FIND("-",V12)+1,10))-TIMEVALUE(LEFT(V12,FIND("-",V12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="W28" s="5">
-        <f>IF(W12="",0,IFERROR((TIMEVALUE(MID(W12,FIND("-",W12)+1,10))-TIMEVALUE(LEFT(W12,FIND("-",W12)-1)))*24-1,0))</f>
+        <f>IF(W12="",0,IFERROR((TIMEVALUE(MID(W12,FIND("-",W12)+1,10))-TIMEVALUE(LEFT(W12,FIND("-",W12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="X28" s="5">
@@ -4657,27 +4662,27 @@
         <v/>
       </c>
       <c r="Y28" s="5">
-        <f>IF(Y12="",0,IFERROR((TIMEVALUE(MID(Y12,FIND("-",Y12)+1,10))-TIMEVALUE(LEFT(Y12,FIND("-",Y12)-1)))*24-1,0))</f>
+        <f>IF(Y12="",0,IFERROR((TIMEVALUE(MID(Y12,FIND("-",Y12)+1,10))-TIMEVALUE(LEFT(Y12,FIND("-",Y12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Z28" s="5">
-        <f>IF(Z12="",0,IFERROR((TIMEVALUE(MID(Z12,FIND("-",Z12)+1,10))-TIMEVALUE(LEFT(Z12,FIND("-",Z12)-1)))*24-1,0))</f>
+        <f>IF(Z12="",0,IFERROR((TIMEVALUE(MID(Z12,FIND("-",Z12)+1,10))-TIMEVALUE(LEFT(Z12,FIND("-",Z12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AA28" s="5">
-        <f>IF(AA12="",0,IFERROR((TIMEVALUE(MID(AA12,FIND("-",AA12)+1,10))-TIMEVALUE(LEFT(AA12,FIND("-",AA12)-1)))*24-1,0))</f>
+        <f>IF(AA12="",0,IFERROR((TIMEVALUE(MID(AA12,FIND("-",AA12)+1,10))-TIMEVALUE(LEFT(AA12,FIND("-",AA12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AB28" s="5">
-        <f>IF(AB12="",0,IFERROR((TIMEVALUE(MID(AB12,FIND("-",AB12)+1,10))-TIMEVALUE(LEFT(AB12,FIND("-",AB12)-1)))*24-1,0))</f>
+        <f>IF(AB12="",0,IFERROR((TIMEVALUE(MID(AB12,FIND("-",AB12)+1,10))-TIMEVALUE(LEFT(AB12,FIND("-",AB12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AC28" s="5">
-        <f>IF(AC12="",0,IFERROR((TIMEVALUE(MID(AC12,FIND("-",AC12)+1,10))-TIMEVALUE(LEFT(AC12,FIND("-",AC12)-1)))*24-1,0))</f>
+        <f>IF(AC12="",0,IFERROR((TIMEVALUE(MID(AC12,FIND("-",AC12)+1,10))-TIMEVALUE(LEFT(AC12,FIND("-",AC12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AD28" s="5">
-        <f>IF(AD12="",0,IFERROR((TIMEVALUE(MID(AD12,FIND("-",AD12)+1,10))-TIMEVALUE(LEFT(AD12,FIND("-",AD12)-1)))*24-1,0))</f>
+        <f>IF(AD12="",0,IFERROR((TIMEVALUE(MID(AD12,FIND("-",AD12)+1,10))-TIMEVALUE(LEFT(AD12,FIND("-",AD12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AE28" s="5">
@@ -4685,11 +4690,11 @@
         <v/>
       </c>
       <c r="AF28" s="5">
-        <f>IF(AF12="",0,IFERROR((TIMEVALUE(MID(AF12,FIND("-",AF12)+1,10))-TIMEVALUE(LEFT(AF12,FIND("-",AF12)-1)))*24-1,0))</f>
+        <f>IF(AF12="",0,IFERROR((TIMEVALUE(MID(AF12,FIND("-",AF12)+1,10))-TIMEVALUE(LEFT(AF12,FIND("-",AF12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AG28" s="5">
-        <f>IF(AG12="",0,IFERROR((TIMEVALUE(MID(AG12,FIND("-",AG12)+1,10))-TIMEVALUE(LEFT(AG12,FIND("-",AG12)-1)))*24-1,0))</f>
+        <f>IF(AG12="",0,IFERROR((TIMEVALUE(MID(AG12,FIND("-",AG12)+1,10))-TIMEVALUE(LEFT(AG12,FIND("-",AG12)-1)))*24-IF(ISNUMBER(FIND("-",$C12)),IFERROR((TIMEVALUE(MID($C12,FIND("-",$C12)+1,10))-TIMEVALUE(LEFT($C12,FIND("-",$C12)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AH28" s="5">
@@ -4735,27 +4740,27 @@
         <v/>
       </c>
       <c r="D29" s="5">
-        <f>IF(D13="",0,IFERROR((TIMEVALUE(MID(D13,FIND("-",D13)+1,10))-TIMEVALUE(LEFT(D13,FIND("-",D13)-1)))*24-1,0))</f>
+        <f>IF(D13="",0,IFERROR((TIMEVALUE(MID(D13,FIND("-",D13)+1,10))-TIMEVALUE(LEFT(D13,FIND("-",D13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="E29" s="5">
-        <f>IF(E13="",0,IFERROR((TIMEVALUE(MID(E13,FIND("-",E13)+1,10))-TIMEVALUE(LEFT(E13,FIND("-",E13)-1)))*24-1,0))</f>
+        <f>IF(E13="",0,IFERROR((TIMEVALUE(MID(E13,FIND("-",E13)+1,10))-TIMEVALUE(LEFT(E13,FIND("-",E13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="F29" s="5">
-        <f>IF(F13="",0,IFERROR((TIMEVALUE(MID(F13,FIND("-",F13)+1,10))-TIMEVALUE(LEFT(F13,FIND("-",F13)-1)))*24-1,0))</f>
+        <f>IF(F13="",0,IFERROR((TIMEVALUE(MID(F13,FIND("-",F13)+1,10))-TIMEVALUE(LEFT(F13,FIND("-",F13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="G29" s="5">
-        <f>IF(G13="",0,IFERROR((TIMEVALUE(MID(G13,FIND("-",G13)+1,10))-TIMEVALUE(LEFT(G13,FIND("-",G13)-1)))*24-1,0))</f>
+        <f>IF(G13="",0,IFERROR((TIMEVALUE(MID(G13,FIND("-",G13)+1,10))-TIMEVALUE(LEFT(G13,FIND("-",G13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="H29" s="5">
-        <f>IF(H13="",0,IFERROR((TIMEVALUE(MID(H13,FIND("-",H13)+1,10))-TIMEVALUE(LEFT(H13,FIND("-",H13)-1)))*24-1,0))</f>
+        <f>IF(H13="",0,IFERROR((TIMEVALUE(MID(H13,FIND("-",H13)+1,10))-TIMEVALUE(LEFT(H13,FIND("-",H13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="I29" s="5">
-        <f>IF(I13="",0,IFERROR((TIMEVALUE(MID(I13,FIND("-",I13)+1,10))-TIMEVALUE(LEFT(I13,FIND("-",I13)-1)))*24-1,0))</f>
+        <f>IF(I13="",0,IFERROR((TIMEVALUE(MID(I13,FIND("-",I13)+1,10))-TIMEVALUE(LEFT(I13,FIND("-",I13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="J29" s="5">
@@ -4763,27 +4768,27 @@
         <v/>
       </c>
       <c r="K29" s="5">
-        <f>IF(K13="",0,IFERROR((TIMEVALUE(MID(K13,FIND("-",K13)+1,10))-TIMEVALUE(LEFT(K13,FIND("-",K13)-1)))*24-1,0))</f>
+        <f>IF(K13="",0,IFERROR((TIMEVALUE(MID(K13,FIND("-",K13)+1,10))-TIMEVALUE(LEFT(K13,FIND("-",K13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="L29" s="5">
-        <f>IF(L13="",0,IFERROR((TIMEVALUE(MID(L13,FIND("-",L13)+1,10))-TIMEVALUE(LEFT(L13,FIND("-",L13)-1)))*24-1,0))</f>
+        <f>IF(L13="",0,IFERROR((TIMEVALUE(MID(L13,FIND("-",L13)+1,10))-TIMEVALUE(LEFT(L13,FIND("-",L13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="M29" s="5">
-        <f>IF(M13="",0,IFERROR((TIMEVALUE(MID(M13,FIND("-",M13)+1,10))-TIMEVALUE(LEFT(M13,FIND("-",M13)-1)))*24-1,0))</f>
+        <f>IF(M13="",0,IFERROR((TIMEVALUE(MID(M13,FIND("-",M13)+1,10))-TIMEVALUE(LEFT(M13,FIND("-",M13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="N29" s="5">
-        <f>IF(N13="",0,IFERROR((TIMEVALUE(MID(N13,FIND("-",N13)+1,10))-TIMEVALUE(LEFT(N13,FIND("-",N13)-1)))*24-1,0))</f>
+        <f>IF(N13="",0,IFERROR((TIMEVALUE(MID(N13,FIND("-",N13)+1,10))-TIMEVALUE(LEFT(N13,FIND("-",N13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="O29" s="5">
-        <f>IF(O13="",0,IFERROR((TIMEVALUE(MID(O13,FIND("-",O13)+1,10))-TIMEVALUE(LEFT(O13,FIND("-",O13)-1)))*24-1,0))</f>
+        <f>IF(O13="",0,IFERROR((TIMEVALUE(MID(O13,FIND("-",O13)+1,10))-TIMEVALUE(LEFT(O13,FIND("-",O13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="P29" s="5">
-        <f>IF(P13="",0,IFERROR((TIMEVALUE(MID(P13,FIND("-",P13)+1,10))-TIMEVALUE(LEFT(P13,FIND("-",P13)-1)))*24-1,0))</f>
+        <f>IF(P13="",0,IFERROR((TIMEVALUE(MID(P13,FIND("-",P13)+1,10))-TIMEVALUE(LEFT(P13,FIND("-",P13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Q29" s="5">
@@ -4791,27 +4796,27 @@
         <v/>
       </c>
       <c r="R29" s="5">
-        <f>IF(R13="",0,IFERROR((TIMEVALUE(MID(R13,FIND("-",R13)+1,10))-TIMEVALUE(LEFT(R13,FIND("-",R13)-1)))*24-1,0))</f>
+        <f>IF(R13="",0,IFERROR((TIMEVALUE(MID(R13,FIND("-",R13)+1,10))-TIMEVALUE(LEFT(R13,FIND("-",R13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="S29" s="5">
-        <f>IF(S13="",0,IFERROR((TIMEVALUE(MID(S13,FIND("-",S13)+1,10))-TIMEVALUE(LEFT(S13,FIND("-",S13)-1)))*24-1,0))</f>
+        <f>IF(S13="",0,IFERROR((TIMEVALUE(MID(S13,FIND("-",S13)+1,10))-TIMEVALUE(LEFT(S13,FIND("-",S13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="T29" s="5">
-        <f>IF(T13="",0,IFERROR((TIMEVALUE(MID(T13,FIND("-",T13)+1,10))-TIMEVALUE(LEFT(T13,FIND("-",T13)-1)))*24-1,0))</f>
+        <f>IF(T13="",0,IFERROR((TIMEVALUE(MID(T13,FIND("-",T13)+1,10))-TIMEVALUE(LEFT(T13,FIND("-",T13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="U29" s="5">
-        <f>IF(U13="",0,IFERROR((TIMEVALUE(MID(U13,FIND("-",U13)+1,10))-TIMEVALUE(LEFT(U13,FIND("-",U13)-1)))*24-1,0))</f>
+        <f>IF(U13="",0,IFERROR((TIMEVALUE(MID(U13,FIND("-",U13)+1,10))-TIMEVALUE(LEFT(U13,FIND("-",U13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="V29" s="5">
-        <f>IF(V13="",0,IFERROR((TIMEVALUE(MID(V13,FIND("-",V13)+1,10))-TIMEVALUE(LEFT(V13,FIND("-",V13)-1)))*24-1,0))</f>
+        <f>IF(V13="",0,IFERROR((TIMEVALUE(MID(V13,FIND("-",V13)+1,10))-TIMEVALUE(LEFT(V13,FIND("-",V13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="W29" s="5">
-        <f>IF(W13="",0,IFERROR((TIMEVALUE(MID(W13,FIND("-",W13)+1,10))-TIMEVALUE(LEFT(W13,FIND("-",W13)-1)))*24-1,0))</f>
+        <f>IF(W13="",0,IFERROR((TIMEVALUE(MID(W13,FIND("-",W13)+1,10))-TIMEVALUE(LEFT(W13,FIND("-",W13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="X29" s="5">
@@ -4819,27 +4824,27 @@
         <v/>
       </c>
       <c r="Y29" s="5">
-        <f>IF(Y13="",0,IFERROR((TIMEVALUE(MID(Y13,FIND("-",Y13)+1,10))-TIMEVALUE(LEFT(Y13,FIND("-",Y13)-1)))*24-1,0))</f>
+        <f>IF(Y13="",0,IFERROR((TIMEVALUE(MID(Y13,FIND("-",Y13)+1,10))-TIMEVALUE(LEFT(Y13,FIND("-",Y13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Z29" s="5">
-        <f>IF(Z13="",0,IFERROR((TIMEVALUE(MID(Z13,FIND("-",Z13)+1,10))-TIMEVALUE(LEFT(Z13,FIND("-",Z13)-1)))*24-1,0))</f>
+        <f>IF(Z13="",0,IFERROR((TIMEVALUE(MID(Z13,FIND("-",Z13)+1,10))-TIMEVALUE(LEFT(Z13,FIND("-",Z13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AA29" s="5">
-        <f>IF(AA13="",0,IFERROR((TIMEVALUE(MID(AA13,FIND("-",AA13)+1,10))-TIMEVALUE(LEFT(AA13,FIND("-",AA13)-1)))*24-1,0))</f>
+        <f>IF(AA13="",0,IFERROR((TIMEVALUE(MID(AA13,FIND("-",AA13)+1,10))-TIMEVALUE(LEFT(AA13,FIND("-",AA13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AB29" s="5">
-        <f>IF(AB13="",0,IFERROR((TIMEVALUE(MID(AB13,FIND("-",AB13)+1,10))-TIMEVALUE(LEFT(AB13,FIND("-",AB13)-1)))*24-1,0))</f>
+        <f>IF(AB13="",0,IFERROR((TIMEVALUE(MID(AB13,FIND("-",AB13)+1,10))-TIMEVALUE(LEFT(AB13,FIND("-",AB13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AC29" s="5">
-        <f>IF(AC13="",0,IFERROR((TIMEVALUE(MID(AC13,FIND("-",AC13)+1,10))-TIMEVALUE(LEFT(AC13,FIND("-",AC13)-1)))*24-1,0))</f>
+        <f>IF(AC13="",0,IFERROR((TIMEVALUE(MID(AC13,FIND("-",AC13)+1,10))-TIMEVALUE(LEFT(AC13,FIND("-",AC13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AD29" s="5">
-        <f>IF(AD13="",0,IFERROR((TIMEVALUE(MID(AD13,FIND("-",AD13)+1,10))-TIMEVALUE(LEFT(AD13,FIND("-",AD13)-1)))*24-1,0))</f>
+        <f>IF(AD13="",0,IFERROR((TIMEVALUE(MID(AD13,FIND("-",AD13)+1,10))-TIMEVALUE(LEFT(AD13,FIND("-",AD13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AE29" s="5">
@@ -4847,11 +4852,11 @@
         <v/>
       </c>
       <c r="AF29" s="5">
-        <f>IF(AF13="",0,IFERROR((TIMEVALUE(MID(AF13,FIND("-",AF13)+1,10))-TIMEVALUE(LEFT(AF13,FIND("-",AF13)-1)))*24-1,0))</f>
+        <f>IF(AF13="",0,IFERROR((TIMEVALUE(MID(AF13,FIND("-",AF13)+1,10))-TIMEVALUE(LEFT(AF13,FIND("-",AF13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AG29" s="5">
-        <f>IF(AG13="",0,IFERROR((TIMEVALUE(MID(AG13,FIND("-",AG13)+1,10))-TIMEVALUE(LEFT(AG13,FIND("-",AG13)-1)))*24-1,0))</f>
+        <f>IF(AG13="",0,IFERROR((TIMEVALUE(MID(AG13,FIND("-",AG13)+1,10))-TIMEVALUE(LEFT(AG13,FIND("-",AG13)-1)))*24-IF(ISNUMBER(FIND("-",$C13)),IFERROR((TIMEVALUE(MID($C13,FIND("-",$C13)+1,10))-TIMEVALUE(LEFT($C13,FIND("-",$C13)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AH29" s="5">
@@ -4897,27 +4902,27 @@
         <v/>
       </c>
       <c r="D30" s="5">
-        <f>IF(D14="",0,IFERROR((TIMEVALUE(MID(D14,FIND("-",D14)+1,10))-TIMEVALUE(LEFT(D14,FIND("-",D14)-1)))*24-1,0))</f>
+        <f>IF(D14="",0,IFERROR((TIMEVALUE(MID(D14,FIND("-",D14)+1,10))-TIMEVALUE(LEFT(D14,FIND("-",D14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="E30" s="5">
-        <f>IF(E14="",0,IFERROR((TIMEVALUE(MID(E14,FIND("-",E14)+1,10))-TIMEVALUE(LEFT(E14,FIND("-",E14)-1)))*24-1,0))</f>
+        <f>IF(E14="",0,IFERROR((TIMEVALUE(MID(E14,FIND("-",E14)+1,10))-TIMEVALUE(LEFT(E14,FIND("-",E14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="F30" s="5">
-        <f>IF(F14="",0,IFERROR((TIMEVALUE(MID(F14,FIND("-",F14)+1,10))-TIMEVALUE(LEFT(F14,FIND("-",F14)-1)))*24-1,0))</f>
+        <f>IF(F14="",0,IFERROR((TIMEVALUE(MID(F14,FIND("-",F14)+1,10))-TIMEVALUE(LEFT(F14,FIND("-",F14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="G30" s="5">
-        <f>IF(G14="",0,IFERROR((TIMEVALUE(MID(G14,FIND("-",G14)+1,10))-TIMEVALUE(LEFT(G14,FIND("-",G14)-1)))*24-1,0))</f>
+        <f>IF(G14="",0,IFERROR((TIMEVALUE(MID(G14,FIND("-",G14)+1,10))-TIMEVALUE(LEFT(G14,FIND("-",G14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="H30" s="5">
-        <f>IF(H14="",0,IFERROR((TIMEVALUE(MID(H14,FIND("-",H14)+1,10))-TIMEVALUE(LEFT(H14,FIND("-",H14)-1)))*24-1,0))</f>
+        <f>IF(H14="",0,IFERROR((TIMEVALUE(MID(H14,FIND("-",H14)+1,10))-TIMEVALUE(LEFT(H14,FIND("-",H14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="I30" s="5">
-        <f>IF(I14="",0,IFERROR((TIMEVALUE(MID(I14,FIND("-",I14)+1,10))-TIMEVALUE(LEFT(I14,FIND("-",I14)-1)))*24-1,0))</f>
+        <f>IF(I14="",0,IFERROR((TIMEVALUE(MID(I14,FIND("-",I14)+1,10))-TIMEVALUE(LEFT(I14,FIND("-",I14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="J30" s="5">
@@ -4925,27 +4930,27 @@
         <v/>
       </c>
       <c r="K30" s="5">
-        <f>IF(K14="",0,IFERROR((TIMEVALUE(MID(K14,FIND("-",K14)+1,10))-TIMEVALUE(LEFT(K14,FIND("-",K14)-1)))*24-1,0))</f>
+        <f>IF(K14="",0,IFERROR((TIMEVALUE(MID(K14,FIND("-",K14)+1,10))-TIMEVALUE(LEFT(K14,FIND("-",K14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="L30" s="5">
-        <f>IF(L14="",0,IFERROR((TIMEVALUE(MID(L14,FIND("-",L14)+1,10))-TIMEVALUE(LEFT(L14,FIND("-",L14)-1)))*24-1,0))</f>
+        <f>IF(L14="",0,IFERROR((TIMEVALUE(MID(L14,FIND("-",L14)+1,10))-TIMEVALUE(LEFT(L14,FIND("-",L14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="M30" s="5">
-        <f>IF(M14="",0,IFERROR((TIMEVALUE(MID(M14,FIND("-",M14)+1,10))-TIMEVALUE(LEFT(M14,FIND("-",M14)-1)))*24-1,0))</f>
+        <f>IF(M14="",0,IFERROR((TIMEVALUE(MID(M14,FIND("-",M14)+1,10))-TIMEVALUE(LEFT(M14,FIND("-",M14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="N30" s="5">
-        <f>IF(N14="",0,IFERROR((TIMEVALUE(MID(N14,FIND("-",N14)+1,10))-TIMEVALUE(LEFT(N14,FIND("-",N14)-1)))*24-1,0))</f>
+        <f>IF(N14="",0,IFERROR((TIMEVALUE(MID(N14,FIND("-",N14)+1,10))-TIMEVALUE(LEFT(N14,FIND("-",N14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="O30" s="5">
-        <f>IF(O14="",0,IFERROR((TIMEVALUE(MID(O14,FIND("-",O14)+1,10))-TIMEVALUE(LEFT(O14,FIND("-",O14)-1)))*24-1,0))</f>
+        <f>IF(O14="",0,IFERROR((TIMEVALUE(MID(O14,FIND("-",O14)+1,10))-TIMEVALUE(LEFT(O14,FIND("-",O14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="P30" s="5">
-        <f>IF(P14="",0,IFERROR((TIMEVALUE(MID(P14,FIND("-",P14)+1,10))-TIMEVALUE(LEFT(P14,FIND("-",P14)-1)))*24-1,0))</f>
+        <f>IF(P14="",0,IFERROR((TIMEVALUE(MID(P14,FIND("-",P14)+1,10))-TIMEVALUE(LEFT(P14,FIND("-",P14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Q30" s="5">
@@ -4953,27 +4958,27 @@
         <v/>
       </c>
       <c r="R30" s="5">
-        <f>IF(R14="",0,IFERROR((TIMEVALUE(MID(R14,FIND("-",R14)+1,10))-TIMEVALUE(LEFT(R14,FIND("-",R14)-1)))*24-1,0))</f>
+        <f>IF(R14="",0,IFERROR((TIMEVALUE(MID(R14,FIND("-",R14)+1,10))-TIMEVALUE(LEFT(R14,FIND("-",R14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="S30" s="5">
-        <f>IF(S14="",0,IFERROR((TIMEVALUE(MID(S14,FIND("-",S14)+1,10))-TIMEVALUE(LEFT(S14,FIND("-",S14)-1)))*24-1,0))</f>
+        <f>IF(S14="",0,IFERROR((TIMEVALUE(MID(S14,FIND("-",S14)+1,10))-TIMEVALUE(LEFT(S14,FIND("-",S14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="T30" s="5">
-        <f>IF(T14="",0,IFERROR((TIMEVALUE(MID(T14,FIND("-",T14)+1,10))-TIMEVALUE(LEFT(T14,FIND("-",T14)-1)))*24-1,0))</f>
+        <f>IF(T14="",0,IFERROR((TIMEVALUE(MID(T14,FIND("-",T14)+1,10))-TIMEVALUE(LEFT(T14,FIND("-",T14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="U30" s="5">
-        <f>IF(U14="",0,IFERROR((TIMEVALUE(MID(U14,FIND("-",U14)+1,10))-TIMEVALUE(LEFT(U14,FIND("-",U14)-1)))*24-1,0))</f>
+        <f>IF(U14="",0,IFERROR((TIMEVALUE(MID(U14,FIND("-",U14)+1,10))-TIMEVALUE(LEFT(U14,FIND("-",U14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="V30" s="5">
-        <f>IF(V14="",0,IFERROR((TIMEVALUE(MID(V14,FIND("-",V14)+1,10))-TIMEVALUE(LEFT(V14,FIND("-",V14)-1)))*24-1,0))</f>
+        <f>IF(V14="",0,IFERROR((TIMEVALUE(MID(V14,FIND("-",V14)+1,10))-TIMEVALUE(LEFT(V14,FIND("-",V14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="W30" s="5">
-        <f>IF(W14="",0,IFERROR((TIMEVALUE(MID(W14,FIND("-",W14)+1,10))-TIMEVALUE(LEFT(W14,FIND("-",W14)-1)))*24-1,0))</f>
+        <f>IF(W14="",0,IFERROR((TIMEVALUE(MID(W14,FIND("-",W14)+1,10))-TIMEVALUE(LEFT(W14,FIND("-",W14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="X30" s="5">
@@ -4981,27 +4986,27 @@
         <v/>
       </c>
       <c r="Y30" s="5">
-        <f>IF(Y14="",0,IFERROR((TIMEVALUE(MID(Y14,FIND("-",Y14)+1,10))-TIMEVALUE(LEFT(Y14,FIND("-",Y14)-1)))*24-1,0))</f>
+        <f>IF(Y14="",0,IFERROR((TIMEVALUE(MID(Y14,FIND("-",Y14)+1,10))-TIMEVALUE(LEFT(Y14,FIND("-",Y14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Z30" s="5">
-        <f>IF(Z14="",0,IFERROR((TIMEVALUE(MID(Z14,FIND("-",Z14)+1,10))-TIMEVALUE(LEFT(Z14,FIND("-",Z14)-1)))*24-1,0))</f>
+        <f>IF(Z14="",0,IFERROR((TIMEVALUE(MID(Z14,FIND("-",Z14)+1,10))-TIMEVALUE(LEFT(Z14,FIND("-",Z14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AA30" s="5">
-        <f>IF(AA14="",0,IFERROR((TIMEVALUE(MID(AA14,FIND("-",AA14)+1,10))-TIMEVALUE(LEFT(AA14,FIND("-",AA14)-1)))*24-1,0))</f>
+        <f>IF(AA14="",0,IFERROR((TIMEVALUE(MID(AA14,FIND("-",AA14)+1,10))-TIMEVALUE(LEFT(AA14,FIND("-",AA14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AB30" s="5">
-        <f>IF(AB14="",0,IFERROR((TIMEVALUE(MID(AB14,FIND("-",AB14)+1,10))-TIMEVALUE(LEFT(AB14,FIND("-",AB14)-1)))*24-1,0))</f>
+        <f>IF(AB14="",0,IFERROR((TIMEVALUE(MID(AB14,FIND("-",AB14)+1,10))-TIMEVALUE(LEFT(AB14,FIND("-",AB14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AC30" s="5">
-        <f>IF(AC14="",0,IFERROR((TIMEVALUE(MID(AC14,FIND("-",AC14)+1,10))-TIMEVALUE(LEFT(AC14,FIND("-",AC14)-1)))*24-1,0))</f>
+        <f>IF(AC14="",0,IFERROR((TIMEVALUE(MID(AC14,FIND("-",AC14)+1,10))-TIMEVALUE(LEFT(AC14,FIND("-",AC14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AD30" s="5">
-        <f>IF(AD14="",0,IFERROR((TIMEVALUE(MID(AD14,FIND("-",AD14)+1,10))-TIMEVALUE(LEFT(AD14,FIND("-",AD14)-1)))*24-1,0))</f>
+        <f>IF(AD14="",0,IFERROR((TIMEVALUE(MID(AD14,FIND("-",AD14)+1,10))-TIMEVALUE(LEFT(AD14,FIND("-",AD14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AE30" s="5">
@@ -5009,11 +5014,11 @@
         <v/>
       </c>
       <c r="AF30" s="5">
-        <f>IF(AF14="",0,IFERROR((TIMEVALUE(MID(AF14,FIND("-",AF14)+1,10))-TIMEVALUE(LEFT(AF14,FIND("-",AF14)-1)))*24-1,0))</f>
+        <f>IF(AF14="",0,IFERROR((TIMEVALUE(MID(AF14,FIND("-",AF14)+1,10))-TIMEVALUE(LEFT(AF14,FIND("-",AF14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AG30" s="5">
-        <f>IF(AG14="",0,IFERROR((TIMEVALUE(MID(AG14,FIND("-",AG14)+1,10))-TIMEVALUE(LEFT(AG14,FIND("-",AG14)-1)))*24-1,0))</f>
+        <f>IF(AG14="",0,IFERROR((TIMEVALUE(MID(AG14,FIND("-",AG14)+1,10))-TIMEVALUE(LEFT(AG14,FIND("-",AG14)-1)))*24-IF(ISNUMBER(FIND("-",$C14)),IFERROR((TIMEVALUE(MID($C14,FIND("-",$C14)+1,10))-TIMEVALUE(LEFT($C14,FIND("-",$C14)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AH30" s="5">
@@ -5059,27 +5064,27 @@
         <v/>
       </c>
       <c r="D31" s="5">
-        <f>IF(D15="",0,IFERROR((TIMEVALUE(MID(D15,FIND("-",D15)+1,10))-TIMEVALUE(LEFT(D15,FIND("-",D15)-1)))*24,0))</f>
+        <f>IF(D15="",0,IFERROR((TIMEVALUE(MID(D15,FIND("-",D15)+1,10))-TIMEVALUE(LEFT(D15,FIND("-",D15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="E31" s="5">
-        <f>IF(E15="",0,IFERROR((TIMEVALUE(MID(E15,FIND("-",E15)+1,10))-TIMEVALUE(LEFT(E15,FIND("-",E15)-1)))*24,0))</f>
+        <f>IF(E15="",0,IFERROR((TIMEVALUE(MID(E15,FIND("-",E15)+1,10))-TIMEVALUE(LEFT(E15,FIND("-",E15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="F31" s="5">
-        <f>IF(F15="",0,IFERROR((TIMEVALUE(MID(F15,FIND("-",F15)+1,10))-TIMEVALUE(LEFT(F15,FIND("-",F15)-1)))*24,0))</f>
+        <f>IF(F15="",0,IFERROR((TIMEVALUE(MID(F15,FIND("-",F15)+1,10))-TIMEVALUE(LEFT(F15,FIND("-",F15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="G31" s="5">
-        <f>IF(G15="",0,IFERROR((TIMEVALUE(MID(G15,FIND("-",G15)+1,10))-TIMEVALUE(LEFT(G15,FIND("-",G15)-1)))*24,0))</f>
+        <f>IF(G15="",0,IFERROR((TIMEVALUE(MID(G15,FIND("-",G15)+1,10))-TIMEVALUE(LEFT(G15,FIND("-",G15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="H31" s="5">
-        <f>IF(H15="",0,IFERROR((TIMEVALUE(MID(H15,FIND("-",H15)+1,10))-TIMEVALUE(LEFT(H15,FIND("-",H15)-1)))*24,0))</f>
+        <f>IF(H15="",0,IFERROR((TIMEVALUE(MID(H15,FIND("-",H15)+1,10))-TIMEVALUE(LEFT(H15,FIND("-",H15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="I31" s="5">
-        <f>IF(I15="",0,IFERROR((TIMEVALUE(MID(I15,FIND("-",I15)+1,10))-TIMEVALUE(LEFT(I15,FIND("-",I15)-1)))*24,0))</f>
+        <f>IF(I15="",0,IFERROR((TIMEVALUE(MID(I15,FIND("-",I15)+1,10))-TIMEVALUE(LEFT(I15,FIND("-",I15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="J31" s="5">
@@ -5087,27 +5092,27 @@
         <v/>
       </c>
       <c r="K31" s="5">
-        <f>IF(K15="",0,IFERROR((TIMEVALUE(MID(K15,FIND("-",K15)+1,10))-TIMEVALUE(LEFT(K15,FIND("-",K15)-1)))*24,0))</f>
+        <f>IF(K15="",0,IFERROR((TIMEVALUE(MID(K15,FIND("-",K15)+1,10))-TIMEVALUE(LEFT(K15,FIND("-",K15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="L31" s="5">
-        <f>IF(L15="",0,IFERROR((TIMEVALUE(MID(L15,FIND("-",L15)+1,10))-TIMEVALUE(LEFT(L15,FIND("-",L15)-1)))*24,0))</f>
+        <f>IF(L15="",0,IFERROR((TIMEVALUE(MID(L15,FIND("-",L15)+1,10))-TIMEVALUE(LEFT(L15,FIND("-",L15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="M31" s="5">
-        <f>IF(M15="",0,IFERROR((TIMEVALUE(MID(M15,FIND("-",M15)+1,10))-TIMEVALUE(LEFT(M15,FIND("-",M15)-1)))*24,0))</f>
+        <f>IF(M15="",0,IFERROR((TIMEVALUE(MID(M15,FIND("-",M15)+1,10))-TIMEVALUE(LEFT(M15,FIND("-",M15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="N31" s="5">
-        <f>IF(N15="",0,IFERROR((TIMEVALUE(MID(N15,FIND("-",N15)+1,10))-TIMEVALUE(LEFT(N15,FIND("-",N15)-1)))*24,0))</f>
+        <f>IF(N15="",0,IFERROR((TIMEVALUE(MID(N15,FIND("-",N15)+1,10))-TIMEVALUE(LEFT(N15,FIND("-",N15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="O31" s="5">
-        <f>IF(O15="",0,IFERROR((TIMEVALUE(MID(O15,FIND("-",O15)+1,10))-TIMEVALUE(LEFT(O15,FIND("-",O15)-1)))*24,0))</f>
+        <f>IF(O15="",0,IFERROR((TIMEVALUE(MID(O15,FIND("-",O15)+1,10))-TIMEVALUE(LEFT(O15,FIND("-",O15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="P31" s="5">
-        <f>IF(P15="",0,IFERROR((TIMEVALUE(MID(P15,FIND("-",P15)+1,10))-TIMEVALUE(LEFT(P15,FIND("-",P15)-1)))*24,0))</f>
+        <f>IF(P15="",0,IFERROR((TIMEVALUE(MID(P15,FIND("-",P15)+1,10))-TIMEVALUE(LEFT(P15,FIND("-",P15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Q31" s="5">
@@ -5115,27 +5120,27 @@
         <v/>
       </c>
       <c r="R31" s="5">
-        <f>IF(R15="",0,IFERROR((TIMEVALUE(MID(R15,FIND("-",R15)+1,10))-TIMEVALUE(LEFT(R15,FIND("-",R15)-1)))*24,0))</f>
+        <f>IF(R15="",0,IFERROR((TIMEVALUE(MID(R15,FIND("-",R15)+1,10))-TIMEVALUE(LEFT(R15,FIND("-",R15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="S31" s="5">
-        <f>IF(S15="",0,IFERROR((TIMEVALUE(MID(S15,FIND("-",S15)+1,10))-TIMEVALUE(LEFT(S15,FIND("-",S15)-1)))*24,0))</f>
+        <f>IF(S15="",0,IFERROR((TIMEVALUE(MID(S15,FIND("-",S15)+1,10))-TIMEVALUE(LEFT(S15,FIND("-",S15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="T31" s="5">
-        <f>IF(T15="",0,IFERROR((TIMEVALUE(MID(T15,FIND("-",T15)+1,10))-TIMEVALUE(LEFT(T15,FIND("-",T15)-1)))*24,0))</f>
+        <f>IF(T15="",0,IFERROR((TIMEVALUE(MID(T15,FIND("-",T15)+1,10))-TIMEVALUE(LEFT(T15,FIND("-",T15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="U31" s="5">
-        <f>IF(U15="",0,IFERROR((TIMEVALUE(MID(U15,FIND("-",U15)+1,10))-TIMEVALUE(LEFT(U15,FIND("-",U15)-1)))*24,0))</f>
+        <f>IF(U15="",0,IFERROR((TIMEVALUE(MID(U15,FIND("-",U15)+1,10))-TIMEVALUE(LEFT(U15,FIND("-",U15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="V31" s="5">
-        <f>IF(V15="",0,IFERROR((TIMEVALUE(MID(V15,FIND("-",V15)+1,10))-TIMEVALUE(LEFT(V15,FIND("-",V15)-1)))*24,0))</f>
+        <f>IF(V15="",0,IFERROR((TIMEVALUE(MID(V15,FIND("-",V15)+1,10))-TIMEVALUE(LEFT(V15,FIND("-",V15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="W31" s="5">
-        <f>IF(W15="",0,IFERROR((TIMEVALUE(MID(W15,FIND("-",W15)+1,10))-TIMEVALUE(LEFT(W15,FIND("-",W15)-1)))*24,0))</f>
+        <f>IF(W15="",0,IFERROR((TIMEVALUE(MID(W15,FIND("-",W15)+1,10))-TIMEVALUE(LEFT(W15,FIND("-",W15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="X31" s="5">
@@ -5143,27 +5148,27 @@
         <v/>
       </c>
       <c r="Y31" s="5">
-        <f>IF(Y15="",0,IFERROR((TIMEVALUE(MID(Y15,FIND("-",Y15)+1,10))-TIMEVALUE(LEFT(Y15,FIND("-",Y15)-1)))*24,0))</f>
+        <f>IF(Y15="",0,IFERROR((TIMEVALUE(MID(Y15,FIND("-",Y15)+1,10))-TIMEVALUE(LEFT(Y15,FIND("-",Y15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Z31" s="5">
-        <f>IF(Z15="",0,IFERROR((TIMEVALUE(MID(Z15,FIND("-",Z15)+1,10))-TIMEVALUE(LEFT(Z15,FIND("-",Z15)-1)))*24,0))</f>
+        <f>IF(Z15="",0,IFERROR((TIMEVALUE(MID(Z15,FIND("-",Z15)+1,10))-TIMEVALUE(LEFT(Z15,FIND("-",Z15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AA31" s="5">
-        <f>IF(AA15="",0,IFERROR((TIMEVALUE(MID(AA15,FIND("-",AA15)+1,10))-TIMEVALUE(LEFT(AA15,FIND("-",AA15)-1)))*24,0))</f>
+        <f>IF(AA15="",0,IFERROR((TIMEVALUE(MID(AA15,FIND("-",AA15)+1,10))-TIMEVALUE(LEFT(AA15,FIND("-",AA15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AB31" s="5">
-        <f>IF(AB15="",0,IFERROR((TIMEVALUE(MID(AB15,FIND("-",AB15)+1,10))-TIMEVALUE(LEFT(AB15,FIND("-",AB15)-1)))*24,0))</f>
+        <f>IF(AB15="",0,IFERROR((TIMEVALUE(MID(AB15,FIND("-",AB15)+1,10))-TIMEVALUE(LEFT(AB15,FIND("-",AB15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AC31" s="5">
-        <f>IF(AC15="",0,IFERROR((TIMEVALUE(MID(AC15,FIND("-",AC15)+1,10))-TIMEVALUE(LEFT(AC15,FIND("-",AC15)-1)))*24,0))</f>
+        <f>IF(AC15="",0,IFERROR((TIMEVALUE(MID(AC15,FIND("-",AC15)+1,10))-TIMEVALUE(LEFT(AC15,FIND("-",AC15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AD31" s="5">
-        <f>IF(AD15="",0,IFERROR((TIMEVALUE(MID(AD15,FIND("-",AD15)+1,10))-TIMEVALUE(LEFT(AD15,FIND("-",AD15)-1)))*24,0))</f>
+        <f>IF(AD15="",0,IFERROR((TIMEVALUE(MID(AD15,FIND("-",AD15)+1,10))-TIMEVALUE(LEFT(AD15,FIND("-",AD15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AE31" s="5">
@@ -5171,11 +5176,11 @@
         <v/>
       </c>
       <c r="AF31" s="5">
-        <f>IF(AF15="",0,IFERROR((TIMEVALUE(MID(AF15,FIND("-",AF15)+1,10))-TIMEVALUE(LEFT(AF15,FIND("-",AF15)-1)))*24,0))</f>
+        <f>IF(AF15="",0,IFERROR((TIMEVALUE(MID(AF15,FIND("-",AF15)+1,10))-TIMEVALUE(LEFT(AF15,FIND("-",AF15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AG31" s="5">
-        <f>IF(AG15="",0,IFERROR((TIMEVALUE(MID(AG15,FIND("-",AG15)+1,10))-TIMEVALUE(LEFT(AG15,FIND("-",AG15)-1)))*24,0))</f>
+        <f>IF(AG15="",0,IFERROR((TIMEVALUE(MID(AG15,FIND("-",AG15)+1,10))-TIMEVALUE(LEFT(AG15,FIND("-",AG15)-1)))*24-IF(ISNUMBER(FIND("-",$C15)),IFERROR((TIMEVALUE(MID($C15,FIND("-",$C15)+1,10))-TIMEVALUE(LEFT($C15,FIND("-",$C15)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AH31" s="5">
@@ -6027,27 +6032,27 @@
         </is>
       </c>
       <c r="D5">
-        <f>IF(D2="",0,IFERROR((TIMEVALUE(MID(D2,FIND("-",D2)+1,10))-TIMEVALUE(LEFT(D2,FIND("-",D2)-1)))*24,0))</f>
+        <f>IF(D2="",0,IFERROR((TIMEVALUE(MID(D2,FIND("-",D2)+1,10))-TIMEVALUE(LEFT(D2,FIND("-",D2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="E5">
-        <f>IF(E2="",0,IFERROR((TIMEVALUE(MID(E2,FIND("-",E2)+1,10))-TIMEVALUE(LEFT(E2,FIND("-",E2)-1)))*24,0))</f>
+        <f>IF(E2="",0,IFERROR((TIMEVALUE(MID(E2,FIND("-",E2)+1,10))-TIMEVALUE(LEFT(E2,FIND("-",E2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="F5">
-        <f>IF(F2="",0,IFERROR((TIMEVALUE(MID(F2,FIND("-",F2)+1,10))-TIMEVALUE(LEFT(F2,FIND("-",F2)-1)))*24,0))</f>
+        <f>IF(F2="",0,IFERROR((TIMEVALUE(MID(F2,FIND("-",F2)+1,10))-TIMEVALUE(LEFT(F2,FIND("-",F2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="G5">
-        <f>IF(G2="",0,IFERROR((TIMEVALUE(MID(G2,FIND("-",G2)+1,10))-TIMEVALUE(LEFT(G2,FIND("-",G2)-1)))*24,0))</f>
+        <f>IF(G2="",0,IFERROR((TIMEVALUE(MID(G2,FIND("-",G2)+1,10))-TIMEVALUE(LEFT(G2,FIND("-",G2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="H5">
-        <f>IF(H2="",0,IFERROR((TIMEVALUE(MID(H2,FIND("-",H2)+1,10))-TIMEVALUE(LEFT(H2,FIND("-",H2)-1)))*24,0))</f>
+        <f>IF(H2="",0,IFERROR((TIMEVALUE(MID(H2,FIND("-",H2)+1,10))-TIMEVALUE(LEFT(H2,FIND("-",H2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="I5">
-        <f>IF(I2="",0,IFERROR((TIMEVALUE(MID(I2,FIND("-",I2)+1,10))-TIMEVALUE(LEFT(I2,FIND("-",I2)-1)))*24,0))</f>
+        <f>IF(I2="",0,IFERROR((TIMEVALUE(MID(I2,FIND("-",I2)+1,10))-TIMEVALUE(LEFT(I2,FIND("-",I2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="J5">
@@ -6055,27 +6060,27 @@
         <v/>
       </c>
       <c r="K5">
-        <f>IF(K2="",0,IFERROR((TIMEVALUE(MID(K2,FIND("-",K2)+1,10))-TIMEVALUE(LEFT(K2,FIND("-",K2)-1)))*24,0))</f>
+        <f>IF(K2="",0,IFERROR((TIMEVALUE(MID(K2,FIND("-",K2)+1,10))-TIMEVALUE(LEFT(K2,FIND("-",K2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="L5">
-        <f>IF(L2="",0,IFERROR((TIMEVALUE(MID(L2,FIND("-",L2)+1,10))-TIMEVALUE(LEFT(L2,FIND("-",L2)-1)))*24,0))</f>
+        <f>IF(L2="",0,IFERROR((TIMEVALUE(MID(L2,FIND("-",L2)+1,10))-TIMEVALUE(LEFT(L2,FIND("-",L2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="M5">
-        <f>IF(M2="",0,IFERROR((TIMEVALUE(MID(M2,FIND("-",M2)+1,10))-TIMEVALUE(LEFT(M2,FIND("-",M2)-1)))*24,0))</f>
+        <f>IF(M2="",0,IFERROR((TIMEVALUE(MID(M2,FIND("-",M2)+1,10))-TIMEVALUE(LEFT(M2,FIND("-",M2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="N5">
-        <f>IF(N2="",0,IFERROR((TIMEVALUE(MID(N2,FIND("-",N2)+1,10))-TIMEVALUE(LEFT(N2,FIND("-",N2)-1)))*24,0))</f>
+        <f>IF(N2="",0,IFERROR((TIMEVALUE(MID(N2,FIND("-",N2)+1,10))-TIMEVALUE(LEFT(N2,FIND("-",N2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="O5">
-        <f>IF(O2="",0,IFERROR((TIMEVALUE(MID(O2,FIND("-",O2)+1,10))-TIMEVALUE(LEFT(O2,FIND("-",O2)-1)))*24,0))</f>
+        <f>IF(O2="",0,IFERROR((TIMEVALUE(MID(O2,FIND("-",O2)+1,10))-TIMEVALUE(LEFT(O2,FIND("-",O2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="P5">
-        <f>IF(P2="",0,IFERROR((TIMEVALUE(MID(P2,FIND("-",P2)+1,10))-TIMEVALUE(LEFT(P2,FIND("-",P2)-1)))*24,0))</f>
+        <f>IF(P2="",0,IFERROR((TIMEVALUE(MID(P2,FIND("-",P2)+1,10))-TIMEVALUE(LEFT(P2,FIND("-",P2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Q5">
@@ -6083,27 +6088,27 @@
         <v/>
       </c>
       <c r="R5">
-        <f>IF(R2="",0,IFERROR((TIMEVALUE(MID(R2,FIND("-",R2)+1,10))-TIMEVALUE(LEFT(R2,FIND("-",R2)-1)))*24,0))</f>
+        <f>IF(R2="",0,IFERROR((TIMEVALUE(MID(R2,FIND("-",R2)+1,10))-TIMEVALUE(LEFT(R2,FIND("-",R2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="S5">
-        <f>IF(S2="",0,IFERROR((TIMEVALUE(MID(S2,FIND("-",S2)+1,10))-TIMEVALUE(LEFT(S2,FIND("-",S2)-1)))*24,0))</f>
+        <f>IF(S2="",0,IFERROR((TIMEVALUE(MID(S2,FIND("-",S2)+1,10))-TIMEVALUE(LEFT(S2,FIND("-",S2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="T5">
-        <f>IF(T2="",0,IFERROR((TIMEVALUE(MID(T2,FIND("-",T2)+1,10))-TIMEVALUE(LEFT(T2,FIND("-",T2)-1)))*24,0))</f>
+        <f>IF(T2="",0,IFERROR((TIMEVALUE(MID(T2,FIND("-",T2)+1,10))-TIMEVALUE(LEFT(T2,FIND("-",T2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="U5">
-        <f>IF(U2="",0,IFERROR((TIMEVALUE(MID(U2,FIND("-",U2)+1,10))-TIMEVALUE(LEFT(U2,FIND("-",U2)-1)))*24,0))</f>
+        <f>IF(U2="",0,IFERROR((TIMEVALUE(MID(U2,FIND("-",U2)+1,10))-TIMEVALUE(LEFT(U2,FIND("-",U2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="V5">
-        <f>IF(V2="",0,IFERROR((TIMEVALUE(MID(V2,FIND("-",V2)+1,10))-TIMEVALUE(LEFT(V2,FIND("-",V2)-1)))*24,0))</f>
+        <f>IF(V2="",0,IFERROR((TIMEVALUE(MID(V2,FIND("-",V2)+1,10))-TIMEVALUE(LEFT(V2,FIND("-",V2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="W5">
-        <f>IF(W2="",0,IFERROR((TIMEVALUE(MID(W2,FIND("-",W2)+1,10))-TIMEVALUE(LEFT(W2,FIND("-",W2)-1)))*24,0))</f>
+        <f>IF(W2="",0,IFERROR((TIMEVALUE(MID(W2,FIND("-",W2)+1,10))-TIMEVALUE(LEFT(W2,FIND("-",W2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="X5">
@@ -6111,27 +6116,27 @@
         <v/>
       </c>
       <c r="Y5">
-        <f>IF(Y2="",0,IFERROR((TIMEVALUE(MID(Y2,FIND("-",Y2)+1,10))-TIMEVALUE(LEFT(Y2,FIND("-",Y2)-1)))*24,0))</f>
+        <f>IF(Y2="",0,IFERROR((TIMEVALUE(MID(Y2,FIND("-",Y2)+1,10))-TIMEVALUE(LEFT(Y2,FIND("-",Y2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Z5">
-        <f>IF(Z2="",0,IFERROR((TIMEVALUE(MID(Z2,FIND("-",Z2)+1,10))-TIMEVALUE(LEFT(Z2,FIND("-",Z2)-1)))*24,0))</f>
+        <f>IF(Z2="",0,IFERROR((TIMEVALUE(MID(Z2,FIND("-",Z2)+1,10))-TIMEVALUE(LEFT(Z2,FIND("-",Z2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AA5">
-        <f>IF(AA2="",0,IFERROR((TIMEVALUE(MID(AA2,FIND("-",AA2)+1,10))-TIMEVALUE(LEFT(AA2,FIND("-",AA2)-1)))*24,0))</f>
+        <f>IF(AA2="",0,IFERROR((TIMEVALUE(MID(AA2,FIND("-",AA2)+1,10))-TIMEVALUE(LEFT(AA2,FIND("-",AA2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AB5">
-        <f>IF(AB2="",0,IFERROR((TIMEVALUE(MID(AB2,FIND("-",AB2)+1,10))-TIMEVALUE(LEFT(AB2,FIND("-",AB2)-1)))*24,0))</f>
+        <f>IF(AB2="",0,IFERROR((TIMEVALUE(MID(AB2,FIND("-",AB2)+1,10))-TIMEVALUE(LEFT(AB2,FIND("-",AB2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AC5">
-        <f>IF(AC2="",0,IFERROR((TIMEVALUE(MID(AC2,FIND("-",AC2)+1,10))-TIMEVALUE(LEFT(AC2,FIND("-",AC2)-1)))*24,0))</f>
+        <f>IF(AC2="",0,IFERROR((TIMEVALUE(MID(AC2,FIND("-",AC2)+1,10))-TIMEVALUE(LEFT(AC2,FIND("-",AC2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AD5">
-        <f>IF(AD2="",0,IFERROR((TIMEVALUE(MID(AD2,FIND("-",AD2)+1,10))-TIMEVALUE(LEFT(AD2,FIND("-",AD2)-1)))*24,0))</f>
+        <f>IF(AD2="",0,IFERROR((TIMEVALUE(MID(AD2,FIND("-",AD2)+1,10))-TIMEVALUE(LEFT(AD2,FIND("-",AD2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AE5">
@@ -6139,11 +6144,11 @@
         <v/>
       </c>
       <c r="AF5">
-        <f>IF(AF2="",0,IFERROR((TIMEVALUE(MID(AF2,FIND("-",AF2)+1,10))-TIMEVALUE(LEFT(AF2,FIND("-",AF2)-1)))*24,0))</f>
+        <f>IF(AF2="",0,IFERROR((TIMEVALUE(MID(AF2,FIND("-",AF2)+1,10))-TIMEVALUE(LEFT(AF2,FIND("-",AF2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AG5">
-        <f>IF(AG2="",0,IFERROR((TIMEVALUE(MID(AG2,FIND("-",AG2)+1,10))-TIMEVALUE(LEFT(AG2,FIND("-",AG2)-1)))*24,0))</f>
+        <f>IF(AG2="",0,IFERROR((TIMEVALUE(MID(AG2,FIND("-",AG2)+1,10))-TIMEVALUE(LEFT(AG2,FIND("-",AG2)-1)))*24-IF(ISNUMBER(FIND("-",$C2)),IFERROR((TIMEVALUE(MID($C2,FIND("-",$C2)+1,10))-TIMEVALUE(LEFT($C2,FIND("-",$C2)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AH5">
@@ -6178,27 +6183,27 @@
         </is>
       </c>
       <c r="D6">
-        <f>IF(D3="",0,IFERROR((TIMEVALUE(MID(D3,FIND("-",D3)+1,10))-TIMEVALUE(LEFT(D3,FIND("-",D3)-1)))*24,0))</f>
+        <f>IF(D3="",0,IFERROR((TIMEVALUE(MID(D3,FIND("-",D3)+1,10))-TIMEVALUE(LEFT(D3,FIND("-",D3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="E6">
-        <f>IF(E3="",0,IFERROR((TIMEVALUE(MID(E3,FIND("-",E3)+1,10))-TIMEVALUE(LEFT(E3,FIND("-",E3)-1)))*24,0))</f>
+        <f>IF(E3="",0,IFERROR((TIMEVALUE(MID(E3,FIND("-",E3)+1,10))-TIMEVALUE(LEFT(E3,FIND("-",E3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="F6">
-        <f>IF(F3="",0,IFERROR((TIMEVALUE(MID(F3,FIND("-",F3)+1,10))-TIMEVALUE(LEFT(F3,FIND("-",F3)-1)))*24,0))</f>
+        <f>IF(F3="",0,IFERROR((TIMEVALUE(MID(F3,FIND("-",F3)+1,10))-TIMEVALUE(LEFT(F3,FIND("-",F3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="G6">
-        <f>IF(G3="",0,IFERROR((TIMEVALUE(MID(G3,FIND("-",G3)+1,10))-TIMEVALUE(LEFT(G3,FIND("-",G3)-1)))*24,0))</f>
+        <f>IF(G3="",0,IFERROR((TIMEVALUE(MID(G3,FIND("-",G3)+1,10))-TIMEVALUE(LEFT(G3,FIND("-",G3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="H6">
-        <f>IF(H3="",0,IFERROR((TIMEVALUE(MID(H3,FIND("-",H3)+1,10))-TIMEVALUE(LEFT(H3,FIND("-",H3)-1)))*24,0))</f>
+        <f>IF(H3="",0,IFERROR((TIMEVALUE(MID(H3,FIND("-",H3)+1,10))-TIMEVALUE(LEFT(H3,FIND("-",H3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="I6">
-        <f>IF(I3="",0,IFERROR((TIMEVALUE(MID(I3,FIND("-",I3)+1,10))-TIMEVALUE(LEFT(I3,FIND("-",I3)-1)))*24,0))</f>
+        <f>IF(I3="",0,IFERROR((TIMEVALUE(MID(I3,FIND("-",I3)+1,10))-TIMEVALUE(LEFT(I3,FIND("-",I3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="J6">
@@ -6206,27 +6211,27 @@
         <v/>
       </c>
       <c r="K6">
-        <f>IF(K3="",0,IFERROR((TIMEVALUE(MID(K3,FIND("-",K3)+1,10))-TIMEVALUE(LEFT(K3,FIND("-",K3)-1)))*24,0))</f>
+        <f>IF(K3="",0,IFERROR((TIMEVALUE(MID(K3,FIND("-",K3)+1,10))-TIMEVALUE(LEFT(K3,FIND("-",K3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="L6">
-        <f>IF(L3="",0,IFERROR((TIMEVALUE(MID(L3,FIND("-",L3)+1,10))-TIMEVALUE(LEFT(L3,FIND("-",L3)-1)))*24,0))</f>
+        <f>IF(L3="",0,IFERROR((TIMEVALUE(MID(L3,FIND("-",L3)+1,10))-TIMEVALUE(LEFT(L3,FIND("-",L3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="M6">
-        <f>IF(M3="",0,IFERROR((TIMEVALUE(MID(M3,FIND("-",M3)+1,10))-TIMEVALUE(LEFT(M3,FIND("-",M3)-1)))*24,0))</f>
+        <f>IF(M3="",0,IFERROR((TIMEVALUE(MID(M3,FIND("-",M3)+1,10))-TIMEVALUE(LEFT(M3,FIND("-",M3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="N6">
-        <f>IF(N3="",0,IFERROR((TIMEVALUE(MID(N3,FIND("-",N3)+1,10))-TIMEVALUE(LEFT(N3,FIND("-",N3)-1)))*24,0))</f>
+        <f>IF(N3="",0,IFERROR((TIMEVALUE(MID(N3,FIND("-",N3)+1,10))-TIMEVALUE(LEFT(N3,FIND("-",N3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="O6">
-        <f>IF(O3="",0,IFERROR((TIMEVALUE(MID(O3,FIND("-",O3)+1,10))-TIMEVALUE(LEFT(O3,FIND("-",O3)-1)))*24,0))</f>
+        <f>IF(O3="",0,IFERROR((TIMEVALUE(MID(O3,FIND("-",O3)+1,10))-TIMEVALUE(LEFT(O3,FIND("-",O3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="P6">
-        <f>IF(P3="",0,IFERROR((TIMEVALUE(MID(P3,FIND("-",P3)+1,10))-TIMEVALUE(LEFT(P3,FIND("-",P3)-1)))*24,0))</f>
+        <f>IF(P3="",0,IFERROR((TIMEVALUE(MID(P3,FIND("-",P3)+1,10))-TIMEVALUE(LEFT(P3,FIND("-",P3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Q6">
@@ -6234,27 +6239,27 @@
         <v/>
       </c>
       <c r="R6">
-        <f>IF(R3="",0,IFERROR((TIMEVALUE(MID(R3,FIND("-",R3)+1,10))-TIMEVALUE(LEFT(R3,FIND("-",R3)-1)))*24,0))</f>
+        <f>IF(R3="",0,IFERROR((TIMEVALUE(MID(R3,FIND("-",R3)+1,10))-TIMEVALUE(LEFT(R3,FIND("-",R3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="S6">
-        <f>IF(S3="",0,IFERROR((TIMEVALUE(MID(S3,FIND("-",S3)+1,10))-TIMEVALUE(LEFT(S3,FIND("-",S3)-1)))*24,0))</f>
+        <f>IF(S3="",0,IFERROR((TIMEVALUE(MID(S3,FIND("-",S3)+1,10))-TIMEVALUE(LEFT(S3,FIND("-",S3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="T6">
-        <f>IF(T3="",0,IFERROR((TIMEVALUE(MID(T3,FIND("-",T3)+1,10))-TIMEVALUE(LEFT(T3,FIND("-",T3)-1)))*24,0))</f>
+        <f>IF(T3="",0,IFERROR((TIMEVALUE(MID(T3,FIND("-",T3)+1,10))-TIMEVALUE(LEFT(T3,FIND("-",T3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="U6">
-        <f>IF(U3="",0,IFERROR((TIMEVALUE(MID(U3,FIND("-",U3)+1,10))-TIMEVALUE(LEFT(U3,FIND("-",U3)-1)))*24,0))</f>
+        <f>IF(U3="",0,IFERROR((TIMEVALUE(MID(U3,FIND("-",U3)+1,10))-TIMEVALUE(LEFT(U3,FIND("-",U3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="V6">
-        <f>IF(V3="",0,IFERROR((TIMEVALUE(MID(V3,FIND("-",V3)+1,10))-TIMEVALUE(LEFT(V3,FIND("-",V3)-1)))*24,0))</f>
+        <f>IF(V3="",0,IFERROR((TIMEVALUE(MID(V3,FIND("-",V3)+1,10))-TIMEVALUE(LEFT(V3,FIND("-",V3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="W6">
-        <f>IF(W3="",0,IFERROR((TIMEVALUE(MID(W3,FIND("-",W3)+1,10))-TIMEVALUE(LEFT(W3,FIND("-",W3)-1)))*24,0))</f>
+        <f>IF(W3="",0,IFERROR((TIMEVALUE(MID(W3,FIND("-",W3)+1,10))-TIMEVALUE(LEFT(W3,FIND("-",W3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="X6">
@@ -6262,27 +6267,27 @@
         <v/>
       </c>
       <c r="Y6">
-        <f>IF(Y3="",0,IFERROR((TIMEVALUE(MID(Y3,FIND("-",Y3)+1,10))-TIMEVALUE(LEFT(Y3,FIND("-",Y3)-1)))*24,0))</f>
+        <f>IF(Y3="",0,IFERROR((TIMEVALUE(MID(Y3,FIND("-",Y3)+1,10))-TIMEVALUE(LEFT(Y3,FIND("-",Y3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="Z6">
-        <f>IF(Z3="",0,IFERROR((TIMEVALUE(MID(Z3,FIND("-",Z3)+1,10))-TIMEVALUE(LEFT(Z3,FIND("-",Z3)-1)))*24,0))</f>
+        <f>IF(Z3="",0,IFERROR((TIMEVALUE(MID(Z3,FIND("-",Z3)+1,10))-TIMEVALUE(LEFT(Z3,FIND("-",Z3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AA6">
-        <f>IF(AA3="",0,IFERROR((TIMEVALUE(MID(AA3,FIND("-",AA3)+1,10))-TIMEVALUE(LEFT(AA3,FIND("-",AA3)-1)))*24,0))</f>
+        <f>IF(AA3="",0,IFERROR((TIMEVALUE(MID(AA3,FIND("-",AA3)+1,10))-TIMEVALUE(LEFT(AA3,FIND("-",AA3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AB6">
-        <f>IF(AB3="",0,IFERROR((TIMEVALUE(MID(AB3,FIND("-",AB3)+1,10))-TIMEVALUE(LEFT(AB3,FIND("-",AB3)-1)))*24,0))</f>
+        <f>IF(AB3="",0,IFERROR((TIMEVALUE(MID(AB3,FIND("-",AB3)+1,10))-TIMEVALUE(LEFT(AB3,FIND("-",AB3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AC6">
-        <f>IF(AC3="",0,IFERROR((TIMEVALUE(MID(AC3,FIND("-",AC3)+1,10))-TIMEVALUE(LEFT(AC3,FIND("-",AC3)-1)))*24,0))</f>
+        <f>IF(AC3="",0,IFERROR((TIMEVALUE(MID(AC3,FIND("-",AC3)+1,10))-TIMEVALUE(LEFT(AC3,FIND("-",AC3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AD6">
-        <f>IF(AD3="",0,IFERROR((TIMEVALUE(MID(AD3,FIND("-",AD3)+1,10))-TIMEVALUE(LEFT(AD3,FIND("-",AD3)-1)))*24,0))</f>
+        <f>IF(AD3="",0,IFERROR((TIMEVALUE(MID(AD3,FIND("-",AD3)+1,10))-TIMEVALUE(LEFT(AD3,FIND("-",AD3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AE6">
@@ -6290,11 +6295,11 @@
         <v/>
       </c>
       <c r="AF6">
-        <f>IF(AF3="",0,IFERROR((TIMEVALUE(MID(AF3,FIND("-",AF3)+1,10))-TIMEVALUE(LEFT(AF3,FIND("-",AF3)-1)))*24,0))</f>
+        <f>IF(AF3="",0,IFERROR((TIMEVALUE(MID(AF3,FIND("-",AF3)+1,10))-TIMEVALUE(LEFT(AF3,FIND("-",AF3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AG6">
-        <f>IF(AG3="",0,IFERROR((TIMEVALUE(MID(AG3,FIND("-",AG3)+1,10))-TIMEVALUE(LEFT(AG3,FIND("-",AG3)-1)))*24,0))</f>
+        <f>IF(AG3="",0,IFERROR((TIMEVALUE(MID(AG3,FIND("-",AG3)+1,10))-TIMEVALUE(LEFT(AG3,FIND("-",AG3)-1)))*24-IF(ISNUMBER(FIND("-",$C3)),IFERROR((TIMEVALUE(MID($C3,FIND("-",$C3)+1,10))-TIMEVALUE(LEFT($C3,FIND("-",$C3)-1)))*24,0),0),0))</f>
         <v/>
       </c>
       <c r="AH6">

</xml_diff>